<commit_message>
seperated the logic of sheet and bargraph
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="277">
   <si>
     <t>Sr. No</t>
   </si>
@@ -32,789 +32,780 @@
     <t>How much is the difference in the number of travelers between the vehicle used most and least?</t>
   </si>
   <si>
+    <t>Difference: 40</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>Difference: 72</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>Difference: 27</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>Difference: 57</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>Difference: 17</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>Difference: 7</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>Difference: 74</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
+  </si>
+  <si>
+    <t>Difference: 8</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_11.png</t>
+  </si>
+  <si>
+    <t>Difference: 31</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_12.png</t>
+  </si>
+  <si>
+    <t>Difference: 55</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_13.png</t>
+  </si>
+  <si>
+    <t>Difference: 51</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_14.png</t>
+  </si>
+  <si>
+    <t>Difference: 59</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_15.png</t>
+  </si>
+  <si>
+    <t>Difference: 69</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_16.png</t>
+  </si>
+  <si>
+    <t>Difference: 48</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_17.png</t>
+  </si>
+  <si>
+    <t>Difference: 18</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_18.png</t>
+  </si>
+  <si>
+    <t>Difference: 35</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_19.png</t>
+  </si>
+  <si>
+    <t>Difference: 64</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_20.png</t>
+  </si>
+  <si>
+    <t>Difference: 11</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_21.png</t>
+  </si>
+  <si>
+    <t>Difference: 32</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_22.png</t>
+  </si>
+  <si>
+    <t>Difference: 30</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_23.png</t>
+  </si>
+  <si>
+    <t>Difference: 4</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_24.png</t>
+  </si>
+  <si>
+    <t>Difference: 36</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_25.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_26.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_27.png</t>
+  </si>
+  <si>
+    <t>Difference: 52</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_28.png</t>
+  </si>
+  <si>
+    <t>Difference: 19</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_29.png</t>
+  </si>
+  <si>
+    <t>Difference: 68</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_30.png</t>
+  </si>
+  <si>
+    <t>Difference: 2</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_31.png</t>
+  </si>
+  <si>
+    <t>Difference: 24</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_32.png</t>
+  </si>
+  <si>
+    <t>Difference: 49</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_33.png</t>
+  </si>
+  <si>
+    <t>Difference: 10</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_34.png</t>
+  </si>
+  <si>
+    <t>Difference: 9</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_35.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_36.png</t>
+  </si>
+  <si>
+    <t>Difference: 5</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_37.png</t>
+  </si>
+  <si>
+    <t>Difference: 46</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_38.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_39.png</t>
+  </si>
+  <si>
+    <t>Difference: 21</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_40.png</t>
+  </si>
+  <si>
+    <t>Difference: 56</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_41.png</t>
+  </si>
+  <si>
+    <t>Difference: 16</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_42.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_43.png</t>
+  </si>
+  <si>
+    <t>Difference: 71</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_44.png</t>
+  </si>
+  <si>
+    <t>Difference: 39</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_45.png</t>
+  </si>
+  <si>
+    <t>Difference: 0</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_46.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_47.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_48.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_49.png</t>
+  </si>
+  <si>
+    <t>Difference: 38</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_50.png</t>
+  </si>
+  <si>
+    <t>Difference: 22</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_51.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_52.png</t>
+  </si>
+  <si>
+    <t>Difference: 78</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_53.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_54.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_55.png</t>
+  </si>
+  <si>
+    <t>Difference: 3</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_56.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_57.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_58.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_59.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_60.png</t>
+  </si>
+  <si>
+    <t>Difference: 50</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_61.png</t>
+  </si>
+  <si>
+    <t>Difference: 34</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_62.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_63.png</t>
+  </si>
+  <si>
+    <t>Difference: 83</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_64.png</t>
+  </si>
+  <si>
+    <t>Difference: 26</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_65.png</t>
+  </si>
+  <si>
+    <t>Difference: 12</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_66.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_67.png</t>
+  </si>
+  <si>
+    <t>Difference: 29</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_68.png</t>
+  </si>
+  <si>
+    <t>Difference: 82</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_69.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_70.png</t>
+  </si>
+  <si>
+    <t>Difference: 13</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_71.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_72.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_73.png</t>
+  </si>
+  <si>
+    <t>Difference: 65</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_74.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_75.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_76.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_77.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_78.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_79.png</t>
+  </si>
+  <si>
+    <t>Difference: 15</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_80.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_81.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_82.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_83.png</t>
+  </si>
+  <si>
+    <t>Difference: 63</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_84.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_85.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_86.png</t>
+  </si>
+  <si>
+    <t>Difference: 89</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_87.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_88.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_89.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_90.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_91.png</t>
+  </si>
+  <si>
+    <t>Difference: 44</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_92.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_93.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_94.png</t>
+  </si>
+  <si>
+    <t>Difference: 45</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_95.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_96.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_97.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_98.png</t>
+  </si>
+  <si>
+    <t>Difference: 76</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_99.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_100.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_101.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_102.png</t>
+  </si>
+  <si>
+    <t>Difference: 1</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_103.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_104.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_105.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_106.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_107.png</t>
+  </si>
+  <si>
     <t>Difference: 20</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>Difference: 29</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>Difference: 13</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>Difference: 78</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_108.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_109.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_110.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_111.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_112.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_113.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_114.png</t>
   </si>
   <si>
     <t>Difference: 47</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>Difference: 42</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_115.png</t>
+  </si>
+  <si>
+    <t>Difference: 43</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_116.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_117.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_118.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_119.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_120.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_121.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_122.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_123.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_124.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_125.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_126.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_127.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_128.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_129.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_130.png</t>
+  </si>
+  <si>
+    <t>Difference: 97</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_131.png</t>
   </si>
   <si>
     <t>Difference: 6</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>Difference: 31</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>Difference: 35</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
-  </si>
-  <si>
-    <t>Difference: 5</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_11.png</t>
-  </si>
-  <si>
-    <t>Difference: 19</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_12.png</t>
-  </si>
-  <si>
-    <t>Difference: 60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_13.png</t>
-  </si>
-  <si>
-    <t>Difference: 15</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_14.png</t>
-  </si>
-  <si>
-    <t>Difference: 58</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_15.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_16.png</t>
-  </si>
-  <si>
-    <t>Difference: 27</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_17.png</t>
-  </si>
-  <si>
-    <t>Difference: 38</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_18.png</t>
-  </si>
-  <si>
-    <t>Difference: 62</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_19.png</t>
-  </si>
-  <si>
-    <t>Difference: 21</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_20.png</t>
-  </si>
-  <si>
-    <t>Difference: 82</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_21.png</t>
-  </si>
-  <si>
-    <t>Difference: 46</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_22.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_23.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_24.png</t>
-  </si>
-  <si>
-    <t>Difference: 55</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_25.png</t>
-  </si>
-  <si>
-    <t>Difference: 50</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_26.png</t>
-  </si>
-  <si>
-    <t>Difference: 59</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_27.png</t>
-  </si>
-  <si>
-    <t>Difference: 22</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_28.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_29.png</t>
-  </si>
-  <si>
-    <t>Difference: 64</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_30.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_31.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_32.png</t>
-  </si>
-  <si>
-    <t>Difference: 57</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_33.png</t>
-  </si>
-  <si>
-    <t>Difference: 49</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_34.png</t>
-  </si>
-  <si>
-    <t>Difference: 34</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_35.png</t>
-  </si>
-  <si>
-    <t>Difference: 72</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_36.png</t>
-  </si>
-  <si>
-    <t>Difference: 8</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_37.png</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_132.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_133.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_134.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_135.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_136.png</t>
+  </si>
+  <si>
+    <t>Difference: 37</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_137.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_138.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_139.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_140.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_141.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_142.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_143.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_144.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_145.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_146.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_147.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_148.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_149.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_150.png</t>
   </si>
   <si>
     <t>Difference: 41</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_38.png</t>
-  </si>
-  <si>
-    <t>Difference: 77</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_39.png</t>
-  </si>
-  <si>
-    <t>Difference: 28</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_40.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_41.png</t>
-  </si>
-  <si>
-    <t>Difference: 71</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_42.png</t>
-  </si>
-  <si>
-    <t>Difference: 76</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_43.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_44.png</t>
-  </si>
-  <si>
-    <t>Difference: 4</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_45.png</t>
-  </si>
-  <si>
-    <t>Difference: 11</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_46.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_47.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_48.png</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_151.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_152.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_153.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_154.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_155.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_156.png</t>
+  </si>
+  <si>
+    <t>Difference: 66</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_157.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_158.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_159.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_160.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_161.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_162.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_163.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_164.png</t>
+  </si>
+  <si>
+    <t>Difference: 73</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_165.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_166.png</t>
+  </si>
+  <si>
+    <t>Difference: 80</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_167.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_168.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_169.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_170.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_171.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_172.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_173.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_174.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_175.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_176.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_177.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_178.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_179.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_180.png</t>
+  </si>
+  <si>
+    <t>Difference: 33</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_181.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_182.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_183.png</t>
+  </si>
+  <si>
+    <t>Difference: 61</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_184.png</t>
+  </si>
+  <si>
+    <t>Difference: 91</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_185.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_186.png</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_187.png</t>
   </si>
   <si>
     <t>Difference: 25</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_49.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_50.png</t>
-  </si>
-  <si>
-    <t>Difference: 23</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_51.png</t>
-  </si>
-  <si>
-    <t>Difference: 95</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_52.png</t>
-  </si>
-  <si>
-    <t>Difference: 75</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_53.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_54.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_55.png</t>
-  </si>
-  <si>
-    <t>Difference: 2</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_56.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_57.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_58.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_59.png</t>
-  </si>
-  <si>
-    <t>Difference: 14</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_60.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_61.png</t>
-  </si>
-  <si>
-    <t>Difference: 40</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_62.png</t>
-  </si>
-  <si>
-    <t>Difference: 10</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_63.png</t>
-  </si>
-  <si>
-    <t>Difference: 52</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_64.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_65.png</t>
-  </si>
-  <si>
-    <t>Difference: 18</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_66.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_67.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_68.png</t>
-  </si>
-  <si>
-    <t>Difference: 81</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_69.png</t>
-  </si>
-  <si>
-    <t>Difference: 16</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_70.png</t>
-  </si>
-  <si>
-    <t>Difference: 32</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_71.png</t>
-  </si>
-  <si>
-    <t>Difference: 24</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_72.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_73.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_74.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_75.png</t>
-  </si>
-  <si>
-    <t>Difference: 61</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_76.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_77.png</t>
-  </si>
-  <si>
-    <t>Difference: 12</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_78.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_79.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_80.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_81.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_82.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_83.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_84.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_85.png</t>
-  </si>
-  <si>
-    <t>Difference: 39</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_86.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_87.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_88.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_89.png</t>
-  </si>
-  <si>
-    <t>Difference: 17</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_90.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_91.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_92.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_93.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_94.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_95.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_96.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_97.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_98.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_99.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_100.png</t>
-  </si>
-  <si>
-    <t>Difference: 36</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_101.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_102.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_103.png</t>
-  </si>
-  <si>
-    <t>Difference: 30</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_104.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_105.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_106.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_107.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_108.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_109.png</t>
-  </si>
-  <si>
-    <t>Difference: 1</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_110.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_111.png</t>
-  </si>
-  <si>
-    <t>Difference: 66</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_112.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_113.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_114.png</t>
-  </si>
-  <si>
-    <t>Difference: 80</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_115.png</t>
-  </si>
-  <si>
-    <t>Difference: 26</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_116.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_117.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_118.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_119.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_120.png</t>
-  </si>
-  <si>
-    <t>Difference: 79</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_121.png</t>
-  </si>
-  <si>
-    <t>Difference: 9</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_122.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_123.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_124.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_125.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_126.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_127.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_128.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_129.png</t>
-  </si>
-  <si>
-    <t>Difference: 37</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_130.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_131.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_132.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_133.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_134.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_135.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_136.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_137.png</t>
-  </si>
-  <si>
-    <t>Difference: 53</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_138.png</t>
-  </si>
-  <si>
-    <t>Difference: 45</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_139.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_140.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_141.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_142.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_143.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_144.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_145.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_146.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_147.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_148.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_149.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_150.png</t>
-  </si>
-  <si>
-    <t>Difference: 63</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_151.png</t>
-  </si>
-  <si>
-    <t>Difference: 54</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_152.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_153.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_154.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_155.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_156.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_157.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_158.png</t>
-  </si>
-  <si>
-    <t>Difference: 0</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_159.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_160.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_161.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_162.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_163.png</t>
-  </si>
-  <si>
-    <t>Difference: 68</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_164.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_165.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_166.png</t>
-  </si>
-  <si>
-    <t>Difference: 43</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_167.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_168.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_169.png</t>
-  </si>
-  <si>
-    <t>Difference: 65</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_170.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_171.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_172.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_173.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_174.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_175.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_176.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_177.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_178.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_179.png</t>
-  </si>
-  <si>
-    <t>Difference: 3</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_180.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_181.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_182.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_183.png</t>
-  </si>
-  <si>
-    <t>Difference: 51</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_184.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_185.png</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_186.png</t>
-  </si>
-  <si>
-    <t>Difference: 56</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_187.png</t>
-  </si>
-  <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_188.png</t>
   </si>
   <si>
@@ -824,16 +815,10 @@
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_190.png</t>
   </si>
   <si>
-    <t>Difference: 33</t>
-  </si>
-  <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_191.png</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_192.png</t>
-  </si>
-  <si>
-    <t>Difference: 85</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_193.png</t>
@@ -1020,7 +1005,7 @@
         <v>5</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1028,13 +1013,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" t="s">
         <v>19</v>
-      </c>
-      <c r="C9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1042,13 +1027,13 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" t="s">
         <v>21</v>
-      </c>
-      <c r="C10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="11">
@@ -1056,13 +1041,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
         <v>5</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -1070,13 +1055,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13">
@@ -1084,13 +1069,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
         <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
@@ -1098,13 +1083,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
         <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -1112,13 +1097,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -1126,13 +1111,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
@@ -1140,13 +1125,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
         <v>34</v>
-      </c>
-      <c r="C17" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="18">
@@ -1154,13 +1139,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" t="s">
         <v>36</v>
-      </c>
-      <c r="C18" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="19">
@@ -1168,13 +1153,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
         <v>38</v>
-      </c>
-      <c r="C19" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="20">
@@ -1182,13 +1167,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" t="s">
         <v>40</v>
-      </c>
-      <c r="C20" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="21">
@@ -1196,13 +1181,13 @@
         <v>20.0</v>
       </c>
       <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" t="s">
         <v>42</v>
-      </c>
-      <c r="C21" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="22">
@@ -1210,13 +1195,13 @@
         <v>21.0</v>
       </c>
       <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" t="s">
         <v>44</v>
-      </c>
-      <c r="C22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="23">
@@ -1224,13 +1209,13 @@
         <v>22.0</v>
       </c>
       <c r="B23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
         <v>46</v>
-      </c>
-      <c r="C23" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="24">
@@ -1244,7 +1229,7 @@
         <v>5</v>
       </c>
       <c r="D24" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25">
@@ -1252,13 +1237,13 @@
         <v>24.0</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C25" t="s">
         <v>5</v>
       </c>
       <c r="D25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26">
@@ -1266,13 +1251,13 @@
         <v>25.0</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C26" t="s">
         <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27">
@@ -1286,7 +1271,7 @@
         <v>5</v>
       </c>
       <c r="D27" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28">
@@ -1294,13 +1279,13 @@
         <v>27.0</v>
       </c>
       <c r="B28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" t="s">
         <v>54</v>
-      </c>
-      <c r="C28" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="29">
@@ -1308,13 +1293,13 @@
         <v>28.0</v>
       </c>
       <c r="B29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" t="s">
         <v>56</v>
-      </c>
-      <c r="C29" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="30">
@@ -1342,7 +1327,7 @@
         <v>5</v>
       </c>
       <c r="D31" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32">
@@ -1350,13 +1335,13 @@
         <v>31.0</v>
       </c>
       <c r="B32" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C32" t="s">
         <v>5</v>
       </c>
       <c r="D32" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33">
@@ -1364,13 +1349,13 @@
         <v>32.0</v>
       </c>
       <c r="B33" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C33" t="s">
         <v>5</v>
       </c>
       <c r="D33" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34">
@@ -1378,13 +1363,13 @@
         <v>33.0</v>
       </c>
       <c r="B34" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
         <v>5</v>
       </c>
       <c r="D34" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35">
@@ -1392,13 +1377,13 @@
         <v>34.0</v>
       </c>
       <c r="B35" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C35" t="s">
         <v>5</v>
       </c>
       <c r="D35" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36">
@@ -1406,13 +1391,13 @@
         <v>35.0</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C36" t="s">
         <v>5</v>
       </c>
       <c r="D36" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
     </row>
     <row r="37">
@@ -1420,13 +1405,13 @@
         <v>36.0</v>
       </c>
       <c r="B37" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C37" t="s">
         <v>5</v>
       </c>
       <c r="D37" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38">
@@ -1434,13 +1419,13 @@
         <v>37.0</v>
       </c>
       <c r="B38" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C38" t="s">
         <v>5</v>
       </c>
       <c r="D38" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39">
@@ -1448,13 +1433,13 @@
         <v>38.0</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C39" t="s">
         <v>5</v>
       </c>
       <c r="D39" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40">
@@ -1482,7 +1467,7 @@
         <v>5</v>
       </c>
       <c r="D41" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42">
@@ -1490,13 +1475,13 @@
         <v>41.0</v>
       </c>
       <c r="B42" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C42" t="s">
         <v>5</v>
       </c>
       <c r="D42" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="43">
@@ -1504,13 +1489,13 @@
         <v>42.0</v>
       </c>
       <c r="B43" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C43" t="s">
         <v>5</v>
       </c>
       <c r="D43" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
     </row>
     <row r="44">
@@ -1524,7 +1509,7 @@
         <v>5</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
     </row>
     <row r="45">
@@ -1532,13 +1517,13 @@
         <v>44.0</v>
       </c>
       <c r="B45" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C45" t="s">
         <v>5</v>
       </c>
       <c r="D45" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46">
@@ -1546,13 +1531,13 @@
         <v>45.0</v>
       </c>
       <c r="B46" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C46" t="s">
         <v>5</v>
       </c>
       <c r="D46" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47">
@@ -1560,13 +1545,13 @@
         <v>46.0</v>
       </c>
       <c r="B47" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C47" t="s">
         <v>5</v>
       </c>
       <c r="D47" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48">
@@ -1574,13 +1559,13 @@
         <v>47.0</v>
       </c>
       <c r="B48" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C48" t="s">
         <v>5</v>
       </c>
       <c r="D48" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49">
@@ -1588,13 +1573,13 @@
         <v>48.0</v>
       </c>
       <c r="B49" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
         <v>5</v>
       </c>
       <c r="D49" t="s">
-        <v>90</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50">
@@ -1608,7 +1593,7 @@
         <v>5</v>
       </c>
       <c r="D50" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
     </row>
     <row r="51">
@@ -1616,13 +1601,13 @@
         <v>50.0</v>
       </c>
       <c r="B51" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C51" t="s">
         <v>5</v>
       </c>
       <c r="D51" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52">
@@ -1630,13 +1615,13 @@
         <v>51.0</v>
       </c>
       <c r="B52" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C52" t="s">
         <v>5</v>
       </c>
       <c r="D52" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="53">
@@ -1664,7 +1649,7 @@
         <v>5</v>
       </c>
       <c r="D54" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
     </row>
     <row r="55">
@@ -1678,7 +1663,7 @@
         <v>5</v>
       </c>
       <c r="D55" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56">
@@ -1706,7 +1691,7 @@
         <v>5</v>
       </c>
       <c r="D57" t="s">
-        <v>64</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58">
@@ -1720,7 +1705,7 @@
         <v>5</v>
       </c>
       <c r="D58" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59">
@@ -1734,7 +1719,7 @@
         <v>5</v>
       </c>
       <c r="D59" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60">
@@ -1748,7 +1733,7 @@
         <v>5</v>
       </c>
       <c r="D60" t="s">
-        <v>106</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61">
@@ -1756,13 +1741,13 @@
         <v>60.0</v>
       </c>
       <c r="B61" t="s">
+        <v>106</v>
+      </c>
+      <c r="C61" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" t="s">
         <v>107</v>
-      </c>
-      <c r="C61" t="s">
-        <v>5</v>
-      </c>
-      <c r="D61" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="62">
@@ -1790,7 +1775,7 @@
         <v>5</v>
       </c>
       <c r="D63" t="s">
-        <v>111</v>
+        <v>44</v>
       </c>
     </row>
     <row r="64">
@@ -1798,13 +1783,13 @@
         <v>63.0</v>
       </c>
       <c r="B64" t="s">
+        <v>111</v>
+      </c>
+      <c r="C64" t="s">
+        <v>5</v>
+      </c>
+      <c r="D64" t="s">
         <v>112</v>
-      </c>
-      <c r="C64" t="s">
-        <v>5</v>
-      </c>
-      <c r="D64" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="65">
@@ -1812,13 +1797,13 @@
         <v>64.0</v>
       </c>
       <c r="B65" t="s">
+        <v>113</v>
+      </c>
+      <c r="C65" t="s">
+        <v>5</v>
+      </c>
+      <c r="D65" t="s">
         <v>114</v>
-      </c>
-      <c r="C65" t="s">
-        <v>5</v>
-      </c>
-      <c r="D65" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="66">
@@ -1846,7 +1831,7 @@
         <v>5</v>
       </c>
       <c r="D67" t="s">
-        <v>116</v>
+        <v>50</v>
       </c>
     </row>
     <row r="68">
@@ -1860,7 +1845,7 @@
         <v>5</v>
       </c>
       <c r="D68" t="s">
-        <v>35</v>
+        <v>119</v>
       </c>
     </row>
     <row r="69">
@@ -1868,13 +1853,13 @@
         <v>68.0</v>
       </c>
       <c r="B69" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C69" t="s">
         <v>5</v>
       </c>
       <c r="D69" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70">
@@ -1882,13 +1867,13 @@
         <v>69.0</v>
       </c>
       <c r="B70" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C70" t="s">
         <v>5</v>
       </c>
       <c r="D70" t="s">
-        <v>122</v>
+        <v>42</v>
       </c>
     </row>
     <row r="71">
@@ -1916,7 +1901,7 @@
         <v>5</v>
       </c>
       <c r="D72" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
     </row>
     <row r="73">
@@ -1924,13 +1909,13 @@
         <v>72.0</v>
       </c>
       <c r="B73" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C73" t="s">
         <v>5</v>
       </c>
       <c r="D73" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
     </row>
     <row r="74">
@@ -1938,13 +1923,13 @@
         <v>73.0</v>
       </c>
       <c r="B74" t="s">
+        <v>127</v>
+      </c>
+      <c r="C74" t="s">
+        <v>5</v>
+      </c>
+      <c r="D74" t="s">
         <v>128</v>
-      </c>
-      <c r="C74" t="s">
-        <v>5</v>
-      </c>
-      <c r="D74" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="75">
@@ -1958,7 +1943,7 @@
         <v>5</v>
       </c>
       <c r="D75" t="s">
-        <v>90</v>
+        <v>42</v>
       </c>
     </row>
     <row r="76">
@@ -1972,7 +1957,7 @@
         <v>5</v>
       </c>
       <c r="D76" t="s">
-        <v>131</v>
+        <v>94</v>
       </c>
     </row>
     <row r="77">
@@ -1980,13 +1965,13 @@
         <v>76.0</v>
       </c>
       <c r="B77" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C77" t="s">
         <v>5</v>
       </c>
       <c r="D77" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="78">
@@ -1994,13 +1979,13 @@
         <v>77.0</v>
       </c>
       <c r="B78" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C78" t="s">
         <v>5</v>
       </c>
       <c r="D78" t="s">
-        <v>134</v>
+        <v>97</v>
       </c>
     </row>
     <row r="79">
@@ -2008,13 +1993,13 @@
         <v>78.0</v>
       </c>
       <c r="B79" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C79" t="s">
         <v>5</v>
       </c>
       <c r="D79" t="s">
-        <v>122</v>
+        <v>36</v>
       </c>
     </row>
     <row r="80">
@@ -2022,13 +2007,13 @@
         <v>79.0</v>
       </c>
       <c r="B80" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C80" t="s">
         <v>5</v>
       </c>
       <c r="D80" t="s">
-        <v>43</v>
+        <v>135</v>
       </c>
     </row>
     <row r="81">
@@ -2036,13 +2021,13 @@
         <v>80.0</v>
       </c>
       <c r="B81" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C81" t="s">
         <v>5</v>
       </c>
       <c r="D81" t="s">
-        <v>106</v>
+        <v>26</v>
       </c>
     </row>
     <row r="82">
@@ -2050,13 +2035,13 @@
         <v>81.0</v>
       </c>
       <c r="B82" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C82" t="s">
         <v>5</v>
       </c>
       <c r="D82" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
     </row>
     <row r="83">
@@ -2064,13 +2049,13 @@
         <v>82.0</v>
       </c>
       <c r="B83" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C83" t="s">
         <v>5</v>
       </c>
       <c r="D83" t="s">
-        <v>39</v>
+        <v>87</v>
       </c>
     </row>
     <row r="84">
@@ -2078,13 +2063,13 @@
         <v>83.0</v>
       </c>
       <c r="B84" t="s">
+        <v>139</v>
+      </c>
+      <c r="C84" t="s">
+        <v>5</v>
+      </c>
+      <c r="D84" t="s">
         <v>140</v>
-      </c>
-      <c r="C84" t="s">
-        <v>5</v>
-      </c>
-      <c r="D84" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="85">
@@ -2098,7 +2083,7 @@
         <v>5</v>
       </c>
       <c r="D85" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
     </row>
     <row r="86">
@@ -2112,7 +2097,7 @@
         <v>5</v>
       </c>
       <c r="D86" t="s">
-        <v>143</v>
+        <v>36</v>
       </c>
     </row>
     <row r="87">
@@ -2120,13 +2105,13 @@
         <v>86.0</v>
       </c>
       <c r="B87" t="s">
+        <v>143</v>
+      </c>
+      <c r="C87" t="s">
+        <v>5</v>
+      </c>
+      <c r="D87" t="s">
         <v>144</v>
-      </c>
-      <c r="C87" t="s">
-        <v>5</v>
-      </c>
-      <c r="D87" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="88">
@@ -2140,7 +2125,7 @@
         <v>5</v>
       </c>
       <c r="D88" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
     </row>
     <row r="89">
@@ -2154,7 +2139,7 @@
         <v>5</v>
       </c>
       <c r="D89" t="s">
-        <v>116</v>
+        <v>73</v>
       </c>
     </row>
     <row r="90">
@@ -2168,7 +2153,7 @@
         <v>5</v>
       </c>
       <c r="D90" t="s">
-        <v>148</v>
+        <v>87</v>
       </c>
     </row>
     <row r="91">
@@ -2176,13 +2161,13 @@
         <v>90.0</v>
       </c>
       <c r="B91" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C91" t="s">
         <v>5</v>
       </c>
       <c r="D91" t="s">
-        <v>28</v>
+        <v>80</v>
       </c>
     </row>
     <row r="92">
@@ -2190,13 +2175,13 @@
         <v>91.0</v>
       </c>
       <c r="B92" t="s">
+        <v>149</v>
+      </c>
+      <c r="C92" t="s">
+        <v>5</v>
+      </c>
+      <c r="D92" t="s">
         <v>150</v>
-      </c>
-      <c r="C92" t="s">
-        <v>5</v>
-      </c>
-      <c r="D92" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="93">
@@ -2210,7 +2195,7 @@
         <v>5</v>
       </c>
       <c r="D93" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94">
@@ -2224,7 +2209,7 @@
         <v>5</v>
       </c>
       <c r="D94" t="s">
-        <v>111</v>
+        <v>28</v>
       </c>
     </row>
     <row r="95">
@@ -2238,7 +2223,7 @@
         <v>5</v>
       </c>
       <c r="D95" t="s">
-        <v>6</v>
+        <v>154</v>
       </c>
     </row>
     <row r="96">
@@ -2246,13 +2231,13 @@
         <v>95.0</v>
       </c>
       <c r="B96" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C96" t="s">
         <v>5</v>
       </c>
       <c r="D96" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
     </row>
     <row r="97">
@@ -2260,13 +2245,13 @@
         <v>96.0</v>
       </c>
       <c r="B97" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C97" t="s">
         <v>5</v>
       </c>
       <c r="D97" t="s">
-        <v>93</v>
+        <v>44</v>
       </c>
     </row>
     <row r="98">
@@ -2274,13 +2259,13 @@
         <v>97.0</v>
       </c>
       <c r="B98" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C98" t="s">
         <v>5</v>
       </c>
       <c r="D98" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="99">
@@ -2288,13 +2273,13 @@
         <v>98.0</v>
       </c>
       <c r="B99" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C99" t="s">
         <v>5</v>
       </c>
       <c r="D99" t="s">
-        <v>49</v>
+        <v>159</v>
       </c>
     </row>
     <row r="100">
@@ -2302,13 +2287,13 @@
         <v>99.0</v>
       </c>
       <c r="B100" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C100" t="s">
         <v>5</v>
       </c>
       <c r="D100" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
     </row>
     <row r="101">
@@ -2316,13 +2301,13 @@
         <v>100.0</v>
       </c>
       <c r="B101" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C101" t="s">
         <v>5</v>
       </c>
       <c r="D101" t="s">
-        <v>160</v>
+        <v>46</v>
       </c>
     </row>
     <row r="102">
@@ -2330,13 +2315,13 @@
         <v>101.0</v>
       </c>
       <c r="B102" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C102" t="s">
         <v>5</v>
       </c>
       <c r="D102" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
     </row>
     <row r="103">
@@ -2344,13 +2329,13 @@
         <v>102.0</v>
       </c>
       <c r="B103" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C103" t="s">
         <v>5</v>
       </c>
       <c r="D103" t="s">
-        <v>124</v>
+        <v>164</v>
       </c>
     </row>
     <row r="104">
@@ -2358,13 +2343,13 @@
         <v>103.0</v>
       </c>
       <c r="B104" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C104" t="s">
         <v>5</v>
       </c>
       <c r="D104" t="s">
-        <v>164</v>
+        <v>144</v>
       </c>
     </row>
     <row r="105">
@@ -2372,13 +2357,13 @@
         <v>104.0</v>
       </c>
       <c r="B105" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C105" t="s">
         <v>5</v>
       </c>
       <c r="D105" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="106">
@@ -2386,13 +2371,13 @@
         <v>105.0</v>
       </c>
       <c r="B106" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C106" t="s">
         <v>5</v>
       </c>
       <c r="D106" t="s">
-        <v>164</v>
+        <v>116</v>
       </c>
     </row>
     <row r="107">
@@ -2400,13 +2385,13 @@
         <v>106.0</v>
       </c>
       <c r="B107" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C107" t="s">
         <v>5</v>
       </c>
       <c r="D107" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
     </row>
     <row r="108">
@@ -2414,13 +2399,13 @@
         <v>107.0</v>
       </c>
       <c r="B108" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C108" t="s">
         <v>5</v>
       </c>
       <c r="D108" t="s">
-        <v>122</v>
+        <v>170</v>
       </c>
     </row>
     <row r="109">
@@ -2428,13 +2413,13 @@
         <v>108.0</v>
       </c>
       <c r="B109" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C109" t="s">
         <v>5</v>
       </c>
       <c r="D109" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="110">
@@ -2442,13 +2427,13 @@
         <v>109.0</v>
       </c>
       <c r="B110" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C110" t="s">
         <v>5</v>
       </c>
       <c r="D110" t="s">
-        <v>171</v>
+        <v>32</v>
       </c>
     </row>
     <row r="111">
@@ -2456,13 +2441,13 @@
         <v>110.0</v>
       </c>
       <c r="B111" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C111" t="s">
         <v>5</v>
       </c>
       <c r="D111" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="112">
@@ -2470,13 +2455,13 @@
         <v>111.0</v>
       </c>
       <c r="B112" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C112" t="s">
         <v>5</v>
       </c>
       <c r="D112" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
     </row>
     <row r="113">
@@ -2490,7 +2475,7 @@
         <v>5</v>
       </c>
       <c r="D113" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
     </row>
     <row r="114">
@@ -2504,7 +2489,7 @@
         <v>5</v>
       </c>
       <c r="D114" t="s">
-        <v>111</v>
+        <v>54</v>
       </c>
     </row>
     <row r="115">
@@ -2546,7 +2531,7 @@
         <v>5</v>
       </c>
       <c r="D117" t="s">
-        <v>116</v>
+        <v>85</v>
       </c>
     </row>
     <row r="118">
@@ -2560,7 +2545,7 @@
         <v>5</v>
       </c>
       <c r="D118" t="s">
-        <v>171</v>
+        <v>50</v>
       </c>
     </row>
     <row r="119">
@@ -2574,7 +2559,7 @@
         <v>5</v>
       </c>
       <c r="D119" t="s">
-        <v>72</v>
+        <v>24</v>
       </c>
     </row>
     <row r="120">
@@ -2588,7 +2573,7 @@
         <v>5</v>
       </c>
       <c r="D120" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
     </row>
     <row r="121">
@@ -2602,7 +2587,7 @@
         <v>5</v>
       </c>
       <c r="D121" t="s">
-        <v>186</v>
+        <v>114</v>
       </c>
     </row>
     <row r="122">
@@ -2610,13 +2595,13 @@
         <v>121.0</v>
       </c>
       <c r="B122" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C122" t="s">
         <v>5</v>
       </c>
       <c r="D122" t="s">
-        <v>188</v>
+        <v>78</v>
       </c>
     </row>
     <row r="123">
@@ -2624,13 +2609,13 @@
         <v>122.0</v>
       </c>
       <c r="B123" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C123" t="s">
         <v>5</v>
       </c>
       <c r="D123" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="124">
@@ -2638,13 +2623,13 @@
         <v>123.0</v>
       </c>
       <c r="B124" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C124" t="s">
         <v>5</v>
       </c>
       <c r="D124" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="125">
@@ -2652,13 +2637,13 @@
         <v>124.0</v>
       </c>
       <c r="B125" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C125" t="s">
         <v>5</v>
       </c>
       <c r="D125" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
     </row>
     <row r="126">
@@ -2666,13 +2651,13 @@
         <v>125.0</v>
       </c>
       <c r="B126" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C126" t="s">
         <v>5</v>
       </c>
       <c r="D126" t="s">
-        <v>171</v>
+        <v>73</v>
       </c>
     </row>
     <row r="127">
@@ -2680,13 +2665,13 @@
         <v>126.0</v>
       </c>
       <c r="B127" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C127" t="s">
         <v>5</v>
       </c>
       <c r="D127" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
     </row>
     <row r="128">
@@ -2694,13 +2679,13 @@
         <v>127.0</v>
       </c>
       <c r="B128" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C128" t="s">
         <v>5</v>
       </c>
       <c r="D128" t="s">
-        <v>79</v>
+        <v>32</v>
       </c>
     </row>
     <row r="129">
@@ -2708,13 +2693,13 @@
         <v>128.0</v>
       </c>
       <c r="B129" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C129" t="s">
         <v>5</v>
       </c>
       <c r="D129" t="s">
-        <v>72</v>
+        <v>135</v>
       </c>
     </row>
     <row r="130">
@@ -2722,13 +2707,13 @@
         <v>129.0</v>
       </c>
       <c r="B130" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C130" t="s">
         <v>5</v>
       </c>
       <c r="D130" t="s">
-        <v>197</v>
+        <v>34</v>
       </c>
     </row>
     <row r="131">
@@ -2736,13 +2721,13 @@
         <v>130.0</v>
       </c>
       <c r="B131" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C131" t="s">
         <v>5</v>
       </c>
       <c r="D131" t="s">
-        <v>124</v>
+        <v>196</v>
       </c>
     </row>
     <row r="132">
@@ -2750,13 +2735,13 @@
         <v>131.0</v>
       </c>
       <c r="B132" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C132" t="s">
         <v>5</v>
       </c>
       <c r="D132" t="s">
-        <v>171</v>
+        <v>198</v>
       </c>
     </row>
     <row r="133">
@@ -2764,13 +2749,13 @@
         <v>132.0</v>
       </c>
       <c r="B133" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C133" t="s">
         <v>5</v>
       </c>
       <c r="D133" t="s">
-        <v>174</v>
+        <v>12</v>
       </c>
     </row>
     <row r="134">
@@ -2778,13 +2763,13 @@
         <v>133.0</v>
       </c>
       <c r="B134" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C134" t="s">
         <v>5</v>
       </c>
       <c r="D134" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
     </row>
     <row r="135">
@@ -2792,13 +2777,13 @@
         <v>134.0</v>
       </c>
       <c r="B135" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C135" t="s">
         <v>5</v>
       </c>
       <c r="D135" t="s">
-        <v>97</v>
+        <v>38</v>
       </c>
     </row>
     <row r="136">
@@ -2806,13 +2791,13 @@
         <v>135.0</v>
       </c>
       <c r="B136" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C136" t="s">
         <v>5</v>
       </c>
       <c r="D136" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="137">
@@ -2820,13 +2805,13 @@
         <v>136.0</v>
       </c>
       <c r="B137" t="s">
+        <v>203</v>
+      </c>
+      <c r="C137" t="s">
+        <v>5</v>
+      </c>
+      <c r="D137" t="s">
         <v>204</v>
-      </c>
-      <c r="C137" t="s">
-        <v>5</v>
-      </c>
-      <c r="D137" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="138">
@@ -2840,7 +2825,7 @@
         <v>5</v>
       </c>
       <c r="D138" t="s">
-        <v>206</v>
+        <v>24</v>
       </c>
     </row>
     <row r="139">
@@ -2848,13 +2833,13 @@
         <v>138.0</v>
       </c>
       <c r="B139" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C139" t="s">
         <v>5</v>
       </c>
       <c r="D139" t="s">
-        <v>208</v>
+        <v>135</v>
       </c>
     </row>
     <row r="140">
@@ -2862,13 +2847,13 @@
         <v>139.0</v>
       </c>
       <c r="B140" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C140" t="s">
         <v>5</v>
       </c>
       <c r="D140" t="s">
-        <v>66</v>
+        <v>6</v>
       </c>
     </row>
     <row r="141">
@@ -2876,13 +2861,13 @@
         <v>140.0</v>
       </c>
       <c r="B141" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C141" t="s">
         <v>5</v>
       </c>
       <c r="D141" t="s">
-        <v>109</v>
+        <v>34</v>
       </c>
     </row>
     <row r="142">
@@ -2890,13 +2875,13 @@
         <v>141.0</v>
       </c>
       <c r="B142" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C142" t="s">
         <v>5</v>
       </c>
       <c r="D142" t="s">
-        <v>14</v>
+        <v>170</v>
       </c>
     </row>
     <row r="143">
@@ -2904,13 +2889,13 @@
         <v>142.0</v>
       </c>
       <c r="B143" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C143" t="s">
         <v>5</v>
       </c>
       <c r="D143" t="s">
-        <v>188</v>
+        <v>68</v>
       </c>
     </row>
     <row r="144">
@@ -2918,13 +2903,13 @@
         <v>143.0</v>
       </c>
       <c r="B144" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C144" t="s">
         <v>5</v>
       </c>
       <c r="D144" t="s">
-        <v>113</v>
+        <v>21</v>
       </c>
     </row>
     <row r="145">
@@ -2932,13 +2917,13 @@
         <v>144.0</v>
       </c>
       <c r="B145" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C145" t="s">
         <v>5</v>
       </c>
       <c r="D145" t="s">
-        <v>35</v>
+        <v>109</v>
       </c>
     </row>
     <row r="146">
@@ -2946,13 +2931,13 @@
         <v>145.0</v>
       </c>
       <c r="B146" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C146" t="s">
         <v>5</v>
       </c>
       <c r="D146" t="s">
-        <v>174</v>
+        <v>16</v>
       </c>
     </row>
     <row r="147">
@@ -2960,13 +2945,13 @@
         <v>146.0</v>
       </c>
       <c r="B147" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C147" t="s">
         <v>5</v>
       </c>
       <c r="D147" t="s">
-        <v>79</v>
+        <v>101</v>
       </c>
     </row>
     <row r="148">
@@ -2974,13 +2959,13 @@
         <v>147.0</v>
       </c>
       <c r="B148" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C148" t="s">
         <v>5</v>
       </c>
       <c r="D148" t="s">
-        <v>131</v>
+        <v>94</v>
       </c>
     </row>
     <row r="149">
@@ -2988,13 +2973,13 @@
         <v>148.0</v>
       </c>
       <c r="B149" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C149" t="s">
         <v>5</v>
       </c>
       <c r="D149" t="s">
-        <v>134</v>
+        <v>10</v>
       </c>
     </row>
     <row r="150">
@@ -3002,13 +2987,13 @@
         <v>149.0</v>
       </c>
       <c r="B150" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C150" t="s">
         <v>5</v>
       </c>
       <c r="D150" t="s">
-        <v>116</v>
+        <v>68</v>
       </c>
     </row>
     <row r="151">
@@ -3016,13 +3001,13 @@
         <v>150.0</v>
       </c>
       <c r="B151" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C151" t="s">
         <v>5</v>
       </c>
       <c r="D151" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="152">
@@ -3030,13 +3015,13 @@
         <v>151.0</v>
       </c>
       <c r="B152" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C152" t="s">
         <v>5</v>
       </c>
       <c r="D152" t="s">
-        <v>223</v>
+        <v>107</v>
       </c>
     </row>
     <row r="153">
@@ -3044,13 +3029,13 @@
         <v>152.0</v>
       </c>
       <c r="B153" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C153" t="s">
         <v>5</v>
       </c>
       <c r="D153" t="s">
-        <v>70</v>
+        <v>135</v>
       </c>
     </row>
     <row r="154">
@@ -3058,13 +3043,13 @@
         <v>153.0</v>
       </c>
       <c r="B154" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C154" t="s">
         <v>5</v>
       </c>
       <c r="D154" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
     </row>
     <row r="155">
@@ -3072,13 +3057,13 @@
         <v>154.0</v>
       </c>
       <c r="B155" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C155" t="s">
         <v>5</v>
       </c>
       <c r="D155" t="s">
-        <v>37</v>
+        <v>97</v>
       </c>
     </row>
     <row r="156">
@@ -3086,13 +3071,13 @@
         <v>155.0</v>
       </c>
       <c r="B156" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C156" t="s">
         <v>5</v>
       </c>
       <c r="D156" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
     </row>
     <row r="157">
@@ -3100,13 +3085,13 @@
         <v>156.0</v>
       </c>
       <c r="B157" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C157" t="s">
         <v>5</v>
       </c>
       <c r="D157" t="s">
-        <v>93</v>
+        <v>226</v>
       </c>
     </row>
     <row r="158">
@@ -3114,13 +3099,13 @@
         <v>157.0</v>
       </c>
       <c r="B158" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C158" t="s">
         <v>5</v>
       </c>
       <c r="D158" t="s">
-        <v>55</v>
+        <v>80</v>
       </c>
     </row>
     <row r="159">
@@ -3128,13 +3113,13 @@
         <v>158.0</v>
       </c>
       <c r="B159" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C159" t="s">
         <v>5</v>
       </c>
       <c r="D159" t="s">
-        <v>231</v>
+        <v>85</v>
       </c>
     </row>
     <row r="160">
@@ -3142,13 +3127,13 @@
         <v>159.0</v>
       </c>
       <c r="B160" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C160" t="s">
         <v>5</v>
       </c>
       <c r="D160" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="161">
@@ -3156,13 +3141,13 @@
         <v>160.0</v>
       </c>
       <c r="B161" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C161" t="s">
         <v>5</v>
       </c>
       <c r="D161" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
     </row>
     <row r="162">
@@ -3170,13 +3155,13 @@
         <v>161.0</v>
       </c>
       <c r="B162" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C162" t="s">
         <v>5</v>
       </c>
       <c r="D162" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
     </row>
     <row r="163">
@@ -3184,13 +3169,13 @@
         <v>162.0</v>
       </c>
       <c r="B163" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C163" t="s">
         <v>5</v>
       </c>
       <c r="D163" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="164">
@@ -3198,13 +3183,13 @@
         <v>163.0</v>
       </c>
       <c r="B164" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C164" t="s">
         <v>5</v>
       </c>
       <c r="D164" t="s">
-        <v>237</v>
+        <v>135</v>
       </c>
     </row>
     <row r="165">
@@ -3212,13 +3197,13 @@
         <v>164.0</v>
       </c>
       <c r="B165" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C165" t="s">
         <v>5</v>
       </c>
       <c r="D165" t="s">
-        <v>24</v>
+        <v>235</v>
       </c>
     </row>
     <row r="166">
@@ -3226,13 +3211,13 @@
         <v>165.0</v>
       </c>
       <c r="B166" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C166" t="s">
         <v>5</v>
       </c>
       <c r="D166" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="167">
@@ -3240,13 +3225,13 @@
         <v>166.0</v>
       </c>
       <c r="B167" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C167" t="s">
         <v>5</v>
       </c>
       <c r="D167" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="168">
@@ -3254,13 +3239,13 @@
         <v>167.0</v>
       </c>
       <c r="B168" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C168" t="s">
         <v>5</v>
       </c>
       <c r="D168" t="s">
-        <v>109</v>
+        <v>180</v>
       </c>
     </row>
     <row r="169">
@@ -3268,13 +3253,13 @@
         <v>168.0</v>
       </c>
       <c r="B169" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C169" t="s">
         <v>5</v>
       </c>
       <c r="D169" t="s">
-        <v>188</v>
+        <v>24</v>
       </c>
     </row>
     <row r="170">
@@ -3282,13 +3267,13 @@
         <v>169.0</v>
       </c>
       <c r="B170" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C170" t="s">
         <v>5</v>
       </c>
       <c r="D170" t="s">
-        <v>245</v>
+        <v>16</v>
       </c>
     </row>
     <row r="171">
@@ -3296,13 +3281,13 @@
         <v>170.0</v>
       </c>
       <c r="B171" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="C171" t="s">
         <v>5</v>
       </c>
       <c r="D171" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="172">
@@ -3310,13 +3295,13 @@
         <v>171.0</v>
       </c>
       <c r="B172" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C172" t="s">
         <v>5</v>
       </c>
       <c r="D172" t="s">
-        <v>84</v>
+        <v>60</v>
       </c>
     </row>
     <row r="173">
@@ -3324,13 +3309,13 @@
         <v>172.0</v>
       </c>
       <c r="B173" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="C173" t="s">
         <v>5</v>
       </c>
       <c r="D173" t="s">
-        <v>84</v>
+        <v>164</v>
       </c>
     </row>
     <row r="174">
@@ -3338,13 +3323,13 @@
         <v>173.0</v>
       </c>
       <c r="B174" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="C174" t="s">
         <v>5</v>
       </c>
       <c r="D174" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
     </row>
     <row r="175">
@@ -3352,13 +3337,13 @@
         <v>174.0</v>
       </c>
       <c r="B175" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="C175" t="s">
         <v>5</v>
       </c>
       <c r="D175" t="s">
-        <v>231</v>
+        <v>21</v>
       </c>
     </row>
     <row r="176">
@@ -3366,13 +3351,13 @@
         <v>175.0</v>
       </c>
       <c r="B176" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="C176" t="s">
         <v>5</v>
       </c>
       <c r="D176" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="177">
@@ -3380,13 +3365,13 @@
         <v>176.0</v>
       </c>
       <c r="B177" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C177" t="s">
         <v>5</v>
       </c>
       <c r="D177" t="s">
-        <v>188</v>
+        <v>6</v>
       </c>
     </row>
     <row r="178">
@@ -3394,13 +3379,13 @@
         <v>177.0</v>
       </c>
       <c r="B178" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="C178" t="s">
         <v>5</v>
       </c>
       <c r="D178" t="s">
-        <v>245</v>
+        <v>76</v>
       </c>
     </row>
     <row r="179">
@@ -3408,13 +3393,13 @@
         <v>178.0</v>
       </c>
       <c r="B179" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="C179" t="s">
         <v>5</v>
       </c>
       <c r="D179" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
     </row>
     <row r="180">
@@ -3422,13 +3407,13 @@
         <v>179.0</v>
       </c>
       <c r="B180" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="C180" t="s">
         <v>5</v>
       </c>
       <c r="D180" t="s">
-        <v>256</v>
+        <v>164</v>
       </c>
     </row>
     <row r="181">
@@ -3436,13 +3421,13 @@
         <v>180.0</v>
       </c>
       <c r="B181" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C181" t="s">
         <v>5</v>
       </c>
       <c r="D181" t="s">
-        <v>221</v>
+        <v>253</v>
       </c>
     </row>
     <row r="182">
@@ -3450,13 +3435,13 @@
         <v>181.0</v>
       </c>
       <c r="B182" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="C182" t="s">
         <v>5</v>
       </c>
       <c r="D182" t="s">
-        <v>174</v>
+        <v>78</v>
       </c>
     </row>
     <row r="183">
@@ -3464,13 +3449,13 @@
         <v>182.0</v>
       </c>
       <c r="B183" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="C183" t="s">
         <v>5</v>
       </c>
       <c r="D183" t="s">
-        <v>131</v>
+        <v>36</v>
       </c>
     </row>
     <row r="184">
@@ -3478,13 +3463,13 @@
         <v>183.0</v>
       </c>
       <c r="B184" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C184" t="s">
         <v>5</v>
       </c>
       <c r="D184" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
     </row>
     <row r="185">
@@ -3492,13 +3477,13 @@
         <v>184.0</v>
       </c>
       <c r="B185" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C185" t="s">
         <v>5</v>
       </c>
       <c r="D185" t="s">
-        <v>86</v>
+        <v>259</v>
       </c>
     </row>
     <row r="186">
@@ -3506,13 +3491,13 @@
         <v>185.0</v>
       </c>
       <c r="B186" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C186" t="s">
         <v>5</v>
       </c>
       <c r="D186" t="s">
-        <v>197</v>
+        <v>94</v>
       </c>
     </row>
     <row r="187">
@@ -3520,13 +3505,13 @@
         <v>186.0</v>
       </c>
       <c r="B187" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C187" t="s">
         <v>5</v>
       </c>
       <c r="D187" t="s">
-        <v>265</v>
+        <v>50</v>
       </c>
     </row>
     <row r="188">
@@ -3534,13 +3519,13 @@
         <v>187.0</v>
       </c>
       <c r="B188" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C188" t="s">
         <v>5</v>
       </c>
       <c r="D188" t="s">
-        <v>26</v>
+        <v>263</v>
       </c>
     </row>
     <row r="189">
@@ -3548,13 +3533,13 @@
         <v>188.0</v>
       </c>
       <c r="B189" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C189" t="s">
         <v>5</v>
       </c>
       <c r="D189" t="s">
-        <v>86</v>
+        <v>24</v>
       </c>
     </row>
     <row r="190">
@@ -3562,13 +3547,13 @@
         <v>189.0</v>
       </c>
       <c r="B190" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C190" t="s">
         <v>5</v>
       </c>
       <c r="D190" t="s">
-        <v>58</v>
+        <v>219</v>
       </c>
     </row>
     <row r="191">
@@ -3576,13 +3561,13 @@
         <v>190.0</v>
       </c>
       <c r="B191" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C191" t="s">
         <v>5</v>
       </c>
       <c r="D191" t="s">
-        <v>270</v>
+        <v>164</v>
       </c>
     </row>
     <row r="192">
@@ -3590,13 +3575,13 @@
         <v>191.0</v>
       </c>
       <c r="B192" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C192" t="s">
         <v>5</v>
       </c>
       <c r="D192" t="s">
-        <v>109</v>
+        <v>42</v>
       </c>
     </row>
     <row r="193">
@@ -3604,13 +3589,13 @@
         <v>192.0</v>
       </c>
       <c r="B193" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C193" t="s">
         <v>5</v>
       </c>
       <c r="D193" t="s">
-        <v>273</v>
+        <v>42</v>
       </c>
     </row>
     <row r="194">
@@ -3618,13 +3603,13 @@
         <v>193.0</v>
       </c>
       <c r="B194" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C194" t="s">
         <v>5</v>
       </c>
       <c r="D194" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
     </row>
     <row r="195">
@@ -3632,13 +3617,13 @@
         <v>194.0</v>
       </c>
       <c r="B195" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C195" t="s">
         <v>5</v>
       </c>
       <c r="D195" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
     </row>
     <row r="196">
@@ -3646,13 +3631,13 @@
         <v>195.0</v>
       </c>
       <c r="B196" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C196" t="s">
         <v>5</v>
       </c>
       <c r="D196" t="s">
-        <v>93</v>
+        <v>36</v>
       </c>
     </row>
     <row r="197">
@@ -3660,13 +3645,13 @@
         <v>196.0</v>
       </c>
       <c r="B197" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="C197" t="s">
         <v>5</v>
       </c>
       <c r="D197" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="198">
@@ -3674,13 +3659,13 @@
         <v>197.0</v>
       </c>
       <c r="B198" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="C198" t="s">
         <v>5</v>
       </c>
       <c r="D198" t="s">
-        <v>84</v>
+        <v>6</v>
       </c>
     </row>
     <row r="199">
@@ -3688,13 +3673,13 @@
         <v>198.0</v>
       </c>
       <c r="B199" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="C199" t="s">
         <v>5</v>
       </c>
       <c r="D199" t="s">
-        <v>55</v>
+        <v>109</v>
       </c>
     </row>
     <row r="200">
@@ -3702,13 +3687,13 @@
         <v>199.0</v>
       </c>
       <c r="B200" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="C200" t="s">
         <v>5</v>
       </c>
       <c r="D200" t="s">
-        <v>241</v>
+        <v>87</v>
       </c>
     </row>
     <row r="201">
@@ -3716,13 +3701,13 @@
         <v>200.0</v>
       </c>
       <c r="B201" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="C201" t="s">
         <v>5</v>
       </c>
       <c r="D201" t="s">
-        <v>113</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dollar 1000 100 bug fix
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="124">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,10 +83,115 @@
     <t>09030201</t>
   </si>
   <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of travelers by different means.</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?&lt;br&gt;#उच्च 3 मूल्यांसाठी प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 1$&lt;br&gt;No. of travellers using the Bus  $= 5$&lt;br&gt;No. of travellers using the Scooter  $= 7$&lt;br&gt;No. of travellers using the Car  $= 8$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$1 + 5 + 7 + 8 = 21$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$1 + 5 + 7 + 8 = 21$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Bus, Scooter, Car&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bus$, $Scooter$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bus, Scooter, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bus$, $Scooter$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Bus, Scooter, Car</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
     <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
   </si>
   <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
+    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
@@ -98,397 +203,184 @@
     <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
   </si>
   <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: 810 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 930$&lt;br&gt;No. of travellers using the vehicle least $= 120$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$930 - 120 = 810$  is the answer.&lt;br&gt;#उत्तर : 810&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 930$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 120$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$930 - 120 = 810$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>Ans: Scooter, Bus, Car, Truck&lt;br&gt;From the given graph we can see that, $Scooter$, $Bus$, $Car$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Bus, Car, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Bus$, $Car$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter, Bus, Car, Truck</t>
+  </si>
+  <si>
+    <t>Ans: Car, Motorcycle, Truck, Bicycle&lt;br&gt;From the given graph we can see that, $Car$, $Motorcycle$, $Truck$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Motorcycle, Truck, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Motorcycle$, $Truck$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Motorcycle, Truck, Bicycle</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>Ans: 2 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 8$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$8 - 6 = 2$  is the answer.&lt;br&gt;#उत्तर : 2&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$8 - 6 = 2$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
   </si>
   <si>
-    <t>810</t>
-  </si>
-  <si>
-    <t>809</t>
-  </si>
-  <si>
-    <t>812</t>
-  </si>
-  <si>
-    <t>808</t>
-  </si>
-  <si>
-    <t>811</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?&lt;br&gt;#उच्च 3 मूल्यांसाठी प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>590</t>
-  </si>
-  <si>
-    <t>589</t>
-  </si>
-  <si>
-    <t>591</t>
-  </si>
-  <si>
-    <t>588</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of travelers by different means.</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
+    <t>2</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>11300</t>
+  </si>
+  <si>
+    <t>11301</t>
+  </si>
+  <si>
+    <t>11298</t>
+  </si>
+  <si>
+    <t>11302</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>2370</t>
+  </si>
+  <si>
+    <t>2369</t>
+  </si>
+  <si>
+    <t>2371</t>
+  </si>
+  <si>
+    <t>2372</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 110$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 240$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$110 + 240 = 350$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 110$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$110 + 240 = 350$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>350</t>
-  </si>
-  <si>
-    <t>351</t>
-  </si>
-  <si>
-    <t>352</t>
-  </si>
-  <si>
-    <t>348</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 80$&lt;br&gt;No. of travellers using the Scooter  $= 110$&lt;br&gt;No. of travellers using the Bus  $= 240$&lt;br&gt;No. of travellers using the Bicycle  $= 240$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$80 + 110 + 240 + 240 = 670$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 80$&lt;br&gt;Scooter या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 110$&lt;br&gt;Bus या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$80 + 110 + 240 + 240 = 670$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>670</t>
-  </si>
-  <si>
-    <t>669</t>
-  </si>
-  <si>
-    <t>672</t>
-  </si>
-  <si>
-    <t>668</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 30$&lt;br&gt;No. of travellers using the Bicycle  $= 880$&lt;br&gt;No. of travellers using the Scooter  $= 590$&lt;br&gt;No. of travellers using the Motorcycle  $= 60$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$30 + 880 + 590 + 60 = 1560$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 30$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 880$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 590$&lt;br&gt;Motorcycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 60$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$30 + 880 + 590 + 60 = 1560$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>1560</t>
-  </si>
-  <si>
-    <t>1558</t>
-  </si>
-  <si>
-    <t>1561</t>
-  </si>
-  <si>
-    <t>1559</t>
-  </si>
-  <si>
-    <t>1562</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 2600$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 5800$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$2600 + 5800 = 8400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2600$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5800$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$2600 + 5800 = 8400$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>8400</t>
-  </si>
-  <si>
-    <t>8398</t>
-  </si>
-  <si>
-    <t>8401</t>
-  </si>
-  <si>
-    <t>8399</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>8402</t>
-  </si>
-  <si>
     <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
   </si>
   <si>
-    <t>10200</t>
-  </si>
-  <si>
-    <t>10201</t>
-  </si>
-  <si>
-    <t>10198</t>
-  </si>
-  <si>
-    <t>10202</t>
-  </si>
-  <si>
-    <t>18200</t>
-  </si>
-  <si>
-    <t>18198</t>
-  </si>
-  <si>
-    <t>18201</t>
-  </si>
-  <si>
-    <t>18199</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 10000$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>22800</t>
-  </si>
-  <si>
-    <t>22798</t>
-  </si>
-  <si>
-    <t>22802</t>
-  </si>
-  <si>
-    <t>22801</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 2$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 4$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$2 + 4 = 6$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$2 + 4 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>8</t>
+    <t>9</t>
   </si>
   <si>
     <t>7</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>Ans: 8 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 8$&lt;br&gt;No. of travellers using the vehicle least $= 0$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$8 - 0 = 8$  is the answer.&lt;br&gt;#उत्तर : 8&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 0$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$8 - 0 = 8$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Car, Bicycle, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Car$, $Bicycle$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Bicycle, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Bicycle$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bicycle, Bus, Scooter</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: 720 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 750$&lt;br&gt;No. of travellers using the vehicle least $= 30$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$750 - 30 = 720$  is the answer.&lt;br&gt;#उत्तर : 720&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 750$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 30$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$750 - 30 = 720$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>720</t>
-  </si>
-  <si>
-    <t>721</t>
-  </si>
-  <si>
-    <t>722</t>
-  </si>
-  <si>
-    <t>719</t>
+    <t>11</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: 510 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 650$&lt;br&gt;No. of travellers using the vehicle least $= 140$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$650 - 140 = 510$  is the answer.&lt;br&gt;#उत्तर : 510&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 650$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 140$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$650 - 140 = 510$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>510</t>
-  </si>
-  <si>
-    <t>508</t>
-  </si>
-  <si>
-    <t>509</t>
-  </si>
-  <si>
-    <t>512</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bus$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 720$&lt;br&gt;No. of travellers using the Bicycle  $= 170$&lt;br&gt;No. of travellers using the Car  $= 280$&lt;br&gt;No. of travellers using the Scooter  $= 780$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$720 + 170 + 280 + 780 = 1950$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 720$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 170$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 780$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$720 + 170 + 280 + 780 = 1950$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>1950</t>
-  </si>
-  <si>
-    <t>1948</t>
-  </si>
-  <si>
-    <t>1951</t>
-  </si>
-  <si>
-    <t>1952</t>
-  </si>
-  <si>
-    <t>Ans: 610 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 780$&lt;br&gt;No. of travellers using the vehicle least $= 170$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$780 - 170 = 610$  is the answer.&lt;br&gt;#उत्तर : 610&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 780$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 170$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$780 - 170 = 610$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>610</t>
-  </si>
-  <si>
-    <t>608</t>
-  </si>
-  <si>
-    <t>612</t>
-  </si>
-  <si>
-    <t>611</t>
-  </si>
-  <si>
-    <t>Ans: Scooter, Bus, Car, Bicycle&lt;br&gt;From the given graph we can see that, $Scooter$, $Bus$, $Car$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Bus, Car, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Bus$, $Car$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter, Bus, Car, Bicycle</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Scooter $= 9300$&lt;br&gt;No. of travellers using the Bus  $= 2000$&lt;br&gt;No. of travellers using the Truck  $= 6800$&lt;br&gt;No. of travellers using the Bicycle  $= 5500$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$9300 + 2000 + 6800 + 5500 = 23600$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Scooter या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2000$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6800$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 5500$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$9300 + 2000 + 6800 + 5500 = 23600$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>23600</t>
+  </si>
+  <si>
+    <t>23598</t>
+  </si>
+  <si>
+    <t>23602</t>
+  </si>
+  <si>
+    <t>23601</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 28$&lt;br&gt;No. of travellers using the Bus  $= 23$&lt;br&gt;No. of travellers using the Car  $= 82$&lt;br&gt;No. of travellers using the Bicycle  $= 12$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$28 + 23 + 82 + 12 = 145$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 28$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 23$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 82$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 12$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$28 + 23 + 82 + 12 = 145$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>145</t>
+  </si>
+  <si>
+    <t>146</t>
+  </si>
+  <si>
+    <t>144</t>
+  </si>
+  <si>
+    <t>147</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
   </si>
   <si>
-    <t>18300</t>
-  </si>
-  <si>
-    <t>18302</t>
-  </si>
-  <si>
-    <t>18298</t>
-  </si>
-  <si>
-    <t>18299</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>****</t>
@@ -928,7 +820,7 @@
     <col min="2" max="2" width="13.9140625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="12.4375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.66015625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="193.7734375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="186.99609375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="63.5" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="16.42578125" customWidth="true" bestFit="true"/>
@@ -1021,43 +913,43 @@
         <v>22</v>
       </c>
       <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" t="s">
         <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" t="s">
-        <v>20</v>
       </c>
       <c r="T2" t="n">
         <v>110.0</v>
@@ -1080,10 +972,10 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
         <v>20</v>
@@ -1095,25 +987,25 @@
         <v>20</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N3" t="n">
         <v>4.0</v>
       </c>
       <c r="Q3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R3" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="T3" t="n">
         <v>110.0</v>
@@ -1136,10 +1028,10 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1151,25 +1043,25 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K4" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N4" t="n">
         <v>4.0</v>
       </c>
       <c r="Q4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1192,10 +1084,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1207,25 +1099,25 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="K5" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="L5" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N5" t="n">
         <v>4.0</v>
       </c>
       <c r="Q5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1248,40 +1140,40 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6" t="s">
         <v>39</v>
-      </c>
-      <c r="F6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" t="s">
-        <v>43</v>
-      </c>
-      <c r="K6" t="s">
-        <v>44</v>
-      </c>
-      <c r="L6" t="s">
-        <v>41</v>
-      </c>
-      <c r="M6" t="s">
-        <v>28</v>
-      </c>
-      <c r="N6" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>30</v>
-      </c>
-      <c r="R6" t="s">
-        <v>38</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1304,40 +1196,40 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" t="s">
         <v>45</v>
       </c>
-      <c r="F7" t="s">
+      <c r="K7" t="s">
         <v>46</v>
       </c>
-      <c r="G7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="L7" t="s">
         <v>47</v>
       </c>
-      <c r="K7" t="s">
+      <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P7" t="s">
         <v>48</v>
       </c>
-      <c r="L7" t="s">
-        <v>49</v>
-      </c>
-      <c r="M7" t="s">
-        <v>28</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P7" t="s">
-        <v>50</v>
-      </c>
       <c r="Q7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R7" t="s">
         <v>20</v>
@@ -1363,10 +1255,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1378,25 +1270,25 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K8" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="L8" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="M8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N8" t="n">
         <v>4.0</v>
       </c>
       <c r="Q8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1419,10 +1311,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1434,25 +1326,25 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="K9" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="L9" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="M9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N9" t="n">
         <v>4.0</v>
       </c>
       <c r="Q9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1475,40 +1367,40 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
+        <v>58</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" t="s">
         <v>60</v>
       </c>
-      <c r="F10" t="s">
+      <c r="K10" t="s">
         <v>61</v>
       </c>
-      <c r="G10" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="L10" t="s">
         <v>62</v>
       </c>
-      <c r="K10" t="s">
-        <v>63</v>
-      </c>
-      <c r="L10" t="s">
-        <v>64</v>
-      </c>
       <c r="M10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N10" t="n">
         <v>4.0</v>
       </c>
       <c r="Q10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R10" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="T10" t="n">
         <v>110.0</v>
@@ -1531,10 +1423,10 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>66</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="G11" t="s">
         <v>20</v>
@@ -1546,25 +1438,25 @@
         <v>20</v>
       </c>
       <c r="J11" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="K11" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="L11" t="s">
-        <v>70</v>
+        <v>38</v>
       </c>
       <c r="M11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N11" t="n">
         <v>4.0</v>
       </c>
       <c r="Q11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R11" t="s">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1587,10 +1479,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1602,28 +1494,28 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="K12" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="L12" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="M12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N12" t="n">
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="Q12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R12" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1646,11 +1538,11 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" t="s">
         <v>66</v>
       </c>
-      <c r="F13" t="s">
-        <v>73</v>
-      </c>
       <c r="G13" t="s">
         <v>20</v>
       </c>
@@ -1661,25 +1553,25 @@
         <v>20</v>
       </c>
       <c r="J13" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="K13" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="L13" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="M13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N13" t="n">
         <v>4.0</v>
       </c>
       <c r="Q13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1702,10 +1594,10 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="F14" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="G14" t="s">
         <v>20</v>
@@ -1717,25 +1609,25 @@
         <v>20</v>
       </c>
       <c r="J14" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="K14" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="L14" t="s">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="M14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N14" t="n">
         <v>4.0</v>
       </c>
       <c r="Q14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R14" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1758,10 +1650,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="F15" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1773,25 +1665,25 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="K15" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="L15" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="M15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N15" t="n">
         <v>4.0</v>
       </c>
       <c r="Q15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1814,10 +1706,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="F16" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1829,25 +1721,25 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="K16" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="L16" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="M16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N16" t="n">
         <v>4.0</v>
       </c>
       <c r="Q16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R16" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="T16" t="n">
         <v>110.0</v>
@@ -1870,10 +1762,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1885,28 +1777,28 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="K17" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="L17" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="M17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N17" t="n">
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="Q17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1929,10 +1821,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="F18" t="s">
-        <v>86</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1944,25 +1836,25 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>87</v>
+        <v>26</v>
       </c>
       <c r="K18" t="s">
-        <v>88</v>
+        <v>27</v>
       </c>
       <c r="L18" t="s">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="M18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N18" t="n">
         <v>4.0</v>
       </c>
       <c r="Q18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -1985,40 +1877,40 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
+        <v>58</v>
+      </c>
+      <c r="F19" t="s">
+        <v>59</v>
+      </c>
+      <c r="G19" t="s">
+        <v>20</v>
+      </c>
+      <c r="H19" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" t="s">
         <v>60</v>
       </c>
-      <c r="F19" t="s">
-        <v>80</v>
-      </c>
-      <c r="G19" t="s">
-        <v>20</v>
-      </c>
-      <c r="H19" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" t="s">
-        <v>20</v>
-      </c>
-      <c r="J19" t="s">
-        <v>81</v>
-      </c>
       <c r="K19" t="s">
-        <v>82</v>
+        <v>61</v>
       </c>
       <c r="L19" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
       <c r="M19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N19" t="n">
         <v>4.0</v>
       </c>
       <c r="Q19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2041,10 +1933,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2056,22 +1948,22 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="K20" t="s">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="L20" t="s">
-        <v>95</v>
+        <v>62</v>
       </c>
       <c r="M20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N20" t="n">
         <v>4.0</v>
       </c>
       <c r="Q20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R20" t="s">
         <v>20</v>
@@ -2097,10 +1989,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2112,25 +2004,25 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="K21" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="L21" t="s">
-        <v>99</v>
+        <v>67</v>
       </c>
       <c r="M21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N21" t="n">
         <v>4.0</v>
       </c>
       <c r="Q21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>20</v>
+        <v>79</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2153,10 +2045,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="F22" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2168,28 +2060,28 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="K22" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="L22" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="M22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N22" t="n">
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="Q22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2212,10 +2104,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="F23" t="s">
-        <v>101</v>
+        <v>28</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2227,25 +2119,25 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K23" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="L23" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="M23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N23" t="n">
         <v>4.0</v>
       </c>
       <c r="Q23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2268,10 +2160,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F24" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2283,25 +2175,25 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K24" t="s">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="L24" t="s">
-        <v>104</v>
+        <v>25</v>
       </c>
       <c r="M24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N24" t="n">
         <v>4.0</v>
       </c>
       <c r="Q24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2324,10 +2216,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F25" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2339,22 +2231,22 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="K25" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="L25" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="M25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N25" t="n">
         <v>4.0</v>
       </c>
       <c r="Q25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R25" t="s">
         <v>20</v>
@@ -2380,10 +2272,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="F26" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2395,25 +2287,25 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="K26" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="L26" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="M26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N26" t="n">
         <v>4.0</v>
       </c>
       <c r="Q26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>51</v>
+        <v>92</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2436,10 +2328,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>25</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2451,28 +2343,28 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="K27" t="s">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="L27" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
       <c r="M27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N27" t="n">
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="Q27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>109</v>
+        <v>23</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2495,10 +2387,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F28" t="s">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2510,25 +2402,25 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="K28" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="L28" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="M28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N28" t="n">
         <v>4.0</v>
       </c>
       <c r="Q28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R28" t="s">
-        <v>113</v>
+        <v>20</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2551,10 +2443,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="F29" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2566,25 +2458,25 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="K29" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="L29" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="M29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N29" t="n">
         <v>4.0</v>
       </c>
       <c r="Q29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2607,10 +2499,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="F30" t="s">
-        <v>116</v>
+        <v>27</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2622,25 +2514,25 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K30" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="L30" t="s">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="M30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N30" t="n">
         <v>4.0</v>
       </c>
       <c r="Q30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2663,10 +2555,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>91</v>
+        <v>58</v>
       </c>
       <c r="F31" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2678,22 +2570,22 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>111</v>
+        <v>60</v>
       </c>
       <c r="K31" t="s">
-        <v>114</v>
+        <v>61</v>
       </c>
       <c r="L31" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="M31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N31" t="n">
         <v>4.0</v>
       </c>
       <c r="Q31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R31" t="s">
         <v>20</v>
@@ -2719,10 +2611,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>118</v>
+        <v>32</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2734,28 +2626,28 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>120</v>
+        <v>26</v>
       </c>
       <c r="K32" t="s">
-        <v>121</v>
+        <v>41</v>
       </c>
       <c r="L32" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
       <c r="M32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N32" t="n">
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="Q32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>117</v>
+        <v>86</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2778,10 +2670,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="F33" t="s">
-        <v>24</v>
+        <v>66</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2793,22 +2685,22 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="K33" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="L33" t="s">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="M33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N33" t="n">
         <v>4.0</v>
       </c>
       <c r="Q33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R33" t="s">
         <v>20</v>
@@ -2834,10 +2726,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="F34" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2849,25 +2741,25 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="K34" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="L34" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="M34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N34" t="n">
         <v>4.0</v>
       </c>
       <c r="Q34" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R34" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2890,10 +2782,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="F35" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2905,25 +2797,25 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K35" t="s">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="L35" t="s">
-        <v>104</v>
+        <v>28</v>
       </c>
       <c r="M35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N35" t="n">
         <v>4.0</v>
       </c>
       <c r="Q35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2946,10 +2838,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="F36" t="s">
-        <v>126</v>
+        <v>25</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -2961,25 +2853,25 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>127</v>
+        <v>26</v>
       </c>
       <c r="K36" t="s">
-        <v>128</v>
+        <v>27</v>
       </c>
       <c r="L36" t="s">
-        <v>129</v>
+        <v>28</v>
       </c>
       <c r="M36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N36" t="n">
         <v>4.0</v>
       </c>
       <c r="Q36" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -3002,10 +2894,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>52</v>
+        <v>101</v>
       </c>
       <c r="F37" t="s">
-        <v>53</v>
+        <v>102</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3017,28 +2909,28 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>54</v>
+        <v>103</v>
       </c>
       <c r="K37" t="s">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="L37" t="s">
-        <v>56</v>
+        <v>105</v>
       </c>
       <c r="M37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N37" t="n">
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="Q37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R37" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3061,10 +2953,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="F38" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3076,25 +2968,25 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="K38" t="s">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="L38" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="M38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N38" t="n">
         <v>4.0</v>
       </c>
       <c r="Q38" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R38" t="s">
-        <v>131</v>
+        <v>20</v>
       </c>
       <c r="T38" t="n">
         <v>110.0</v>
@@ -3117,10 +3009,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="F39" t="s">
-        <v>133</v>
+        <v>87</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3132,25 +3024,25 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>134</v>
+        <v>26</v>
       </c>
       <c r="K39" t="s">
-        <v>135</v>
+        <v>41</v>
       </c>
       <c r="L39" t="s">
-        <v>136</v>
+        <v>25</v>
       </c>
       <c r="M39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N39" t="n">
         <v>4.0</v>
       </c>
       <c r="Q39" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3173,10 +3065,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F40" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3188,25 +3080,25 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="K40" t="s">
-        <v>104</v>
+        <v>42</v>
       </c>
       <c r="L40" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="M40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N40" t="n">
         <v>4.0</v>
       </c>
       <c r="Q40" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>137</v>
+        <v>63</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3229,10 +3121,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F41" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3244,25 +3136,25 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>103</v>
+        <v>44</v>
       </c>
       <c r="K41" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="L41" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="M41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N41" t="n">
         <v>4.0</v>
       </c>
       <c r="Q41" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R41" t="s">
-        <v>137</v>
+        <v>20</v>
       </c>
       <c r="T41" t="n">
         <v>110.0</v>
@@ -3285,10 +3177,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="F42" t="s">
-        <v>139</v>
+        <v>41</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3300,28 +3192,28 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K42" t="s">
-        <v>103</v>
+        <v>27</v>
       </c>
       <c r="L42" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N42" t="n">
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="Q42" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R42" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3344,10 +3236,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="F43" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3359,25 +3251,25 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>34</v>
+        <v>90</v>
       </c>
       <c r="K43" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="L43" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="M43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N43" t="n">
         <v>4.0</v>
       </c>
       <c r="Q43" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R43" t="s">
-        <v>131</v>
+        <v>20</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3400,10 +3292,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="F44" t="s">
-        <v>142</v>
+        <v>87</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3415,25 +3307,25 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>143</v>
+        <v>26</v>
       </c>
       <c r="K44" t="s">
-        <v>144</v>
+        <v>41</v>
       </c>
       <c r="L44" t="s">
-        <v>145</v>
+        <v>25</v>
       </c>
       <c r="M44" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N44" t="n">
         <v>4.0</v>
       </c>
       <c r="Q44" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>141</v>
+        <v>86</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3456,10 +3348,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="F45" t="s">
-        <v>147</v>
+        <v>41</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3471,25 +3363,25 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>148</v>
+        <v>26</v>
       </c>
       <c r="K45" t="s">
-        <v>149</v>
+        <v>27</v>
       </c>
       <c r="L45" t="s">
-        <v>150</v>
+        <v>28</v>
       </c>
       <c r="M45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N45" t="n">
         <v>4.0</v>
       </c>
       <c r="Q45" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R45" t="s">
-        <v>146</v>
+        <v>109</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3512,10 +3404,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="F46" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3527,25 +3419,25 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>34</v>
+        <v>113</v>
       </c>
       <c r="K46" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="L46" t="s">
-        <v>33</v>
+        <v>115</v>
       </c>
       <c r="M46" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N46" t="n">
         <v>4.0</v>
       </c>
       <c r="Q46" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3568,43 +3460,43 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
+        <v>50</v>
+      </c>
+      <c r="F47" t="s">
+        <v>117</v>
+      </c>
+      <c r="G47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" t="s">
+        <v>20</v>
+      </c>
+      <c r="I47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J47" t="s">
         <v>118</v>
       </c>
-      <c r="F47" t="s">
-        <v>152</v>
-      </c>
-      <c r="G47" t="s">
-        <v>20</v>
-      </c>
-      <c r="H47" t="s">
-        <v>20</v>
-      </c>
-      <c r="I47" t="s">
-        <v>20</v>
-      </c>
-      <c r="J47" t="s">
+      <c r="K47" t="s">
+        <v>119</v>
+      </c>
+      <c r="L47" t="s">
         <v>120</v>
       </c>
-      <c r="K47" t="s">
+      <c r="M47" t="s">
+        <v>29</v>
+      </c>
+      <c r="N47" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P47" t="s">
         <v>121</v>
       </c>
-      <c r="L47" t="s">
-        <v>122</v>
-      </c>
-      <c r="M47" t="s">
-        <v>28</v>
-      </c>
-      <c r="N47" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P47" t="s">
-        <v>153</v>
-      </c>
       <c r="Q47" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>151</v>
+        <v>116</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3627,10 +3519,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="F48" t="s">
-        <v>139</v>
+        <v>66</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3642,25 +3534,25 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="K48" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="L48" t="s">
-        <v>33</v>
+        <v>69</v>
       </c>
       <c r="M48" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N48" t="n">
         <v>4.0</v>
       </c>
       <c r="Q48" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>138</v>
+        <v>20</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3683,10 +3575,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="F49" t="s">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3698,22 +3590,22 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>155</v>
+        <v>60</v>
       </c>
       <c r="K49" t="s">
-        <v>156</v>
+        <v>61</v>
       </c>
       <c r="L49" t="s">
-        <v>157</v>
+        <v>62</v>
       </c>
       <c r="M49" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N49" t="n">
         <v>4.0</v>
       </c>
       <c r="Q49" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R49" t="s">
         <v>20</v>
@@ -3739,10 +3631,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>78</v>
+        <v>34</v>
       </c>
       <c r="F50" t="s">
-        <v>139</v>
+        <v>35</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3754,25 +3646,25 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="K50" t="s">
-        <v>103</v>
+        <v>37</v>
       </c>
       <c r="L50" t="s">
+        <v>38</v>
+      </c>
+      <c r="M50" t="s">
+        <v>29</v>
+      </c>
+      <c r="N50" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>31</v>
+      </c>
+      <c r="R50" t="s">
         <v>33</v>
-      </c>
-      <c r="M50" t="s">
-        <v>28</v>
-      </c>
-      <c r="N50" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q50" t="s">
-        <v>30</v>
-      </c>
-      <c r="R50" t="s">
-        <v>158</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3795,10 +3687,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F51" t="s">
-        <v>53</v>
+        <v>122</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3810,25 +3702,25 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="K51" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="L51" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="M51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N51" t="n">
         <v>4.0</v>
       </c>
       <c r="Q51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3839,7 +3731,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bugs fixed bhot saare :)
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="158">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,304 +83,406 @@
     <t>09030201</t>
   </si>
   <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of travelers by different means.</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Truck, Motorcycle, Car</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>174</t>
+  </si>
+  <si>
+    <t>172</t>
+  </si>
+  <si>
+    <t>176</t>
+  </si>
+  <si>
+    <t>173</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>Car, Motorcycle, Bus, Truck</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Truck, Motorcycle, Bus, Scooter</t>
+  </si>
+  <si>
+    <t>Ans: $79$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 80$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$80 - 1 = 79$  is the answer.&lt;br&gt;#उत्तर : $79$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 80$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$80 - 1 = 79$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>79</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>166</t>
+  </si>
+  <si>
+    <t>168</t>
+  </si>
+  <si>
+    <t>167</t>
+  </si>
+  <si>
+    <t>164</t>
+  </si>
+  <si>
+    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>87</t>
+  </si>
+  <si>
+    <t>84</t>
+  </si>
+  <si>
+    <t>83</t>
+  </si>
+  <si>
+    <t>1660</t>
+  </si>
+  <si>
+    <t>1658</t>
+  </si>
+  <si>
+    <t>1662</t>
+  </si>
+  <si>
+    <t>1659</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>860</t>
+  </si>
+  <si>
+    <t>859</t>
+  </si>
+  <si>
+    <t>858</t>
+  </si>
+  <si>
+    <t>862</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>91</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>Truck, Motorcycle, Car, Bus</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of travelers by different means.</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?&lt;br&gt;#उच्च 3 मूल्यांसाठी प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>20</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>590</t>
+  </si>
+  <si>
+    <t>591</t>
+  </si>
+  <si>
+    <t>588</t>
+  </si>
+  <si>
+    <t>592</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>460</t>
+  </si>
+  <si>
+    <t>458</t>
+  </si>
+  <si>
+    <t>459</t>
+  </si>
+  <si>
+    <t>461</t>
+  </si>
+  <si>
+    <t>1090</t>
+  </si>
+  <si>
+    <t>1089</t>
+  </si>
+  <si>
+    <t>1088</t>
+  </si>
+  <si>
+    <t>1091</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t>90</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>24</t>
   </si>
   <si>
     <t>22</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 1$&lt;br&gt;No. of travellers using the Bus  $= 5$&lt;br&gt;No. of travellers using the Scooter  $= 7$&lt;br&gt;No. of travellers using the Car  $= 8$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$1 + 5 + 7 + 8 = 21$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$1 + 5 + 7 + 8 = 21$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>Ans: Motorcycle, Bus, Scooter, Car&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bus$, $Scooter$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bus, Scooter, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bus$, $Scooter$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle, Bus, Scooter, Car</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>Ans: Scooter, Bus, Car, Truck&lt;br&gt;From the given graph we can see that, $Scooter$, $Bus$, $Car$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Bus, Car, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Bus$, $Car$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter, Bus, Car, Truck</t>
-  </si>
-  <si>
-    <t>Ans: Car, Motorcycle, Truck, Bicycle&lt;br&gt;From the given graph we can see that, $Car$, $Motorcycle$, $Truck$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Motorcycle, Truck, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Motorcycle$, $Truck$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Motorcycle, Truck, Bicycle</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>Ans: 2 &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 8$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$8 - 6 = 2$  is the answer.&lt;br&gt;#उत्तर : 2&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$8 - 6 = 2$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>11300</t>
-  </si>
-  <si>
-    <t>11301</t>
-  </si>
-  <si>
-    <t>11298</t>
-  </si>
-  <si>
-    <t>11302</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>2370</t>
-  </si>
-  <si>
-    <t>2369</t>
-  </si>
-  <si>
-    <t>2371</t>
-  </si>
-  <si>
-    <t>2372</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bus$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Scooter $= 9300$&lt;br&gt;No. of travellers using the Bus  $= 2000$&lt;br&gt;No. of travellers using the Truck  $= 6800$&lt;br&gt;No. of travellers using the Bicycle  $= 5500$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$9300 + 2000 + 6800 + 5500 = 23600$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Scooter या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2000$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6800$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 5500$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$9300 + 2000 + 6800 + 5500 = 23600$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>23600</t>
-  </si>
-  <si>
-    <t>23598</t>
-  </si>
-  <si>
-    <t>23602</t>
-  </si>
-  <si>
-    <t>23601</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 28$&lt;br&gt;No. of travellers using the Bus  $= 23$&lt;br&gt;No. of travellers using the Car  $= 82$&lt;br&gt;No. of travellers using the Bicycle  $= 12$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$28 + 23 + 82 + 12 = 145$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 28$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 23$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 82$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 12$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$28 + 23 + 82 + 12 = 145$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>145</t>
-  </si>
-  <si>
-    <t>146</t>
-  </si>
-  <si>
-    <t>144</t>
-  </si>
-  <si>
-    <t>147</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
   </si>
   <si>
+    <t>Car, Motorcycle, Scooter, Bus</t>
+  </si>
+  <si>
     <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>127</t>
+  </si>
+  <si>
+    <t>129</t>
+  </si>
+  <si>
+    <t>125</t>
+  </si>
+  <si>
+    <t>126</t>
   </si>
   <si>
     <t>****</t>
@@ -820,7 +922,7 @@
     <col min="2" max="2" width="13.9140625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="12.4375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.66015625" customWidth="true" bestFit="true"/>
-    <col min="5" max="5" width="186.99609375" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="193.7734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="63.5" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="16.42578125" customWidth="true" bestFit="true"/>
@@ -972,10 +1074,10 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G3" t="s">
         <v>20</v>
@@ -987,13 +1089,13 @@
         <v>20</v>
       </c>
       <c r="J3" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="L3" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
         <v>29</v>
@@ -1028,10 +1130,10 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1043,13 +1145,13 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="K4" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="L4" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="M4" t="s">
         <v>29</v>
@@ -1084,10 +1186,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1099,13 +1201,13 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="K5" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="L5" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="M5" t="s">
         <v>29</v>
@@ -1117,7 +1219,7 @@
         <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1140,10 +1242,10 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1155,13 +1257,13 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="K6" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="L6" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="M6" t="s">
         <v>29</v>
@@ -1173,7 +1275,7 @@
         <v>31</v>
       </c>
       <c r="R6" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1196,10 +1298,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1211,13 +1313,13 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="K7" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="L7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="M7" t="s">
         <v>29</v>
@@ -1226,7 +1328,7 @@
         <v>4.0</v>
       </c>
       <c r="P7" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="Q7" t="s">
         <v>31</v>
@@ -1255,10 +1357,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1270,13 +1372,13 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="K8" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="L8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="M8" t="s">
         <v>29</v>
@@ -1288,7 +1390,7 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1311,10 +1413,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1326,13 +1428,13 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="K9" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="L9" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="M9" t="s">
         <v>29</v>
@@ -1344,7 +1446,7 @@
         <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1367,28 +1469,28 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F10" t="s">
         <v>58</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" t="s">
         <v>59</v>
       </c>
-      <c r="G10" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>60</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>61</v>
-      </c>
-      <c r="L10" t="s">
-        <v>62</v>
       </c>
       <c r="M10" t="s">
         <v>29</v>
@@ -1423,29 +1525,29 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" t="s">
         <v>34</v>
       </c>
-      <c r="F11" t="s">
+      <c r="K11" t="s">
         <v>35</v>
       </c>
-      <c r="G11" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="L11" t="s">
         <v>36</v>
       </c>
-      <c r="K11" t="s">
-        <v>37</v>
-      </c>
-      <c r="L11" t="s">
-        <v>38</v>
-      </c>
       <c r="M11" t="s">
         <v>29</v>
       </c>
@@ -1456,7 +1558,7 @@
         <v>31</v>
       </c>
       <c r="R11" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1479,10 +1581,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F12" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1494,13 +1596,13 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="K12" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="L12" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="M12" t="s">
         <v>29</v>
@@ -1509,13 +1611,13 @@
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="Q12" t="s">
         <v>31</v>
       </c>
       <c r="R12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1538,10 +1640,10 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="F13" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="G13" t="s">
         <v>20</v>
@@ -1553,13 +1655,13 @@
         <v>20</v>
       </c>
       <c r="J13" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="K13" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="L13" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="M13" t="s">
         <v>29</v>
@@ -1571,7 +1673,7 @@
         <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1594,10 +1696,10 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="F14" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G14" t="s">
         <v>20</v>
@@ -1609,13 +1711,13 @@
         <v>20</v>
       </c>
       <c r="J14" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="K14" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="L14" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="M14" t="s">
         <v>29</v>
@@ -1627,7 +1729,7 @@
         <v>31</v>
       </c>
       <c r="R14" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1650,10 +1752,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1665,25 +1767,25 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="K15" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="L15" t="s">
+        <v>71</v>
+      </c>
+      <c r="M15" t="s">
+        <v>29</v>
+      </c>
+      <c r="N15" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>31</v>
+      </c>
+      <c r="R15" t="s">
         <v>62</v>
-      </c>
-      <c r="M15" t="s">
-        <v>29</v>
-      </c>
-      <c r="N15" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>31</v>
-      </c>
-      <c r="R15" t="s">
-        <v>20</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1706,10 +1808,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1721,13 +1823,13 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="K16" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="L16" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -1739,7 +1841,7 @@
         <v>31</v>
       </c>
       <c r="R16" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="T16" t="n">
         <v>110.0</v>
@@ -1762,28 +1864,28 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F17" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" t="s">
+        <v>20</v>
+      </c>
+      <c r="H17" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J17" t="s">
+        <v>75</v>
+      </c>
+      <c r="K17" t="s">
+        <v>76</v>
+      </c>
+      <c r="L17" t="s">
         <v>77</v>
-      </c>
-      <c r="G17" t="s">
-        <v>20</v>
-      </c>
-      <c r="H17" t="s">
-        <v>20</v>
-      </c>
-      <c r="I17" t="s">
-        <v>20</v>
-      </c>
-      <c r="J17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K17" t="s">
-        <v>56</v>
-      </c>
-      <c r="L17" t="s">
-        <v>57</v>
       </c>
       <c r="M17" t="s">
         <v>29</v>
@@ -1798,7 +1900,7 @@
         <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1821,10 +1923,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F18" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1836,13 +1938,13 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="K18" t="s">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="L18" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="M18" t="s">
         <v>29</v>
@@ -1854,7 +1956,7 @@
         <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -1877,10 +1979,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>28</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -1892,13 +1994,13 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="K19" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L19" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="M19" t="s">
         <v>29</v>
@@ -1910,7 +2012,7 @@
         <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -1933,10 +2035,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>58</v>
+        <v>83</v>
       </c>
       <c r="F20" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -1948,13 +2050,13 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="K20" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="L20" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="M20" t="s">
         <v>29</v>
@@ -1966,7 +2068,7 @@
         <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -1989,10 +2091,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="F21" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2004,13 +2106,13 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K21" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="L21" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="M21" t="s">
         <v>29</v>
@@ -2022,7 +2124,7 @@
         <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2045,10 +2147,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2060,13 +2162,13 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="K22" t="s">
-        <v>41</v>
+        <v>91</v>
       </c>
       <c r="L22" t="s">
-        <v>42</v>
+        <v>92</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -2075,13 +2177,13 @@
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="Q22" t="s">
         <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2104,29 +2206,29 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="F23" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" t="s">
+        <v>20</v>
+      </c>
+      <c r="H23" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" t="s">
+        <v>20</v>
+      </c>
+      <c r="J23" t="s">
+        <v>25</v>
+      </c>
+      <c r="K23" t="s">
+        <v>26</v>
+      </c>
+      <c r="L23" t="s">
         <v>28</v>
       </c>
-      <c r="G23" t="s">
-        <v>20</v>
-      </c>
-      <c r="H23" t="s">
-        <v>20</v>
-      </c>
-      <c r="I23" t="s">
-        <v>20</v>
-      </c>
-      <c r="J23" t="s">
-        <v>26</v>
-      </c>
-      <c r="K23" t="s">
-        <v>41</v>
-      </c>
-      <c r="L23" t="s">
-        <v>42</v>
-      </c>
       <c r="M23" t="s">
         <v>29</v>
       </c>
@@ -2137,7 +2239,7 @@
         <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2160,10 +2262,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="F24" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2175,13 +2277,13 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
+        <v>25</v>
+      </c>
+      <c r="K24" t="s">
         <v>26</v>
       </c>
-      <c r="K24" t="s">
-        <v>41</v>
-      </c>
       <c r="L24" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="M24" t="s">
         <v>29</v>
@@ -2193,7 +2295,7 @@
         <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>86</v>
+        <v>20</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2216,10 +2318,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
       <c r="F25" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2231,13 +2333,13 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="K25" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="L25" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="M25" t="s">
         <v>29</v>
@@ -2272,10 +2374,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="F26" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2287,13 +2389,13 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>26</v>
+        <v>101</v>
       </c>
       <c r="K26" t="s">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="L26" t="s">
-        <v>42</v>
+        <v>103</v>
       </c>
       <c r="M26" t="s">
         <v>29</v>
@@ -2305,7 +2407,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2328,10 +2430,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="F27" t="s">
-        <v>25</v>
+        <v>104</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2343,13 +2445,13 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="K27" t="s">
-        <v>27</v>
+        <v>106</v>
       </c>
       <c r="L27" t="s">
-        <v>28</v>
+        <v>107</v>
       </c>
       <c r="M27" t="s">
         <v>29</v>
@@ -2358,13 +2460,13 @@
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="Q27" t="s">
         <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2387,10 +2489,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="F28" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2402,13 +2504,13 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="K28" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="L28" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="M28" t="s">
         <v>29</v>
@@ -2443,10 +2545,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="F29" t="s">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2458,13 +2560,13 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="K29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="L29" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="M29" t="s">
         <v>29</v>
@@ -2499,10 +2601,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="F30" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2514,14 +2616,14 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="K30" t="s">
+        <v>40</v>
+      </c>
+      <c r="L30" t="s">
         <v>41</v>
       </c>
-      <c r="L30" t="s">
-        <v>42</v>
-      </c>
       <c r="M30" t="s">
         <v>29</v>
       </c>
@@ -2532,7 +2634,7 @@
         <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2555,10 +2657,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>58</v>
+        <v>114</v>
       </c>
       <c r="F31" t="s">
-        <v>98</v>
+        <v>26</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2570,13 +2672,13 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="K31" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="L31" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="M31" t="s">
         <v>29</v>
@@ -2611,10 +2713,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F32" t="s">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2626,13 +2728,13 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K32" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="L32" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
@@ -2641,13 +2743,13 @@
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="Q32" t="s">
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2670,10 +2772,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="F33" t="s">
-        <v>66</v>
+        <v>118</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2685,13 +2787,13 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>67</v>
+        <v>119</v>
       </c>
       <c r="K33" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="L33" t="s">
-        <v>81</v>
+        <v>121</v>
       </c>
       <c r="M33" t="s">
         <v>29</v>
@@ -2703,7 +2805,7 @@
         <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2726,10 +2828,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>34</v>
+        <v>122</v>
       </c>
       <c r="F34" t="s">
-        <v>35</v>
+        <v>123</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2741,13 +2843,13 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="K34" t="s">
-        <v>37</v>
+        <v>125</v>
       </c>
       <c r="L34" t="s">
-        <v>38</v>
+        <v>126</v>
       </c>
       <c r="M34" t="s">
         <v>29</v>
@@ -2759,7 +2861,7 @@
         <v>31</v>
       </c>
       <c r="R34" t="s">
-        <v>33</v>
+        <v>117</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2782,10 +2884,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="F35" t="s">
-        <v>25</v>
+        <v>127</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2797,13 +2899,13 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>26</v>
+        <v>128</v>
       </c>
       <c r="K35" t="s">
-        <v>27</v>
+        <v>129</v>
       </c>
       <c r="L35" t="s">
-        <v>28</v>
+        <v>130</v>
       </c>
       <c r="M35" t="s">
         <v>29</v>
@@ -2815,7 +2917,7 @@
         <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2838,10 +2940,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="F36" t="s">
-        <v>25</v>
+        <v>131</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -2853,13 +2955,13 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>26</v>
+        <v>132</v>
       </c>
       <c r="K36" t="s">
-        <v>27</v>
+        <v>133</v>
       </c>
       <c r="L36" t="s">
-        <v>28</v>
+        <v>134</v>
       </c>
       <c r="M36" t="s">
         <v>29</v>
@@ -2871,7 +2973,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -2894,10 +2996,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>101</v>
+        <v>65</v>
       </c>
       <c r="F37" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -2909,13 +3011,13 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="K37" t="s">
-        <v>104</v>
+        <v>136</v>
       </c>
       <c r="L37" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="M37" t="s">
         <v>29</v>
@@ -2924,7 +3026,7 @@
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="Q37" t="s">
         <v>31</v>
@@ -2953,10 +3055,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F38" t="s">
-        <v>59</v>
+        <v>138</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -2968,13 +3070,13 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>60</v>
+        <v>139</v>
       </c>
       <c r="K38" t="s">
-        <v>61</v>
+        <v>140</v>
       </c>
       <c r="L38" t="s">
-        <v>62</v>
+        <v>141</v>
       </c>
       <c r="M38" t="s">
         <v>29</v>
@@ -3009,10 +3111,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3024,13 +3126,13 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
+        <v>25</v>
+      </c>
+      <c r="K39" t="s">
         <v>26</v>
       </c>
-      <c r="K39" t="s">
-        <v>41</v>
-      </c>
       <c r="L39" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="M39" t="s">
         <v>29</v>
@@ -3042,7 +3144,7 @@
         <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>107</v>
+        <v>20</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3065,10 +3167,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>24</v>
+        <v>83</v>
       </c>
       <c r="F40" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3080,13 +3182,13 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="K40" t="s">
-        <v>42</v>
+        <v>142</v>
       </c>
       <c r="L40" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="M40" t="s">
         <v>29</v>
@@ -3098,7 +3200,7 @@
         <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3121,10 +3223,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="F41" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3136,13 +3238,13 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="K41" t="s">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="L41" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="M41" t="s">
         <v>29</v>
@@ -3177,10 +3279,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="F42" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3192,13 +3294,13 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="K42" t="s">
-        <v>27</v>
+        <v>68</v>
       </c>
       <c r="L42" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="M42" t="s">
         <v>29</v>
@@ -3207,13 +3309,13 @@
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="Q42" t="s">
         <v>31</v>
       </c>
       <c r="R42" t="s">
-        <v>109</v>
+        <v>20</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3236,10 +3338,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="F43" t="s">
-        <v>88</v>
+        <v>123</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3251,13 +3353,13 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="K43" t="s">
-        <v>91</v>
+        <v>125</v>
       </c>
       <c r="L43" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="M43" t="s">
         <v>29</v>
@@ -3292,10 +3394,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="F44" t="s">
-        <v>87</v>
+        <v>25</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3310,10 +3412,10 @@
         <v>26</v>
       </c>
       <c r="K44" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="L44" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="M44" t="s">
         <v>29</v>
@@ -3325,7 +3427,7 @@
         <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>86</v>
+        <v>20</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3348,10 +3450,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>84</v>
+        <v>44</v>
       </c>
       <c r="F45" t="s">
-        <v>41</v>
+        <v>145</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3363,13 +3465,13 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>26</v>
+        <v>146</v>
       </c>
       <c r="K45" t="s">
-        <v>27</v>
+        <v>147</v>
       </c>
       <c r="L45" t="s">
-        <v>28</v>
+        <v>148</v>
       </c>
       <c r="M45" t="s">
         <v>29</v>
@@ -3381,7 +3483,7 @@
         <v>31</v>
       </c>
       <c r="R45" t="s">
-        <v>109</v>
+        <v>20</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3404,10 +3506,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="F46" t="s">
-        <v>112</v>
+        <v>70</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3419,13 +3521,13 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>113</v>
+        <v>66</v>
       </c>
       <c r="K46" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="L46" t="s">
-        <v>115</v>
+        <v>71</v>
       </c>
       <c r="M46" t="s">
         <v>29</v>
@@ -3437,7 +3539,7 @@
         <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3460,10 +3562,10 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F47" t="s">
-        <v>117</v>
+        <v>25</v>
       </c>
       <c r="G47" t="s">
         <v>20</v>
@@ -3475,13 +3577,13 @@
         <v>20</v>
       </c>
       <c r="J47" t="s">
-        <v>118</v>
+        <v>26</v>
       </c>
       <c r="K47" t="s">
-        <v>119</v>
+        <v>27</v>
       </c>
       <c r="L47" t="s">
-        <v>120</v>
+        <v>28</v>
       </c>
       <c r="M47" t="s">
         <v>29</v>
@@ -3490,13 +3592,13 @@
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>121</v>
+        <v>150</v>
       </c>
       <c r="Q47" t="s">
         <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>116</v>
+        <v>149</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3519,10 +3621,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="F48" t="s">
-        <v>66</v>
+        <v>151</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3534,13 +3636,13 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="K48" t="s">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="L48" t="s">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="M48" t="s">
         <v>29</v>
@@ -3552,7 +3654,7 @@
         <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>20</v>
+        <v>149</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3575,10 +3677,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="F49" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3590,13 +3692,13 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="K49" t="s">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="L49" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="M49" t="s">
         <v>29</v>
@@ -3608,7 +3710,7 @@
         <v>31</v>
       </c>
       <c r="R49" t="s">
-        <v>20</v>
+        <v>149</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3631,10 +3733,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="F50" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3646,13 +3748,13 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>36</v>
+        <v>154</v>
       </c>
       <c r="K50" t="s">
-        <v>37</v>
+        <v>155</v>
       </c>
       <c r="L50" t="s">
-        <v>38</v>
+        <v>156</v>
       </c>
       <c r="M50" t="s">
         <v>29</v>
@@ -3664,7 +3766,7 @@
         <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>33</v>
+        <v>149</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3687,10 +3789,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="F51" t="s">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3702,13 +3804,13 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>60</v>
+        <v>34</v>
       </c>
       <c r="K51" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="L51" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="M51" t="s">
         <v>29</v>
@@ -3720,7 +3822,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>20</v>
+        <v>149</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3731,7 +3833,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
same solution bug fixed
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="163">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,31 +83,142 @@
     <t>09030201</t>
   </si>
   <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>Ans: $63$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 94$&lt;br&gt;No. of travellers using the vehicle least $= 31$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$94 - 31 = 63$  is the answer.&lt;br&gt;#उत्तर : $63$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 94$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 31$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$94 - 31 = 63$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>205</t>
+  </si>
+  <si>
+    <t>204</t>
+  </si>
+  <si>
+    <t>207</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Scooter $= 31$&lt;br&gt;No. of travellers using the Bus  $= 36$&lt;br&gt;No. of travellers using the Car  $= 75$&lt;br&gt;No. of travellers using the Motorcycle  $= 94$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$31 + 36 + 75 + 94 = 236$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Scooter या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 31$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 75$&lt;br&gt;Motorcycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 94$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$31 + 36 + 75 + 94 = 236$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>236</t>
+  </si>
+  <si>
+    <t>238</t>
+  </si>
+  <si>
+    <t>237</t>
+  </si>
+  <si>
+    <t>235</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
     <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
   </si>
   <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 240$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 690$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$240 + 690 = 930$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 690$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$240 + 690 = 930$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>930</t>
+  </si>
+  <si>
+    <t>928</t>
+  </si>
+  <si>
+    <t>931</t>
+  </si>
+  <si>
+    <t>929</t>
+  </si>
+  <si>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
   </si>
   <si>
     <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
@@ -125,10 +236,43 @@
     <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
   </si>
   <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 66$&lt;br&gt;No. of travellers using the Motorcycle  $= 61$&lt;br&gt;No. of travellers using the Scooter  $= 73$&lt;br&gt;No. of travellers using the Bicycle  $= 4$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$66 + 61 + 73 + 4 = 204$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 66$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 73$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$66 + 61 + 73 + 4 = 204$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>206</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Ans: Car, Motorcycle, Scooter, Bicycle&lt;br&gt;From the given graph we can see that, $Car$, $Motorcycle$, $Scooter$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Motorcycle, Scooter, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Motorcycle$, $Scooter$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
     <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
   </si>
   <si>
-    <t>Bicycle, Truck, Motorcycle, Car</t>
+    <t>Car, Motorcycle, Scooter, Bicycle</t>
   </si>
   <si>
     <t>Car, Bus, Truck, Motorcycle</t>
@@ -140,349 +284,220 @@
     <t>Bicycle, Bus, Truck, Motorcycle</t>
   </si>
   <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+    <t>Ans: Scooter, Car, Truck, Bus&lt;br&gt;From the given graph we can see that, $Scooter$, $Car$, $Truck$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Car, Truck, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Car$, $Truck$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter, Car, Truck, Bus</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 7$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 8$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$7 + 8 = 15$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$7 + 8 = 15$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bus$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 37$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 79$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$37 + 79 = 116$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 37$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 79$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$37 + 79 = 116$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>116</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>117</t>
+  </si>
+  <si>
+    <t>114</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Bus, Motorcycle, Scooter, Truck&lt;br&gt;From the given graph we can see that, $Bus$, $Motorcycle$, $Scooter$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bus, Motorcycle, Scooter, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bus$, $Motorcycle$, $Scooter$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus, Motorcycle, Scooter, Truck</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bus$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>Ans: $65$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 86$&lt;br&gt;No. of travellers using the vehicle least $= 21$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$86 - 21 = 65$  is the answer.&lt;br&gt;#उत्तर : $65$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 86$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 21$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$86 - 21 = 65$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>66</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>Ans: $800$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 930$&lt;br&gt;No. of travellers using the vehicle least $= 130$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$930 - 130 = 800$  is the answer.&lt;br&gt;#उत्तर : $800$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 930$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 130$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$930 - 130 = 800$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>800</t>
+  </si>
+  <si>
+    <t>798</t>
+  </si>
+  <si>
+    <t>801</t>
+  </si>
+  <si>
+    <t>799</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 280$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 850$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$280 + 850 = 1130$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 850$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$280 + 850 = 1130$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>1130</t>
+  </si>
+  <si>
+    <t>1131</t>
+  </si>
+  <si>
+    <t>1129</t>
+  </si>
+  <si>
+    <t>1132</t>
+  </si>
+  <si>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>1060</t>
+  </si>
+  <si>
+    <t>1061</t>
+  </si>
+  <si>
+    <t>1062</t>
+  </si>
+  <si>
+    <t>1059</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 4$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 6$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$4 + 6 = 10$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$4 + 6 = 10$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>20</t>
   </si>
   <si>
     <t>18</t>
   </si>
   <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?</t>
-  </si>
-  <si>
-    <t>174</t>
-  </si>
-  <si>
-    <t>172</t>
-  </si>
-  <si>
-    <t>176</t>
-  </si>
-  <si>
-    <t>173</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>Car, Motorcycle, Bus, Truck</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>74</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>75</t>
-  </si>
-  <si>
-    <t>73</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>Truck, Motorcycle, Bus, Scooter</t>
-  </si>
-  <si>
-    <t>Ans: $79$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 80$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$80 - 1 = 79$  is the answer.&lt;br&gt;#उत्तर : $79$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 80$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$80 - 1 = 79$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>79</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>166</t>
-  </si>
-  <si>
-    <t>168</t>
-  </si>
-  <si>
-    <t>167</t>
-  </si>
-  <si>
-    <t>164</t>
-  </si>
-  <si>
-    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>85</t>
-  </si>
-  <si>
-    <t>86</t>
-  </si>
-  <si>
-    <t>87</t>
-  </si>
-  <si>
-    <t>84</t>
-  </si>
-  <si>
-    <t>83</t>
-  </si>
-  <si>
-    <t>1660</t>
-  </si>
-  <si>
-    <t>1658</t>
-  </si>
-  <si>
-    <t>1662</t>
-  </si>
-  <si>
-    <t>1659</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>860</t>
-  </si>
-  <si>
-    <t>859</t>
-  </si>
-  <si>
-    <t>858</t>
-  </si>
-  <si>
-    <t>862</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>93</t>
-  </si>
-  <si>
-    <t>94</t>
-  </si>
-  <si>
-    <t>95</t>
-  </si>
-  <si>
-    <t>91</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>57</t>
-  </si>
-  <si>
-    <t>58</t>
-  </si>
-  <si>
-    <t>55</t>
-  </si>
-  <si>
-    <t>59</t>
-  </si>
-  <si>
-    <t>Truck, Motorcycle, Car, Bus</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>590</t>
-  </si>
-  <si>
-    <t>591</t>
-  </si>
-  <si>
-    <t>588</t>
-  </si>
-  <si>
-    <t>592</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>460</t>
-  </si>
-  <si>
-    <t>458</t>
-  </si>
-  <si>
-    <t>459</t>
-  </si>
-  <si>
-    <t>461</t>
-  </si>
-  <si>
-    <t>1090</t>
-  </si>
-  <si>
-    <t>1089</t>
-  </si>
-  <si>
-    <t>1088</t>
-  </si>
-  <si>
-    <t>1091</t>
-  </si>
-  <si>
-    <t>89</t>
-  </si>
-  <si>
-    <t>90</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>47</t>
-  </si>
-  <si>
-    <t>46</t>
-  </si>
-  <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>72</t>
+    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>14400</t>
+  </si>
+  <si>
+    <t>14401</t>
+  </si>
+  <si>
+    <t>14402</t>
+  </si>
+  <si>
+    <t>14398</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
   </si>
   <si>
-    <t>Car, Motorcycle, Scooter, Bus</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>127</t>
-  </si>
-  <si>
-    <t>129</t>
-  </si>
-  <si>
-    <t>125</t>
-  </si>
-  <si>
-    <t>126</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 36$&lt;br&gt;No. of travellers using the Motorcycle  $= 8$&lt;br&gt;No. of travellers using the Bus  $= 91$&lt;br&gt;No. of travellers using the Scooter  $= 82$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$36 + 8 + 91 + 82 = 217$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;Bus या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 91$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 82$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$36 + 8 + 91 + 82 = 217$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>217</t>
+  </si>
+  <si>
+    <t>218</t>
+  </si>
+  <si>
+    <t>219</t>
+  </si>
+  <si>
+    <t>215</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 36$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 82$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$36 + 82 = 118$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 82$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$36 + 82 = 118$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>119</t>
   </si>
   <si>
     <t>****</t>
@@ -1074,40 +1089,40 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R3" t="s">
         <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>34</v>
-      </c>
-      <c r="K3" t="s">
-        <v>35</v>
-      </c>
-      <c r="L3" t="s">
-        <v>36</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R3" t="s">
-        <v>23</v>
       </c>
       <c r="T3" t="n">
         <v>110.0</v>
@@ -1130,10 +1145,10 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1145,13 +1160,13 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="M4" t="s">
         <v>29</v>
@@ -1163,7 +1178,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1186,10 +1201,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1201,13 +1216,13 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K5" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="L5" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="M5" t="s">
         <v>29</v>
@@ -1219,7 +1234,7 @@
         <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1242,10 +1257,10 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1257,25 +1272,25 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="L6" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6" t="s">
         <v>48</v>
-      </c>
-      <c r="M6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N6" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>31</v>
-      </c>
-      <c r="R6" t="s">
-        <v>23</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1298,10 +1313,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1313,13 +1328,13 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="K7" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="L7" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="M7" t="s">
         <v>29</v>
@@ -1328,7 +1343,7 @@
         <v>4.0</v>
       </c>
       <c r="P7" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="s">
         <v>31</v>
@@ -1357,10 +1372,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1372,13 +1387,13 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="K8" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="L8" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="M8" t="s">
         <v>29</v>
@@ -1390,7 +1405,7 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1413,10 +1428,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1428,13 +1443,13 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>26</v>
+        <v>65</v>
       </c>
       <c r="K9" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
       <c r="L9" t="s">
-        <v>28</v>
+        <v>67</v>
       </c>
       <c r="M9" t="s">
         <v>29</v>
@@ -1446,7 +1461,7 @@
         <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1469,10 +1484,10 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1484,13 +1499,13 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="K10" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="L10" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="M10" t="s">
         <v>29</v>
@@ -1502,7 +1517,7 @@
         <v>31</v>
       </c>
       <c r="R10" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="T10" t="n">
         <v>110.0</v>
@@ -1525,10 +1540,10 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="G11" t="s">
         <v>20</v>
@@ -1540,13 +1555,13 @@
         <v>20</v>
       </c>
       <c r="J11" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K11" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="L11" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="M11" t="s">
         <v>29</v>
@@ -1558,7 +1573,7 @@
         <v>31</v>
       </c>
       <c r="R11" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1581,10 +1596,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1596,13 +1611,13 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="K12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="L12" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="M12" t="s">
         <v>29</v>
@@ -1611,13 +1626,13 @@
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="Q12" t="s">
         <v>31</v>
       </c>
       <c r="R12" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1640,29 +1655,29 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>81</v>
       </c>
       <c r="F13" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L13" t="s">
         <v>28</v>
       </c>
-      <c r="G13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" t="s">
-        <v>20</v>
-      </c>
-      <c r="J13" t="s">
-        <v>25</v>
-      </c>
-      <c r="K13" t="s">
-        <v>64</v>
-      </c>
-      <c r="L13" t="s">
-        <v>43</v>
-      </c>
       <c r="M13" t="s">
         <v>29</v>
       </c>
@@ -1673,7 +1688,7 @@
         <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1696,10 +1711,10 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="G14" t="s">
         <v>20</v>
@@ -1711,13 +1726,13 @@
         <v>20</v>
       </c>
       <c r="J14" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="K14" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="L14" t="s">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="M14" t="s">
         <v>29</v>
@@ -1729,7 +1744,7 @@
         <v>31</v>
       </c>
       <c r="R14" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1752,10 +1767,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1767,13 +1782,13 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>46</v>
       </c>
       <c r="K15" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="L15" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="M15" t="s">
         <v>29</v>
@@ -1785,7 +1800,7 @@
         <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1808,10 +1823,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1823,13 +1838,13 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="K16" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="L16" t="s">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -1841,7 +1856,7 @@
         <v>31</v>
       </c>
       <c r="R16" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="T16" t="n">
         <v>110.0</v>
@@ -1864,10 +1879,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="F17" t="s">
-        <v>74</v>
+        <v>91</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1879,13 +1894,13 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="K17" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="L17" t="s">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="M17" t="s">
         <v>29</v>
@@ -1894,13 +1909,13 @@
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="Q17" t="s">
         <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1923,10 +1938,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1938,13 +1953,13 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="K18" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="L18" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="M18" t="s">
         <v>29</v>
@@ -1956,7 +1971,7 @@
         <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -1979,10 +1994,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="F19" t="s">
-        <v>28</v>
+        <v>99</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -1994,13 +2009,13 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="K19" t="s">
-        <v>64</v>
+        <v>27</v>
       </c>
       <c r="L19" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="M19" t="s">
         <v>29</v>
@@ -2012,7 +2027,7 @@
         <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2035,10 +2050,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="F20" t="s">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2050,13 +2065,13 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>85</v>
+        <v>26</v>
       </c>
       <c r="K20" t="s">
-        <v>86</v>
+        <v>25</v>
       </c>
       <c r="L20" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="M20" t="s">
         <v>29</v>
@@ -2068,7 +2083,7 @@
         <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>73</v>
+        <v>100</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2091,10 +2106,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2106,13 +2121,13 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="K21" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="L21" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="M21" t="s">
         <v>29</v>
@@ -2124,7 +2139,7 @@
         <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>73</v>
+        <v>20</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2147,10 +2162,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F22" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2162,13 +2177,13 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="K22" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="L22" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -2177,13 +2192,13 @@
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="Q22" t="s">
         <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>20</v>
+        <v>102</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2206,10 +2221,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="F23" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2221,13 +2236,13 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="K23" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="L23" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="M23" t="s">
         <v>29</v>
@@ -2262,10 +2277,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="F24" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2277,13 +2292,13 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="K24" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="L24" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="M24" t="s">
         <v>29</v>
@@ -2295,7 +2310,7 @@
         <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2318,10 +2333,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="F25" t="s">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2333,13 +2348,13 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>96</v>
+        <v>26</v>
       </c>
       <c r="K25" t="s">
-        <v>97</v>
+        <v>25</v>
       </c>
       <c r="L25" t="s">
-        <v>98</v>
+        <v>76</v>
       </c>
       <c r="M25" t="s">
         <v>29</v>
@@ -2351,7 +2366,7 @@
         <v>31</v>
       </c>
       <c r="R25" t="s">
-        <v>20</v>
+        <v>74</v>
       </c>
       <c r="T25" t="n">
         <v>110.0</v>
@@ -2374,10 +2389,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="F26" t="s">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2389,13 +2404,13 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>101</v>
+        <v>26</v>
       </c>
       <c r="K26" t="s">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="L26" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="M26" t="s">
         <v>29</v>
@@ -2407,7 +2422,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2430,10 +2445,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>104</v>
+        <v>76</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2445,13 +2460,13 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="K27" t="s">
-        <v>106</v>
+        <v>27</v>
       </c>
       <c r="L27" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
       <c r="M27" t="s">
         <v>29</v>
@@ -2460,13 +2475,13 @@
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="Q27" t="s">
         <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>20</v>
+        <v>112</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2489,10 +2504,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="F28" t="s">
-        <v>109</v>
+        <v>76</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2504,25 +2519,25 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="K28" t="s">
-        <v>111</v>
+        <v>27</v>
       </c>
       <c r="L28" t="s">
+        <v>28</v>
+      </c>
+      <c r="M28" t="s">
+        <v>29</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>31</v>
+      </c>
+      <c r="R28" t="s">
         <v>112</v>
-      </c>
-      <c r="M28" t="s">
-        <v>29</v>
-      </c>
-      <c r="N28" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>31</v>
-      </c>
-      <c r="R28" t="s">
-        <v>20</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2545,10 +2560,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="F29" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2560,13 +2575,13 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="K29" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="L29" t="s">
-        <v>43</v>
+        <v>73</v>
       </c>
       <c r="M29" t="s">
         <v>29</v>
@@ -2578,7 +2593,7 @@
         <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2601,10 +2616,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2616,13 +2631,13 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="K30" t="s">
-        <v>40</v>
+        <v>116</v>
       </c>
       <c r="L30" t="s">
-        <v>41</v>
+        <v>117</v>
       </c>
       <c r="M30" t="s">
         <v>29</v>
@@ -2634,7 +2649,7 @@
         <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>20</v>
+        <v>114</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2657,10 +2672,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>114</v>
+        <v>43</v>
       </c>
       <c r="F31" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2672,13 +2687,13 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="K31" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="L31" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="M31" t="s">
         <v>29</v>
@@ -2713,10 +2728,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F32" t="s">
-        <v>28</v>
+        <v>119</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2728,13 +2743,13 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>25</v>
+        <v>120</v>
       </c>
       <c r="K32" t="s">
-        <v>64</v>
+        <v>121</v>
       </c>
       <c r="L32" t="s">
-        <v>43</v>
+        <v>122</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
@@ -2743,13 +2758,13 @@
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="Q32" t="s">
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2772,10 +2787,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F33" t="s">
-        <v>118</v>
+        <v>99</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2787,13 +2802,13 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>119</v>
+        <v>26</v>
       </c>
       <c r="K33" t="s">
-        <v>120</v>
+        <v>27</v>
       </c>
       <c r="L33" t="s">
-        <v>121</v>
+        <v>61</v>
       </c>
       <c r="M33" t="s">
         <v>29</v>
@@ -2805,7 +2820,7 @@
         <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>117</v>
+        <v>98</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2828,10 +2843,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>122</v>
+        <v>63</v>
       </c>
       <c r="F34" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2843,25 +2858,25 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
+        <v>126</v>
+      </c>
+      <c r="K34" t="s">
+        <v>127</v>
+      </c>
+      <c r="L34" t="s">
+        <v>128</v>
+      </c>
+      <c r="M34" t="s">
+        <v>29</v>
+      </c>
+      <c r="N34" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>31</v>
+      </c>
+      <c r="R34" t="s">
         <v>124</v>
-      </c>
-      <c r="K34" t="s">
-        <v>125</v>
-      </c>
-      <c r="L34" t="s">
-        <v>126</v>
-      </c>
-      <c r="M34" t="s">
-        <v>29</v>
-      </c>
-      <c r="N34" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>31</v>
-      </c>
-      <c r="R34" t="s">
-        <v>117</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2884,10 +2899,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>57</v>
+        <v>129</v>
       </c>
       <c r="F35" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2899,13 +2914,13 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="K35" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="L35" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="M35" t="s">
         <v>29</v>
@@ -2917,7 +2932,7 @@
         <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>117</v>
+        <v>20</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2940,10 +2955,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="F36" t="s">
-        <v>131</v>
+        <v>76</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -2955,13 +2970,13 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>132</v>
+        <v>26</v>
       </c>
       <c r="K36" t="s">
-        <v>133</v>
+        <v>27</v>
       </c>
       <c r="L36" t="s">
-        <v>134</v>
+        <v>28</v>
       </c>
       <c r="M36" t="s">
         <v>29</v>
@@ -2973,7 +2988,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -2996,10 +3011,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>65</v>
+        <v>82</v>
       </c>
       <c r="F37" t="s">
-        <v>135</v>
+        <v>99</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3011,13 +3026,13 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="K37" t="s">
-        <v>136</v>
+        <v>27</v>
       </c>
       <c r="L37" t="s">
-        <v>107</v>
+        <v>61</v>
       </c>
       <c r="M37" t="s">
         <v>29</v>
@@ -3026,13 +3041,13 @@
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="Q37" t="s">
         <v>31</v>
       </c>
       <c r="R37" t="s">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3055,10 +3070,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="F38" t="s">
-        <v>138</v>
+        <v>47</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3070,13 +3085,13 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>139</v>
+        <v>44</v>
       </c>
       <c r="K38" t="s">
-        <v>140</v>
+        <v>45</v>
       </c>
       <c r="L38" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="M38" t="s">
         <v>29</v>
@@ -3111,10 +3126,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="F39" t="s">
-        <v>64</v>
+        <v>137</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3126,13 +3141,13 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>25</v>
+        <v>138</v>
       </c>
       <c r="K39" t="s">
-        <v>26</v>
+        <v>139</v>
       </c>
       <c r="L39" t="s">
-        <v>27</v>
+        <v>140</v>
       </c>
       <c r="M39" t="s">
         <v>29</v>
@@ -3144,7 +3159,7 @@
         <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>20</v>
+        <v>136</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3167,10 +3182,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="F40" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3182,13 +3197,13 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="K40" t="s">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="L40" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="M40" t="s">
         <v>29</v>
@@ -3200,7 +3215,7 @@
         <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3223,10 +3238,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="F41" t="s">
-        <v>25</v>
+        <v>141</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3238,13 +3253,13 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>26</v>
+        <v>142</v>
       </c>
       <c r="K41" t="s">
-        <v>27</v>
+        <v>143</v>
       </c>
       <c r="L41" t="s">
-        <v>28</v>
+        <v>144</v>
       </c>
       <c r="M41" t="s">
         <v>29</v>
@@ -3279,10 +3294,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="F42" t="s">
-        <v>66</v>
+        <v>145</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3294,13 +3309,13 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="K42" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="L42" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="M42" t="s">
         <v>29</v>
@@ -3309,7 +3324,7 @@
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="Q42" t="s">
         <v>31</v>
@@ -3338,10 +3353,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>122</v>
+        <v>24</v>
       </c>
       <c r="F43" t="s">
-        <v>123</v>
+        <v>26</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3353,13 +3368,13 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>126</v>
+        <v>27</v>
       </c>
       <c r="K43" t="s">
-        <v>125</v>
+        <v>28</v>
       </c>
       <c r="L43" t="s">
-        <v>144</v>
+        <v>61</v>
       </c>
       <c r="M43" t="s">
         <v>29</v>
@@ -3371,7 +3386,7 @@
         <v>31</v>
       </c>
       <c r="R43" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3394,10 +3409,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="F44" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3409,13 +3424,13 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="K44" t="s">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="L44" t="s">
-        <v>28</v>
+        <v>73</v>
       </c>
       <c r="M44" t="s">
         <v>29</v>
@@ -3427,7 +3442,7 @@
         <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3450,10 +3465,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="F45" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3465,13 +3480,13 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="K45" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="L45" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="M45" t="s">
         <v>29</v>
@@ -3506,10 +3521,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="F46" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3521,13 +3536,13 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="K46" t="s">
-        <v>68</v>
+        <v>27</v>
       </c>
       <c r="L46" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="M46" t="s">
         <v>29</v>
@@ -3539,7 +3554,7 @@
         <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3562,7 +3577,7 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="F47" t="s">
         <v>25</v>
@@ -3592,13 +3607,13 @@
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="Q47" t="s">
         <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3621,10 +3636,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="F48" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3636,13 +3651,13 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>39</v>
+        <v>156</v>
       </c>
       <c r="K48" t="s">
-        <v>40</v>
+        <v>157</v>
       </c>
       <c r="L48" t="s">
-        <v>41</v>
+        <v>158</v>
       </c>
       <c r="M48" t="s">
         <v>29</v>
@@ -3654,7 +3669,7 @@
         <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3677,40 +3692,40 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="F49" t="s">
+        <v>25</v>
+      </c>
+      <c r="G49" t="s">
+        <v>20</v>
+      </c>
+      <c r="H49" t="s">
+        <v>20</v>
+      </c>
+      <c r="I49" t="s">
+        <v>20</v>
+      </c>
+      <c r="J49" t="s">
+        <v>26</v>
+      </c>
+      <c r="K49" t="s">
+        <v>27</v>
+      </c>
+      <c r="L49" t="s">
+        <v>28</v>
+      </c>
+      <c r="M49" t="s">
+        <v>29</v>
+      </c>
+      <c r="N49" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>31</v>
+      </c>
+      <c r="R49" t="s">
         <v>152</v>
-      </c>
-      <c r="G49" t="s">
-        <v>20</v>
-      </c>
-      <c r="H49" t="s">
-        <v>20</v>
-      </c>
-      <c r="I49" t="s">
-        <v>20</v>
-      </c>
-      <c r="J49" t="s">
-        <v>101</v>
-      </c>
-      <c r="K49" t="s">
-        <v>102</v>
-      </c>
-      <c r="L49" t="s">
-        <v>103</v>
-      </c>
-      <c r="M49" t="s">
-        <v>29</v>
-      </c>
-      <c r="N49" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q49" t="s">
-        <v>31</v>
-      </c>
-      <c r="R49" t="s">
-        <v>149</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3733,10 +3748,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="F50" t="s">
-        <v>153</v>
+        <v>70</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3748,13 +3763,13 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>154</v>
+        <v>71</v>
       </c>
       <c r="K50" t="s">
-        <v>155</v>
+        <v>72</v>
       </c>
       <c r="L50" t="s">
-        <v>156</v>
+        <v>73</v>
       </c>
       <c r="M50" t="s">
         <v>29</v>
@@ -3766,7 +3781,7 @@
         <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>149</v>
+        <v>68</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3789,10 +3804,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="F51" t="s">
-        <v>33</v>
+        <v>104</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3804,13 +3819,13 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>34</v>
+        <v>160</v>
       </c>
       <c r="K51" t="s">
-        <v>35</v>
+        <v>161</v>
       </c>
       <c r="L51" t="s">
-        <v>36</v>
+        <v>103</v>
       </c>
       <c r="M51" t="s">
         <v>29</v>
@@ -3822,7 +3837,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3833,7 +3848,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
marathi vechicle name solution fixed
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="177">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,103 +83,250 @@
     <t>09030201</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of travelers by different means.</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
   </si>
   <si>
     <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
   </si>
   <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
-  </si>
-  <si>
-    <t>Ans: $63$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 94$&lt;br&gt;No. of travellers using the vehicle least $= 31$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$94 - 31 = 63$  is the answer.&lt;br&gt;#उत्तर : $63$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 94$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 31$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$94 - 31 = 63$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 480$&lt;br&gt;No. of travellers using the Bicycle  $= 270$&lt;br&gt;No. of travellers using the Truck  $= 280$&lt;br&gt;No. of travellers using the Bus  $= 100$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$480 + 270 + 280 + 100 = 1130$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 480$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 270$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 100$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$480 + 270 + 280 + 100 = 1130$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>1130</t>
+  </si>
+  <si>
+    <t>1128</t>
+  </si>
+  <si>
+    <t>1132</t>
+  </si>
+  <si>
+    <t>1129</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 270$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 280$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$270 + 280 = 550$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 270$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$270 + 280 = 550$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>550</t>
+  </si>
+  <si>
+    <t>548</t>
+  </si>
+  <si>
+    <t>551</t>
+  </si>
+  <si>
+    <t>549</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Bicycle, Truck, Bus&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bicycle$, $Truck$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bicycle, Truck, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bicycle$, $Truck$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Bicycle, Truck, Bus</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Ans: $5100$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 6600$&lt;br&gt;No. of travellers using the vehicle least $= 1500$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$6600 - 1500 = 5100$  is the answer.&lt;br&gt;#उत्तर : $5100$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6600$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1500$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$6600 - 1500 = 5100$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
   </si>
   <si>
-    <t>63</t>
-  </si>
-  <si>
-    <t>62</t>
-  </si>
-  <si>
-    <t>64</t>
-  </si>
-  <si>
-    <t>61</t>
+    <t>5100</t>
+  </si>
+  <si>
+    <t>5101</t>
+  </si>
+  <si>
+    <t>5099</t>
+  </si>
+  <si>
+    <t>5102</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bicycle $= 2700$&lt;br&gt;No. of travellers using the Truck  $= 1500$&lt;br&gt;No. of travellers using the Motorcycle  $= 6600$&lt;br&gt;No. of travellers using the Bus  $= 3800$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$2700 + 1500 + 6600 + 3800 = 14600$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bicycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 2700$&lt;br&gt;Truck या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 1500$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6600$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$2700 + 1500 + 6600 + 3800 = 14600$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>14600</t>
+  </si>
+  <si>
+    <t>14602</t>
+  </si>
+  <si>
+    <t>14599</t>
+  </si>
+  <si>
+    <t>14601</t>
   </si>
   <si>
     <t>How much is the total of travellers for top 3 values?</t>
   </si>
   <si>
-    <t>205</t>
-  </si>
-  <si>
-    <t>204</t>
-  </si>
-  <si>
-    <t>207</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Scooter $= 31$&lt;br&gt;No. of travellers using the Bus  $= 36$&lt;br&gt;No. of travellers using the Car  $= 75$&lt;br&gt;No. of travellers using the Motorcycle  $= 94$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$31 + 36 + 75 + 94 = 236$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Scooter या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 31$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 75$&lt;br&gt;Motorcycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 94$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$31 + 36 + 75 + 94 = 236$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>236</t>
-  </si>
-  <si>
-    <t>238</t>
-  </si>
-  <si>
-    <t>237</t>
-  </si>
-  <si>
-    <t>235</t>
+    <t>13100</t>
+  </si>
+  <si>
+    <t>13101</t>
+  </si>
+  <si>
+    <t>13099</t>
+  </si>
+  <si>
+    <t>13102</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Truck, Motorcycle, Bus&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Motorcycle$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Motorcycle, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Motorcycle$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Truck, Motorcycle, Bus</t>
+  </si>
+  <si>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>8100</t>
+  </si>
+  <si>
+    <t>8101</t>
+  </si>
+  <si>
+    <t>8102</t>
+  </si>
+  <si>
+    <t>8098</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>79</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 37$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 56$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$37 + 56 = 93$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 37$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 56$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$37 + 56 = 93$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>91</t>
+  </si>
+  <si>
+    <t>94</t>
+  </si>
+  <si>
+    <t>95</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
   </si>
   <si>
     <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
   </si>
   <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
+    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
@@ -191,313 +338,208 @@
     <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Car$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 240$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 690$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$240 + 690 = 930$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 690$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$240 + 690 = 930$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>930</t>
-  </si>
-  <si>
-    <t>928</t>
-  </si>
-  <si>
-    <t>931</t>
-  </si>
-  <si>
-    <t>929</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of travelers by different means.</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Truck$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 66$&lt;br&gt;No. of travellers using the Motorcycle  $= 61$&lt;br&gt;No. of travellers using the Scooter  $= 73$&lt;br&gt;No. of travellers using the Bicycle  $= 4$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$66 + 61 + 73 + 4 = 204$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 66$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 73$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$66 + 61 + 73 + 4 = 204$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>206</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Ans: Car, Motorcycle, Scooter, Bicycle&lt;br&gt;From the given graph we can see that, $Car$, $Motorcycle$, $Scooter$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Motorcycle, Scooter, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Motorcycle$, $Scooter$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Motorcycle, Scooter, Bicycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Ans: Scooter, Car, Truck, Bus&lt;br&gt;From the given graph we can see that, $Scooter$, $Car$, $Truck$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Car, Truck, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Car$, $Truck$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter, Car, Truck, Bus</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 7$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 8$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$7 + 8 = 15$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$7 + 8 = 15$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>16</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>Ans: $6700$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 7200$&lt;br&gt;No. of travellers using the vehicle least $= 500$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$7200 - 500 = 6700$  is the answer.&lt;br&gt;#उत्तर : $6700$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7200$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 500$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$7200 - 500 = 6700$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>6700</t>
+  </si>
+  <si>
+    <t>6699</t>
+  </si>
+  <si>
+    <t>6702</t>
+  </si>
+  <si>
+    <t>6698</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 5300$&lt;br&gt;No. of travellers using the Bus  $= 4700$&lt;br&gt;No. of travellers using the Bicycle  $= 7200$&lt;br&gt;No. of travellers using the Truck  $= 500$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$5300 + 4700 + 7200 + 500 = 17700$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 5300$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 4700$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7200$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 500$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$5300 + 4700 + 7200 + 500 = 17700$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>17700</t>
+  </si>
+  <si>
+    <t>17698</t>
+  </si>
+  <si>
+    <t>17701</t>
+  </si>
+  <si>
+    <t>17702</t>
+  </si>
+  <si>
+    <t>17200</t>
+  </si>
+  <si>
+    <t>17198</t>
+  </si>
+  <si>
+    <t>17201</t>
+  </si>
+  <si>
+    <t>17199</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 2$&lt;br&gt;No. of travellers using the Scooter  $= 2$&lt;br&gt;No. of travellers using the Truck  $= 9$&lt;br&gt;No. of travellers using the Motorcycle  $= 9$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$2 + 2 + 9 + 9 = 22$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;Scooter या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;Motorcycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$2 + 2 + 9 + 9 = 22$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 30$&lt;br&gt;No. of travellers using the Bus  $= 20$&lt;br&gt;No. of travellers using the Car  $= 76$&lt;br&gt;No. of travellers using the Truck  $= 11$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$30 + 20 + 76 + 11 = 137$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 30$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 20$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 76$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 11$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$30 + 20 + 76 + 11 = 137$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>137</t>
+  </si>
+  <si>
+    <t>138</t>
+  </si>
+  <si>
+    <t>139</t>
+  </si>
+  <si>
+    <t>135</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>11200</t>
+  </si>
+  <si>
+    <t>11201</t>
+  </si>
+  <si>
+    <t>11199</t>
+  </si>
+  <si>
+    <t>11202</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bus$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 37$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 79$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$37 + 79 = 116$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 37$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 79$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$37 + 79 = 116$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>116</t>
-  </si>
-  <si>
-    <t>118</t>
-  </si>
-  <si>
-    <t>117</t>
-  </si>
-  <si>
-    <t>114</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Bus, Motorcycle, Scooter, Truck&lt;br&gt;From the given graph we can see that, $Bus$, $Motorcycle$, $Scooter$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bus, Motorcycle, Scooter, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bus$, $Motorcycle$, $Scooter$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus, Motorcycle, Scooter, Truck</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Bus$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Bicycle$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>Ans: $65$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 86$&lt;br&gt;No. of travellers using the vehicle least $= 21$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$86 - 21 = 65$  is the answer.&lt;br&gt;#उत्तर : $65$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 86$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 21$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$86 - 21 = 65$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>65</t>
-  </si>
-  <si>
-    <t>66</t>
-  </si>
-  <si>
-    <t>67</t>
-  </si>
-  <si>
-    <t>Ans: $800$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 930$&lt;br&gt;No. of travellers using the vehicle least $= 130$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$930 - 130 = 800$  is the answer.&lt;br&gt;#उत्तर : $800$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 930$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 130$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$930 - 130 = 800$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>800</t>
-  </si>
-  <si>
-    <t>798</t>
-  </si>
-  <si>
-    <t>801</t>
-  </si>
-  <si>
-    <t>799</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 280$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 850$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$280 + 850 = 1130$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 850$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$280 + 850 = 1130$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>1130</t>
-  </si>
-  <si>
-    <t>1131</t>
-  </si>
-  <si>
-    <t>1129</t>
-  </si>
-  <si>
-    <t>1132</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>1060</t>
-  </si>
-  <si>
-    <t>1061</t>
-  </si>
-  <si>
-    <t>1062</t>
-  </si>
-  <si>
-    <t>1059</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 4$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 6$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$4 + 6 = 10$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$4 + 6 = 10$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 4700$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 4700$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$4700 + 4700 = 9400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4700$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4700$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$4700 + 4700 = 9400$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>9400</t>
+  </si>
+  <si>
+    <t>9402</t>
+  </si>
+  <si>
+    <t>9398</t>
+  </si>
+  <si>
+    <t>9401</t>
+  </si>
+  <si>
+    <t>9800</t>
+  </si>
+  <si>
+    <t>9799</t>
+  </si>
+  <si>
+    <t>9798</t>
+  </si>
+  <si>
+    <t>9802</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
   </si>
   <si>
-    <t>14400</t>
-  </si>
-  <si>
-    <t>14401</t>
-  </si>
-  <si>
-    <t>14402</t>
-  </si>
-  <si>
-    <t>14398</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= Scooter$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= Motorcycle$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>Ans: Bicycle, Car, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Bicycle$, $Car$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Car, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Car$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Car, Bus, Scooter</t>
+  </si>
+  <si>
+    <t>20200</t>
+  </si>
+  <si>
+    <t>20198</t>
+  </si>
+  <si>
+    <t>20202</t>
+  </si>
+  <si>
+    <t>20199</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 36$&lt;br&gt;No. of travellers using the Motorcycle  $= 8$&lt;br&gt;No. of travellers using the Bus  $= 91$&lt;br&gt;No. of travellers using the Scooter  $= 82$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$36 + 8 + 91 + 82 = 217$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;Bus या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 91$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 82$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$36 + 8 + 91 + 82 = 217$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>217</t>
-  </si>
-  <si>
-    <t>218</t>
-  </si>
-  <si>
-    <t>219</t>
-  </si>
-  <si>
-    <t>215</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 36$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 82$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$36 + 82 = 118$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 82$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$36 + 82 = 118$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>120</t>
-  </si>
-  <si>
-    <t>119</t>
+    <t>Ans: $880$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 910$&lt;br&gt;No. of travellers using the vehicle least $= 30$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$910 - 30 = 880$  is the answer.&lt;br&gt;#उत्तर : $880$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 910$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 30$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$910 - 30 = 880$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>880</t>
+  </si>
+  <si>
+    <t>879</t>
+  </si>
+  <si>
+    <t>881</t>
+  </si>
+  <si>
+    <t>882</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 290$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 830$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$290 + 830 = 1120$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 290$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 830$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$290 + 830 = 1120$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>1120</t>
+  </si>
+  <si>
+    <t>1118</t>
+  </si>
+  <si>
+    <t>1121</t>
+  </si>
+  <si>
+    <t>1122</t>
   </si>
   <si>
     <t>****</t>
@@ -1089,10 +1131,10 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
         <v>20</v>
@@ -1104,13 +1146,13 @@
         <v>20</v>
       </c>
       <c r="J3" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="K3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="M3" t="s">
         <v>29</v>
@@ -1122,7 +1164,7 @@
         <v>31</v>
       </c>
       <c r="R3" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="T3" t="n">
         <v>110.0</v>
@@ -1145,10 +1187,10 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1160,13 +1202,13 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="K4" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="M4" t="s">
         <v>29</v>
@@ -1178,7 +1220,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1201,10 +1243,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1216,13 +1258,13 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="K5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="L5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="M5" t="s">
         <v>29</v>
@@ -1234,7 +1276,7 @@
         <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1257,10 +1299,10 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1272,13 +1314,13 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="K6" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="L6" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="M6" t="s">
         <v>29</v>
@@ -1290,7 +1332,7 @@
         <v>31</v>
       </c>
       <c r="R6" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1313,10 +1355,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1328,13 +1370,13 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="L7" t="s">
-        <v>58</v>
+        <v>28</v>
       </c>
       <c r="M7" t="s">
         <v>29</v>
@@ -1343,13 +1385,13 @@
         <v>4.0</v>
       </c>
       <c r="P7" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="Q7" t="s">
         <v>31</v>
       </c>
       <c r="R7" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="T7" t="n">
         <v>110.0</v>
@@ -1372,10 +1414,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="F8" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1387,13 +1429,13 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="K8" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="L8" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="M8" t="s">
         <v>29</v>
@@ -1405,7 +1447,7 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1428,10 +1470,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="F9" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1443,13 +1485,13 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="K9" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="L9" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="M9" t="s">
         <v>29</v>
@@ -1461,7 +1503,7 @@
         <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1484,10 +1526,10 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1499,13 +1541,13 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="K10" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="L10" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="M10" t="s">
         <v>29</v>
@@ -1517,7 +1559,7 @@
         <v>31</v>
       </c>
       <c r="R10" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="T10" t="n">
         <v>110.0</v>
@@ -1540,40 +1582,40 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" t="s">
+        <v>64</v>
+      </c>
+      <c r="K11" t="s">
+        <v>65</v>
+      </c>
+      <c r="L11" t="s">
+        <v>66</v>
+      </c>
+      <c r="M11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" t="s">
         <v>61</v>
-      </c>
-      <c r="G11" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" t="s">
-        <v>26</v>
-      </c>
-      <c r="K11" t="s">
-        <v>25</v>
-      </c>
-      <c r="L11" t="s">
-        <v>76</v>
-      </c>
-      <c r="M11" t="s">
-        <v>29</v>
-      </c>
-      <c r="N11" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>31</v>
-      </c>
-      <c r="R11" t="s">
-        <v>74</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1596,10 +1638,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1611,13 +1653,13 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="K12" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="L12" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="M12" t="s">
         <v>29</v>
@@ -1626,13 +1668,13 @@
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="Q12" t="s">
         <v>31</v>
       </c>
       <c r="R12" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1655,28 +1697,28 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>45</v>
       </c>
       <c r="F13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" t="s">
         <v>76</v>
       </c>
-      <c r="G13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" t="s">
-        <v>20</v>
-      </c>
-      <c r="J13" t="s">
-        <v>26</v>
-      </c>
       <c r="K13" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="L13" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="M13" t="s">
         <v>29</v>
@@ -1688,7 +1730,7 @@
         <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1711,28 +1753,28 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" t="s">
+        <v>81</v>
+      </c>
+      <c r="K14" t="s">
         <v>82</v>
       </c>
-      <c r="F14" t="s">
-        <v>76</v>
-      </c>
-      <c r="G14" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" t="s">
-        <v>26</v>
-      </c>
-      <c r="K14" t="s">
-        <v>27</v>
-      </c>
       <c r="L14" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="M14" t="s">
         <v>29</v>
@@ -1744,7 +1786,7 @@
         <v>31</v>
       </c>
       <c r="R14" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1767,10 +1809,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="F15" t="s">
-        <v>44</v>
+        <v>85</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1782,13 +1824,13 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="K15" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="L15" t="s">
-        <v>83</v>
+        <v>66</v>
       </c>
       <c r="M15" t="s">
         <v>29</v>
@@ -1800,7 +1842,7 @@
         <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1823,10 +1865,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1838,13 +1880,13 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="L16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -1856,7 +1898,7 @@
         <v>31</v>
       </c>
       <c r="R16" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="T16" t="n">
         <v>110.0</v>
@@ -1879,7 +1921,7 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F17" t="s">
         <v>91</v>
@@ -1894,13 +1936,13 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="K17" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="L17" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="M17" t="s">
         <v>29</v>
@@ -1909,13 +1951,13 @@
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="Q17" t="s">
         <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1938,10 +1980,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="F18" t="s">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1953,13 +1995,13 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="K18" t="s">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="L18" t="s">
-        <v>97</v>
+        <v>41</v>
       </c>
       <c r="M18" t="s">
         <v>29</v>
@@ -1971,7 +2013,7 @@
         <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>93</v>
+        <v>36</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -1994,10 +2036,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="F19" t="s">
-        <v>99</v>
+        <v>25</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -2015,7 +2057,7 @@
         <v>27</v>
       </c>
       <c r="L19" t="s">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="M19" t="s">
         <v>29</v>
@@ -2027,7 +2069,7 @@
         <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2050,10 +2092,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="F20" t="s">
-        <v>27</v>
+        <v>97</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2065,13 +2107,13 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>26</v>
+        <v>98</v>
       </c>
       <c r="K20" t="s">
-        <v>25</v>
+        <v>99</v>
       </c>
       <c r="L20" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="M20" t="s">
         <v>29</v>
@@ -2083,7 +2125,7 @@
         <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2106,40 +2148,40 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="F21" t="s">
+        <v>102</v>
+      </c>
+      <c r="G21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21" t="s">
+        <v>20</v>
+      </c>
+      <c r="I21" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" t="s">
+        <v>35</v>
+      </c>
+      <c r="L21" t="s">
+        <v>25</v>
+      </c>
+      <c r="M21" t="s">
+        <v>29</v>
+      </c>
+      <c r="N21" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>31</v>
+      </c>
+      <c r="R21" t="s">
         <v>101</v>
-      </c>
-      <c r="G21" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" t="s">
-        <v>20</v>
-      </c>
-      <c r="I21" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" t="s">
-        <v>56</v>
-      </c>
-      <c r="K21" t="s">
-        <v>57</v>
-      </c>
-      <c r="L21" t="s">
-        <v>58</v>
-      </c>
-      <c r="M21" t="s">
-        <v>29</v>
-      </c>
-      <c r="N21" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>31</v>
-      </c>
-      <c r="R21" t="s">
-        <v>20</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2162,10 +2204,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
       <c r="F22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2177,13 +2219,13 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -2192,13 +2234,13 @@
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="Q22" t="s">
         <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>102</v>
+        <v>20</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2221,10 +2263,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="F23" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2236,13 +2278,13 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>56</v>
+        <v>111</v>
       </c>
       <c r="K23" t="s">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="L23" t="s">
-        <v>58</v>
+        <v>113</v>
       </c>
       <c r="M23" t="s">
         <v>29</v>
@@ -2254,7 +2296,7 @@
         <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2277,10 +2319,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="F24" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2292,13 +2334,13 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>87</v>
+        <v>116</v>
       </c>
       <c r="K24" t="s">
-        <v>88</v>
+        <v>117</v>
       </c>
       <c r="L24" t="s">
-        <v>89</v>
+        <v>118</v>
       </c>
       <c r="M24" t="s">
         <v>29</v>
@@ -2310,7 +2352,7 @@
         <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2333,10 +2375,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F25" t="s">
-        <v>61</v>
+        <v>119</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2348,13 +2390,13 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="K25" t="s">
-        <v>25</v>
+        <v>121</v>
       </c>
       <c r="L25" t="s">
-        <v>76</v>
+        <v>122</v>
       </c>
       <c r="M25" t="s">
         <v>29</v>
@@ -2366,7 +2408,7 @@
         <v>31</v>
       </c>
       <c r="R25" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="T25" t="n">
         <v>110.0</v>
@@ -2389,28 +2431,28 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>81</v>
+        <v>32</v>
       </c>
       <c r="F26" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J26" t="s">
         <v>27</v>
       </c>
-      <c r="G26" t="s">
-        <v>20</v>
-      </c>
-      <c r="H26" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" t="s">
-        <v>20</v>
-      </c>
-      <c r="J26" t="s">
-        <v>26</v>
-      </c>
       <c r="K26" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="L26" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="M26" t="s">
         <v>29</v>
@@ -2422,7 +2464,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2445,10 +2487,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F27" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2460,13 +2502,13 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="K27" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="L27" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="M27" t="s">
         <v>29</v>
@@ -2475,13 +2517,13 @@
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="Q27" t="s">
         <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>112</v>
+        <v>36</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2504,10 +2546,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="F28" t="s">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2519,13 +2561,13 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>26</v>
+        <v>52</v>
       </c>
       <c r="K28" t="s">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="L28" t="s">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="M28" t="s">
         <v>29</v>
@@ -2537,7 +2579,7 @@
         <v>31</v>
       </c>
       <c r="R28" t="s">
-        <v>112</v>
+        <v>20</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2560,10 +2602,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>69</v>
+        <v>32</v>
       </c>
       <c r="F29" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2575,13 +2617,13 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="K29" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="L29" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="M29" t="s">
         <v>29</v>
@@ -2593,7 +2635,7 @@
         <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>68</v>
+        <v>123</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2616,10 +2658,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="F30" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2631,13 +2673,13 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>34</v>
+        <v>126</v>
       </c>
       <c r="K30" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="L30" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="M30" t="s">
         <v>29</v>
@@ -2649,7 +2691,7 @@
         <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>114</v>
+        <v>20</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2672,10 +2714,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F31" t="s">
-        <v>44</v>
+        <v>128</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2687,13 +2729,13 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>47</v>
+        <v>125</v>
       </c>
       <c r="K31" t="s">
-        <v>83</v>
+        <v>130</v>
       </c>
       <c r="L31" t="s">
-        <v>46</v>
+        <v>126</v>
       </c>
       <c r="M31" t="s">
         <v>29</v>
@@ -2705,7 +2747,7 @@
         <v>31</v>
       </c>
       <c r="R31" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="T31" t="n">
         <v>110.0</v>
@@ -2728,10 +2770,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2743,13 +2785,13 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>120</v>
+        <v>26</v>
       </c>
       <c r="K32" t="s">
-        <v>121</v>
+        <v>35</v>
       </c>
       <c r="L32" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
@@ -2758,13 +2800,13 @@
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="Q32" t="s">
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2787,10 +2829,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="F33" t="s">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2802,13 +2844,13 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="K33" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="L33" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="M33" t="s">
         <v>29</v>
@@ -2820,7 +2862,7 @@
         <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>98</v>
+        <v>36</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2843,10 +2885,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>63</v>
+        <v>103</v>
       </c>
       <c r="F34" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2858,13 +2900,13 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="K34" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="L34" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="M34" t="s">
         <v>29</v>
@@ -2876,7 +2918,7 @@
         <v>31</v>
       </c>
       <c r="R34" t="s">
-        <v>124</v>
+        <v>20</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2899,10 +2941,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>129</v>
+        <v>45</v>
       </c>
       <c r="F35" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2914,13 +2956,13 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="K35" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="L35" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="M35" t="s">
         <v>29</v>
@@ -2932,7 +2974,7 @@
         <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>20</v>
+        <v>134</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2955,10 +2997,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="F36" t="s">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -2970,13 +3012,13 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K36" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L36" t="s">
-        <v>28</v>
+        <v>102</v>
       </c>
       <c r="M36" t="s">
         <v>29</v>
@@ -2988,7 +3030,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>112</v>
+        <v>139</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -3011,10 +3053,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="F37" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3026,13 +3068,13 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>26</v>
+        <v>105</v>
       </c>
       <c r="K37" t="s">
-        <v>27</v>
+        <v>106</v>
       </c>
       <c r="L37" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
       <c r="M37" t="s">
         <v>29</v>
@@ -3041,13 +3083,13 @@
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="Q37" t="s">
         <v>31</v>
       </c>
       <c r="R37" t="s">
-        <v>98</v>
+        <v>20</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3070,10 +3112,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>43</v>
+        <v>86</v>
       </c>
       <c r="F38" t="s">
-        <v>47</v>
+        <v>141</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3085,13 +3127,13 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>44</v>
+        <v>142</v>
       </c>
       <c r="K38" t="s">
-        <v>45</v>
+        <v>143</v>
       </c>
       <c r="L38" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="M38" t="s">
         <v>29</v>
@@ -3126,10 +3168,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3141,13 +3183,13 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>138</v>
+        <v>26</v>
       </c>
       <c r="K39" t="s">
-        <v>139</v>
+        <v>27</v>
       </c>
       <c r="L39" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="M39" t="s">
         <v>29</v>
@@ -3159,7 +3201,7 @@
         <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3182,10 +3224,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="F40" t="s">
-        <v>70</v>
+        <v>148</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3197,13 +3239,13 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>71</v>
+        <v>149</v>
       </c>
       <c r="K40" t="s">
-        <v>72</v>
+        <v>150</v>
       </c>
       <c r="L40" t="s">
-        <v>73</v>
+        <v>151</v>
       </c>
       <c r="M40" t="s">
         <v>29</v>
@@ -3215,7 +3257,7 @@
         <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>68</v>
+        <v>147</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3238,11 +3280,11 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
+        <v>37</v>
+      </c>
+      <c r="F41" t="s">
         <v>38</v>
       </c>
-      <c r="F41" t="s">
-        <v>141</v>
-      </c>
       <c r="G41" t="s">
         <v>20</v>
       </c>
@@ -3253,13 +3295,13 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>142</v>
+        <v>39</v>
       </c>
       <c r="K41" t="s">
-        <v>143</v>
+        <v>40</v>
       </c>
       <c r="L41" t="s">
-        <v>144</v>
+        <v>41</v>
       </c>
       <c r="M41" t="s">
         <v>29</v>
@@ -3271,7 +3313,7 @@
         <v>31</v>
       </c>
       <c r="R41" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="T41" t="n">
         <v>110.0</v>
@@ -3294,10 +3336,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="F42" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3309,13 +3351,13 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>56</v>
+        <v>153</v>
       </c>
       <c r="K42" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="L42" t="s">
-        <v>58</v>
+        <v>155</v>
       </c>
       <c r="M42" t="s">
         <v>29</v>
@@ -3324,7 +3366,7 @@
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="Q42" t="s">
         <v>31</v>
@@ -3353,10 +3395,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
       <c r="F43" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3368,13 +3410,13 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="K43" t="s">
-        <v>28</v>
+        <v>106</v>
       </c>
       <c r="L43" t="s">
-        <v>61</v>
+        <v>107</v>
       </c>
       <c r="M43" t="s">
         <v>29</v>
@@ -3386,7 +3428,7 @@
         <v>31</v>
       </c>
       <c r="R43" t="s">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3409,10 +3451,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F44" t="s">
-        <v>70</v>
+        <v>158</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3424,13 +3466,13 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="K44" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="L44" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="M44" t="s">
         <v>29</v>
@@ -3442,7 +3484,7 @@
         <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>68</v>
+        <v>157</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3465,10 +3507,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>38</v>
+        <v>79</v>
       </c>
       <c r="F45" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3480,13 +3522,13 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="K45" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="L45" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="M45" t="s">
         <v>29</v>
@@ -3521,10 +3563,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="F46" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3536,13 +3578,13 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="K46" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="L46" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="M46" t="s">
         <v>29</v>
@@ -3554,7 +3596,7 @@
         <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>151</v>
+        <v>20</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3577,10 +3619,10 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>82</v>
+        <v>24</v>
       </c>
       <c r="F47" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G47" t="s">
         <v>20</v>
@@ -3607,13 +3649,13 @@
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="Q47" t="s">
         <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3636,10 +3678,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F48" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3651,13 +3693,13 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="K48" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="L48" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="M48" t="s">
         <v>29</v>
@@ -3669,7 +3711,7 @@
         <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3692,10 +3734,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>81</v>
+        <v>37</v>
       </c>
       <c r="F49" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3707,13 +3749,13 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="K49" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="L49" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="M49" t="s">
         <v>29</v>
@@ -3725,7 +3767,7 @@
         <v>31</v>
       </c>
       <c r="R49" t="s">
-        <v>152</v>
+        <v>36</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3748,10 +3790,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="F50" t="s">
-        <v>70</v>
+        <v>146</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3763,13 +3805,13 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="K50" t="s">
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="L50" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="M50" t="s">
         <v>29</v>
@@ -3781,7 +3823,7 @@
         <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>68</v>
+        <v>170</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3804,10 +3846,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F51" t="s">
-        <v>104</v>
+        <v>172</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3819,13 +3861,13 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="K51" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="L51" t="s">
-        <v>103</v>
+        <v>175</v>
       </c>
       <c r="M51" t="s">
         <v>29</v>
@@ -3837,7 +3879,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3848,7 +3890,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added $ to numbers
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="136">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,43 +83,109 @@
     <t>09030201</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Truck, Scooter, Bus&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Scooter$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Scooter, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Scooter$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Truck, Scooter, Bus</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
   </si>
   <si>
     <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
   </si>
   <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$9$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$7$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>$1250$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1251$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1249$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1252$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
   </si>
   <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
   </si>
   <si>
     <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
@@ -140,406 +206,217 @@
     <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 480$&lt;br&gt;No. of travellers using the Bicycle  $= 270$&lt;br&gt;No. of travellers using the Truck  $= 280$&lt;br&gt;No. of travellers using the Bus  $= 100$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$480 + 270 + 280 + 100 = 1130$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 480$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 270$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 100$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$480 + 270 + 280 + 100 = 1130$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 210$&lt;br&gt;No. of travellers using the Bus  $= 220$&lt;br&gt;No. of travellers using the Truck  $= 390$&lt;br&gt;No. of travellers using the Scooter  $= 640$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$210 + 220 + 390 + 640 = 1460$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 210$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 220$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 390$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 640$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$210 + 220 + 390 + 640 = 1460$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
   </si>
   <si>
-    <t>1130</t>
-  </si>
-  <si>
-    <t>1128</t>
-  </si>
-  <si>
-    <t>1132</t>
-  </si>
-  <si>
-    <t>1129</t>
+    <t>$1460$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1459$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1458$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1461$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 3$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 6$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$3 + 6 = 9$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3 + 6 = 9$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$11$ &lt;br&gt;</t>
   </si>
   <si>
     <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 270$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 280$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$270 + 280 = 550$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 270$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 280$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$270 + 280 = 550$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>550</t>
-  </si>
-  <si>
-    <t>548</t>
-  </si>
-  <si>
-    <t>551</t>
-  </si>
-  <si>
-    <t>549</t>
-  </si>
-  <si>
-    <t>Ans: Motorcycle, Bicycle, Truck, Bus&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bicycle$, $Truck$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bicycle, Truck, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bicycle$, $Truck$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle, Bicycle, Truck, Bus</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Ans: $5100$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 6600$&lt;br&gt;No. of travellers using the vehicle least $= 1500$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$6600 - 1500 = 5100$  is the answer.&lt;br&gt;#उत्तर : $5100$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6600$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1500$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$6600 - 1500 = 5100$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>$4$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $7$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 8$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$8 - 1 = 7$  is the answer.&lt;br&gt;#उत्तर : $7$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$8 - 1 = 7$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
   </si>
   <si>
-    <t>5100</t>
-  </si>
-  <si>
-    <t>5101</t>
-  </si>
-  <si>
-    <t>5099</t>
-  </si>
-  <si>
-    <t>5102</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bicycle $= 2700$&lt;br&gt;No. of travellers using the Truck  $= 1500$&lt;br&gt;No. of travellers using the Motorcycle  $= 6600$&lt;br&gt;No. of travellers using the Bus  $= 3800$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$2700 + 1500 + 6600 + 3800 = 14600$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bicycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 2700$&lt;br&gt;Truck या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 1500$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6600$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$2700 + 1500 + 6600 + 3800 = 14600$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>14600</t>
-  </si>
-  <si>
-    <t>14602</t>
-  </si>
-  <si>
-    <t>14599</t>
-  </si>
-  <si>
-    <t>14601</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?</t>
-  </si>
-  <si>
-    <t>13100</t>
-  </si>
-  <si>
-    <t>13101</t>
-  </si>
-  <si>
-    <t>13099</t>
-  </si>
-  <si>
-    <t>13102</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Truck, Motorcycle, Bus&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Motorcycle$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Motorcycle, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Motorcycle$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Truck, Motorcycle, Bus</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>8100</t>
-  </si>
-  <si>
-    <t>8101</t>
-  </si>
-  <si>
-    <t>8102</t>
-  </si>
-  <si>
-    <t>8098</t>
-  </si>
-  <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>77</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>79</t>
-  </si>
-  <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 37$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 56$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$37 + 56 = 93$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 37$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 56$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$37 + 56 = 93$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>93</t>
-  </si>
-  <si>
-    <t>91</t>
-  </si>
-  <si>
-    <t>94</t>
-  </si>
-  <si>
-    <t>95</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 4$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 5$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$4 + 5 = 9$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$4 + 5 = 9$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 6$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$6 - 1 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$6 - 1 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$3$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 2$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 7$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$2 + 7 = 9$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$2 + 7 = 9$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$39$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$37$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$38$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$40$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>Ans: Truck, Motorcycle, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Truck$, $Motorcycle$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Truck, Motorcycle, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Truck$, $Motorcycle$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck, Motorcycle, Bus, Scooter</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 1$&lt;br&gt;No. of travellers using the Motorcycle  $= 10$&lt;br&gt;No. of travellers using the Bus  $= 18$&lt;br&gt;No. of travellers using the Scooter  $= 38$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$1 + 10 + 18 + 38 = 67$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 10$&lt;br&gt;Bus या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 18$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 38$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$1 + 10 + 18 + 38 = 67$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$67$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$65$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$66$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$68$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>Ans: $6700$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 7200$&lt;br&gt;No. of travellers using the vehicle least $= 500$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$7200 - 500 = 6700$  is the answer.&lt;br&gt;#उत्तर : $6700$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7200$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 500$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$7200 - 500 = 6700$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>6700</t>
-  </si>
-  <si>
-    <t>6699</t>
-  </si>
-  <si>
-    <t>6702</t>
-  </si>
-  <si>
-    <t>6698</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 5300$&lt;br&gt;No. of travellers using the Bus  $= 4700$&lt;br&gt;No. of travellers using the Bicycle  $= 7200$&lt;br&gt;No. of travellers using the Truck  $= 500$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$5300 + 4700 + 7200 + 500 = 17700$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 5300$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 4700$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7200$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 500$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$5300 + 4700 + 7200 + 500 = 17700$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>17700</t>
-  </si>
-  <si>
-    <t>17698</t>
-  </si>
-  <si>
-    <t>17701</t>
-  </si>
-  <si>
-    <t>17702</t>
-  </si>
-  <si>
-    <t>17200</t>
-  </si>
-  <si>
-    <t>17198</t>
-  </si>
-  <si>
-    <t>17201</t>
-  </si>
-  <si>
-    <t>17199</t>
+    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 2$&lt;br&gt;No. of travellers using the Scooter  $= 2$&lt;br&gt;No. of travellers using the Truck  $= 9$&lt;br&gt;No. of travellers using the Motorcycle  $= 9$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$2 + 2 + 9 + 9 = 22$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;Scooter या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;Motorcycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$2 + 2 + 9 + 9 = 22$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 30$&lt;br&gt;No. of travellers using the Bus  $= 20$&lt;br&gt;No. of travellers using the Car  $= 76$&lt;br&gt;No. of travellers using the Truck  $= 11$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$30 + 20 + 76 + 11 = 137$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 30$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 20$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 76$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 11$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$30 + 20 + 76 + 11 = 137$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>137</t>
-  </si>
-  <si>
-    <t>138</t>
-  </si>
-  <si>
-    <t>139</t>
-  </si>
-  <si>
-    <t>135</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>$990$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$988$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$991$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$989$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 240$&lt;br&gt;No. of travellers using the Car  $= 110$&lt;br&gt;No. of travellers using the Bicycle  $= 870$&lt;br&gt;No. of travellers using the Scooter  $= 880$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$240 + 110 + 870 + 880 = 2100$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 110$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 870$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 880$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$240 + 110 + 870 + 880 = 2100$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2100$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2098$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2102$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2099$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
+  </si>
+  <si>
+    <t>Ans: $920$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 990$&lt;br&gt;No. of travellers using the vehicle least $= 70$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$990 - 70 = 920$  is the answer.&lt;br&gt;#उत्तर : $920$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 990$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 70$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$990 - 70 = 920$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$920$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$922$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$921$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$918$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 260$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 980$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$260 + 980 = 1240$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 260$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 980$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$260 + 980 = 1240$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1240$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1242$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1238$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1239$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Bus, Scooter, Truck&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bus$, $Scooter$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bus, Scooter, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bus$, $Scooter$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Bus, Scooter, Truck</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>11200</t>
-  </si>
-  <si>
-    <t>11201</t>
-  </si>
-  <si>
-    <t>11199</t>
-  </si>
-  <si>
-    <t>11202</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 4700$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 4700$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$4700 + 4700 = 9400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4700$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4700$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$4700 + 4700 = 9400$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>9400</t>
-  </si>
-  <si>
-    <t>9402</t>
-  </si>
-  <si>
-    <t>9398</t>
-  </si>
-  <si>
-    <t>9401</t>
-  </si>
-  <si>
-    <t>9800</t>
-  </si>
-  <si>
-    <t>9799</t>
-  </si>
-  <si>
-    <t>9798</t>
-  </si>
-  <si>
-    <t>9802</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Car, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Bicycle$, $Car$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Car, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Car$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Car, Bus, Scooter</t>
-  </si>
-  <si>
-    <t>20200</t>
-  </si>
-  <si>
-    <t>20198</t>
-  </si>
-  <si>
-    <t>20202</t>
-  </si>
-  <si>
-    <t>20199</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
-  </si>
-  <si>
-    <t>Ans: $880$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 910$&lt;br&gt;No. of travellers using the vehicle least $= 30$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$910 - 30 = 880$  is the answer.&lt;br&gt;#उत्तर : $880$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 910$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 30$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$910 - 30 = 880$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>880</t>
-  </si>
-  <si>
-    <t>879</t>
-  </si>
-  <si>
-    <t>881</t>
-  </si>
-  <si>
-    <t>882</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 290$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 830$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$290 + 830 = 1120$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 290$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 830$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$290 + 830 = 1120$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>1120</t>
-  </si>
-  <si>
-    <t>1118</t>
-  </si>
-  <si>
-    <t>1121</t>
-  </si>
-  <si>
-    <t>1122</t>
   </si>
   <si>
     <t>****</t>
@@ -1131,40 +1008,40 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R3" t="s">
         <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N3" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R3" t="s">
-        <v>23</v>
       </c>
       <c r="T3" t="n">
         <v>110.0</v>
@@ -1187,10 +1064,10 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1205,10 +1082,10 @@
         <v>26</v>
       </c>
       <c r="K4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L4" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="M4" t="s">
         <v>29</v>
@@ -1220,7 +1097,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1243,10 +1120,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1258,13 +1135,13 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="K5" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="L5" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="M5" t="s">
         <v>29</v>
@@ -1276,7 +1153,7 @@
         <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1302,7 +1179,7 @@
         <v>42</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1314,13 +1191,13 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>26</v>
+        <v>44</v>
       </c>
       <c r="K6" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="L6" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="M6" t="s">
         <v>29</v>
@@ -1332,7 +1209,7 @@
         <v>31</v>
       </c>
       <c r="R6" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1355,10 +1232,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1370,13 +1247,13 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="K7" t="s">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="L7" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="M7" t="s">
         <v>29</v>
@@ -1385,13 +1262,13 @@
         <v>4.0</v>
       </c>
       <c r="P7" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="Q7" t="s">
         <v>31</v>
       </c>
       <c r="R7" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="T7" t="n">
         <v>110.0</v>
@@ -1414,10 +1291,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1429,13 +1306,13 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="K8" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="L8" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="M8" t="s">
         <v>29</v>
@@ -1447,7 +1324,7 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1470,10 +1347,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1485,25 +1362,25 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="K9" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="L9" t="s">
+        <v>57</v>
+      </c>
+      <c r="M9" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>31</v>
+      </c>
+      <c r="R9" t="s">
         <v>54</v>
-      </c>
-      <c r="M9" t="s">
-        <v>29</v>
-      </c>
-      <c r="N9" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>31</v>
-      </c>
-      <c r="R9" t="s">
-        <v>20</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1526,10 +1403,10 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1541,25 +1418,25 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
+        <v>61</v>
+      </c>
+      <c r="K10" t="s">
+        <v>62</v>
+      </c>
+      <c r="L10" t="s">
+        <v>63</v>
+      </c>
+      <c r="M10" t="s">
+        <v>29</v>
+      </c>
+      <c r="N10" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>31</v>
+      </c>
+      <c r="R10" t="s">
         <v>58</v>
-      </c>
-      <c r="K10" t="s">
-        <v>59</v>
-      </c>
-      <c r="L10" t="s">
-        <v>60</v>
-      </c>
-      <c r="M10" t="s">
-        <v>29</v>
-      </c>
-      <c r="N10" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>31</v>
-      </c>
-      <c r="R10" t="s">
-        <v>55</v>
       </c>
       <c r="T10" t="n">
         <v>110.0</v>
@@ -1582,10 +1459,10 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G11" t="s">
         <v>20</v>
@@ -1597,25 +1474,25 @@
         <v>20</v>
       </c>
       <c r="J11" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" t="s">
+        <v>68</v>
+      </c>
+      <c r="L11" t="s">
+        <v>69</v>
+      </c>
+      <c r="M11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" t="s">
         <v>64</v>
-      </c>
-      <c r="K11" t="s">
-        <v>65</v>
-      </c>
-      <c r="L11" t="s">
-        <v>66</v>
-      </c>
-      <c r="M11" t="s">
-        <v>29</v>
-      </c>
-      <c r="N11" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>31</v>
-      </c>
-      <c r="R11" t="s">
-        <v>61</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1638,10 +1515,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1653,28 +1530,28 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" t="s">
+        <v>57</v>
+      </c>
+      <c r="M12" t="s">
+        <v>29</v>
+      </c>
+      <c r="N12" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P12" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>31</v>
+      </c>
+      <c r="R12" t="s">
         <v>70</v>
-      </c>
-      <c r="K12" t="s">
-        <v>71</v>
-      </c>
-      <c r="L12" t="s">
-        <v>72</v>
-      </c>
-      <c r="M12" t="s">
-        <v>29</v>
-      </c>
-      <c r="N12" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P12" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>31</v>
-      </c>
-      <c r="R12" t="s">
-        <v>67</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1697,28 +1574,28 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
+        <v>73</v>
+      </c>
+      <c r="F13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" t="s">
         <v>45</v>
       </c>
-      <c r="F13" t="s">
-        <v>75</v>
-      </c>
-      <c r="G13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" t="s">
-        <v>20</v>
-      </c>
-      <c r="J13" t="s">
-        <v>76</v>
-      </c>
-      <c r="K13" t="s">
-        <v>77</v>
-      </c>
       <c r="L13" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="M13" t="s">
         <v>29</v>
@@ -1730,7 +1607,7 @@
         <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1753,28 +1630,28 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" t="s">
+        <v>77</v>
+      </c>
+      <c r="K14" t="s">
+        <v>78</v>
+      </c>
+      <c r="L14" t="s">
         <v>79</v>
-      </c>
-      <c r="F14" t="s">
-        <v>80</v>
-      </c>
-      <c r="G14" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" t="s">
-        <v>81</v>
-      </c>
-      <c r="K14" t="s">
-        <v>82</v>
-      </c>
-      <c r="L14" t="s">
-        <v>83</v>
       </c>
       <c r="M14" t="s">
         <v>29</v>
@@ -1809,10 +1686,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="F15" t="s">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1824,13 +1701,13 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="L15" t="s">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="M15" t="s">
         <v>29</v>
@@ -1842,7 +1719,7 @@
         <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1865,10 +1742,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="F16" t="s">
-        <v>87</v>
+        <v>44</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1880,13 +1757,13 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="K16" t="s">
-        <v>89</v>
+        <v>43</v>
       </c>
       <c r="L16" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -1921,10 +1798,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>45</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1936,13 +1813,13 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K17" t="s">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="L17" t="s">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="M17" t="s">
         <v>29</v>
@@ -1951,7 +1828,7 @@
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="Q17" t="s">
         <v>31</v>
@@ -1980,10 +1857,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>73</v>
       </c>
       <c r="F18" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1995,13 +1872,13 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="K18" t="s">
-        <v>40</v>
+        <v>74</v>
       </c>
       <c r="L18" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="M18" t="s">
         <v>29</v>
@@ -2013,7 +1890,7 @@
         <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>36</v>
+        <v>83</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -2036,10 +1913,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="F19" t="s">
-        <v>25</v>
+        <v>78</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -2051,13 +1928,13 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="K19" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="L19" t="s">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="M19" t="s">
         <v>29</v>
@@ -2069,7 +1946,7 @@
         <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2092,10 +1969,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="F20" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2107,13 +1984,13 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="K20" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="L20" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="M20" t="s">
         <v>29</v>
@@ -2125,7 +2002,7 @@
         <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2148,10 +2025,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="F21" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2163,13 +2040,13 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="K21" t="s">
-        <v>35</v>
+        <v>89</v>
       </c>
       <c r="L21" t="s">
-        <v>25</v>
+        <v>90</v>
       </c>
       <c r="M21" t="s">
         <v>29</v>
@@ -2181,7 +2058,7 @@
         <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>101</v>
+        <v>20</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2204,10 +2081,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>103</v>
+        <v>41</v>
       </c>
       <c r="F22" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2219,13 +2096,13 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="K22" t="s">
-        <v>106</v>
+        <v>27</v>
       </c>
       <c r="L22" t="s">
-        <v>107</v>
+        <v>28</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -2234,13 +2111,13 @@
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="Q22" t="s">
         <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2263,10 +2140,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F23" t="s">
-        <v>110</v>
+        <v>44</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2278,13 +2155,13 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>111</v>
+        <v>74</v>
       </c>
       <c r="K23" t="s">
-        <v>112</v>
+        <v>45</v>
       </c>
       <c r="L23" t="s">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="M23" t="s">
         <v>29</v>
@@ -2296,7 +2173,7 @@
         <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2319,10 +2196,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="F24" t="s">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2334,13 +2211,13 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>116</v>
+        <v>61</v>
       </c>
       <c r="K24" t="s">
-        <v>117</v>
+        <v>62</v>
       </c>
       <c r="L24" t="s">
-        <v>118</v>
+        <v>63</v>
       </c>
       <c r="M24" t="s">
         <v>29</v>
@@ -2352,7 +2229,7 @@
         <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2375,28 +2252,28 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" t="s">
+        <v>76</v>
+      </c>
+      <c r="G25" t="s">
+        <v>20</v>
+      </c>
+      <c r="H25" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" t="s">
+        <v>20</v>
+      </c>
+      <c r="J25" t="s">
+        <v>85</v>
+      </c>
+      <c r="K25" t="s">
         <v>79</v>
       </c>
-      <c r="F25" t="s">
-        <v>119</v>
-      </c>
-      <c r="G25" t="s">
-        <v>20</v>
-      </c>
-      <c r="H25" t="s">
-        <v>20</v>
-      </c>
-      <c r="I25" t="s">
-        <v>20</v>
-      </c>
-      <c r="J25" t="s">
-        <v>120</v>
-      </c>
-      <c r="K25" t="s">
-        <v>121</v>
-      </c>
       <c r="L25" t="s">
-        <v>122</v>
+        <v>78</v>
       </c>
       <c r="M25" t="s">
         <v>29</v>
@@ -2431,10 +2308,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>32</v>
+        <v>86</v>
       </c>
       <c r="F26" t="s">
-        <v>26</v>
+        <v>87</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2446,13 +2323,13 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>27</v>
+        <v>88</v>
       </c>
       <c r="K26" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="L26" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="M26" t="s">
         <v>29</v>
@@ -2464,7 +2341,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>123</v>
+        <v>20</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2487,10 +2364,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F27" t="s">
-        <v>38</v>
+        <v>94</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2502,13 +2379,13 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>39</v>
+        <v>95</v>
       </c>
       <c r="K27" t="s">
-        <v>40</v>
+        <v>96</v>
       </c>
       <c r="L27" t="s">
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="M27" t="s">
         <v>29</v>
@@ -2517,13 +2394,13 @@
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="Q27" t="s">
         <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2546,10 +2423,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F28" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2561,25 +2438,25 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="K28" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="L28" t="s">
+        <v>57</v>
+      </c>
+      <c r="M28" t="s">
+        <v>29</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>31</v>
+      </c>
+      <c r="R28" t="s">
         <v>54</v>
-      </c>
-      <c r="M28" t="s">
-        <v>29</v>
-      </c>
-      <c r="N28" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>31</v>
-      </c>
-      <c r="R28" t="s">
-        <v>20</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2602,29 +2479,29 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F29" t="s">
+        <v>57</v>
+      </c>
+      <c r="G29" t="s">
+        <v>20</v>
+      </c>
+      <c r="H29" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29" t="s">
+        <v>20</v>
+      </c>
+      <c r="J29" t="s">
         <v>26</v>
       </c>
-      <c r="G29" t="s">
-        <v>20</v>
-      </c>
-      <c r="H29" t="s">
-        <v>20</v>
-      </c>
-      <c r="I29" t="s">
-        <v>20</v>
-      </c>
-      <c r="J29" t="s">
+      <c r="K29" t="s">
         <v>27</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>28</v>
       </c>
-      <c r="L29" t="s">
-        <v>102</v>
-      </c>
       <c r="M29" t="s">
         <v>29</v>
       </c>
@@ -2635,7 +2512,7 @@
         <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>123</v>
+        <v>91</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2658,10 +2535,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="F30" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2673,13 +2550,13 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="K30" t="s">
-        <v>127</v>
+        <v>36</v>
       </c>
       <c r="L30" t="s">
-        <v>128</v>
+        <v>37</v>
       </c>
       <c r="M30" t="s">
         <v>29</v>
@@ -2691,7 +2568,7 @@
         <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2714,10 +2591,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="F31" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2729,13 +2606,13 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
       <c r="K31" t="s">
-        <v>130</v>
+        <v>104</v>
       </c>
       <c r="L31" t="s">
-        <v>126</v>
+        <v>105</v>
       </c>
       <c r="M31" t="s">
         <v>29</v>
@@ -2747,7 +2624,7 @@
         <v>31</v>
       </c>
       <c r="R31" t="s">
-        <v>129</v>
+        <v>101</v>
       </c>
       <c r="T31" t="n">
         <v>110.0</v>
@@ -2770,10 +2647,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="F32" t="s">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2785,13 +2662,13 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="K32" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="L32" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
@@ -2800,13 +2677,13 @@
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="Q32" t="s">
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>131</v>
+        <v>58</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2829,10 +2706,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F33" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2844,13 +2721,13 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="K33" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="L33" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="M33" t="s">
         <v>29</v>
@@ -2862,7 +2739,7 @@
         <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2885,10 +2762,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="F34" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2900,13 +2777,13 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>105</v>
+        <v>88</v>
       </c>
       <c r="K34" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="L34" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="M34" t="s">
         <v>29</v>
@@ -2941,10 +2818,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="F35" t="s">
-        <v>135</v>
+        <v>26</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2956,13 +2833,13 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>136</v>
+        <v>25</v>
       </c>
       <c r="K35" t="s">
-        <v>137</v>
+        <v>40</v>
       </c>
       <c r="L35" t="s">
-        <v>138</v>
+        <v>57</v>
       </c>
       <c r="M35" t="s">
         <v>29</v>
@@ -2974,7 +2851,7 @@
         <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>134</v>
+        <v>109</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2997,29 +2874,29 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="F36" t="s">
+        <v>57</v>
+      </c>
+      <c r="G36" t="s">
+        <v>20</v>
+      </c>
+      <c r="H36" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" t="s">
+        <v>20</v>
+      </c>
+      <c r="J36" t="s">
         <v>26</v>
       </c>
-      <c r="G36" t="s">
-        <v>20</v>
-      </c>
-      <c r="H36" t="s">
-        <v>20</v>
-      </c>
-      <c r="I36" t="s">
-        <v>20</v>
-      </c>
-      <c r="J36" t="s">
+      <c r="K36" t="s">
         <v>27</v>
       </c>
-      <c r="K36" t="s">
+      <c r="L36" t="s">
         <v>28</v>
       </c>
-      <c r="L36" t="s">
-        <v>102</v>
-      </c>
       <c r="M36" t="s">
         <v>29</v>
       </c>
@@ -3030,7 +2907,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -3053,10 +2930,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="F37" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3068,13 +2945,13 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="K37" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="L37" t="s">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="M37" t="s">
         <v>29</v>
@@ -3083,13 +2960,13 @@
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="Q37" t="s">
         <v>31</v>
       </c>
       <c r="R37" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3112,10 +2989,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>86</v>
+        <v>42</v>
       </c>
       <c r="F38" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3127,13 +3004,13 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="K38" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="L38" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
       <c r="M38" t="s">
         <v>29</v>
@@ -3168,10 +3045,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="F39" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3183,13 +3060,13 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="K39" t="s">
-        <v>27</v>
+        <v>118</v>
       </c>
       <c r="L39" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="M39" t="s">
         <v>29</v>
@@ -3201,7 +3078,7 @@
         <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3224,11 +3101,11 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
+        <v>55</v>
+      </c>
+      <c r="F40" t="s">
         <v>56</v>
       </c>
-      <c r="F40" t="s">
-        <v>148</v>
-      </c>
       <c r="G40" t="s">
         <v>20</v>
       </c>
@@ -3239,13 +3116,13 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>149</v>
+        <v>26</v>
       </c>
       <c r="K40" t="s">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="L40" t="s">
-        <v>151</v>
+        <v>57</v>
       </c>
       <c r="M40" t="s">
         <v>29</v>
@@ -3257,7 +3134,7 @@
         <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>147</v>
+        <v>54</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3280,10 +3157,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F41" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3295,13 +3172,13 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="K41" t="s">
         <v>40</v>
       </c>
       <c r="L41" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="M41" t="s">
         <v>29</v>
@@ -3313,7 +3190,7 @@
         <v>31</v>
       </c>
       <c r="R41" t="s">
-        <v>36</v>
+        <v>109</v>
       </c>
       <c r="T41" t="n">
         <v>110.0</v>
@@ -3336,10 +3213,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>86</v>
+        <v>41</v>
       </c>
       <c r="F42" t="s">
-        <v>152</v>
+        <v>27</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3351,13 +3228,13 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>153</v>
+        <v>26</v>
       </c>
       <c r="K42" t="s">
-        <v>154</v>
+        <v>25</v>
       </c>
       <c r="L42" t="s">
-        <v>155</v>
+        <v>40</v>
       </c>
       <c r="M42" t="s">
         <v>29</v>
@@ -3366,13 +3243,13 @@
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
       <c r="Q42" t="s">
         <v>31</v>
       </c>
       <c r="R42" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3395,10 +3272,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>103</v>
+        <v>81</v>
       </c>
       <c r="F43" t="s">
-        <v>104</v>
+        <v>122</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3410,13 +3287,13 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="K43" t="s">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="L43" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="M43" t="s">
         <v>29</v>
@@ -3428,7 +3305,7 @@
         <v>31</v>
       </c>
       <c r="R43" t="s">
-        <v>20</v>
+        <v>121</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3451,10 +3328,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="F44" t="s">
-        <v>158</v>
+        <v>108</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3466,13 +3343,13 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="K44" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="L44" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="M44" t="s">
         <v>29</v>
@@ -3484,7 +3361,7 @@
         <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>157</v>
+        <v>20</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3507,10 +3384,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F45" t="s">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3522,13 +3399,13 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>160</v>
+        <v>128</v>
       </c>
       <c r="K45" t="s">
-        <v>161</v>
+        <v>129</v>
       </c>
       <c r="L45" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="M45" t="s">
         <v>29</v>
@@ -3540,7 +3417,7 @@
         <v>31</v>
       </c>
       <c r="R45" t="s">
-        <v>20</v>
+        <v>126</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3563,10 +3440,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="F46" t="s">
-        <v>51</v>
+        <v>132</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3578,13 +3455,13 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="K46" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="L46" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="M46" t="s">
         <v>29</v>
@@ -3596,7 +3473,7 @@
         <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>20</v>
+        <v>131</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3619,10 +3496,10 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="F47" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="G47" t="s">
         <v>20</v>
@@ -3637,10 +3514,10 @@
         <v>26</v>
       </c>
       <c r="K47" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L47" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="M47" t="s">
         <v>29</v>
@@ -3649,13 +3526,13 @@
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>164</v>
+        <v>133</v>
       </c>
       <c r="Q47" t="s">
         <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>163</v>
+        <v>53</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3678,10 +3555,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="F48" t="s">
-        <v>166</v>
+        <v>27</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3693,13 +3570,13 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>167</v>
+        <v>26</v>
       </c>
       <c r="K48" t="s">
-        <v>168</v>
+        <v>25</v>
       </c>
       <c r="L48" t="s">
-        <v>169</v>
+        <v>40</v>
       </c>
       <c r="M48" t="s">
         <v>29</v>
@@ -3711,7 +3588,7 @@
         <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>165</v>
+        <v>53</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3734,10 +3611,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="F49" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3749,13 +3626,13 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="K49" t="s">
-        <v>40</v>
+        <v>78</v>
       </c>
       <c r="L49" t="s">
-        <v>41</v>
+        <v>77</v>
       </c>
       <c r="M49" t="s">
         <v>29</v>
@@ -3767,7 +3644,7 @@
         <v>31</v>
       </c>
       <c r="R49" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3790,10 +3667,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="F50" t="s">
-        <v>146</v>
+        <v>60</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3805,13 +3682,13 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
       <c r="K50" t="s">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="L50" t="s">
-        <v>102</v>
+        <v>63</v>
       </c>
       <c r="M50" t="s">
         <v>29</v>
@@ -3823,7 +3700,7 @@
         <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>170</v>
+        <v>58</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3846,10 +3723,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="F51" t="s">
-        <v>172</v>
+        <v>26</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3861,13 +3738,13 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>173</v>
+        <v>25</v>
       </c>
       <c r="K51" t="s">
-        <v>174</v>
+        <v>40</v>
       </c>
       <c r="L51" t="s">
-        <v>175</v>
+        <v>57</v>
       </c>
       <c r="M51" t="s">
         <v>29</v>
@@ -3879,7 +3756,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>171</v>
+        <v>134</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3890,7 +3767,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>176</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
marathi translation for array
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="179">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,64 +83,424 @@
     <t>09030201</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 36$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 51$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$36 + 51 = 87$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 51$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$36 + 51 = 87$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$87$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$89$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$85$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$88$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
   </si>
   <si>
     <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
   </si>
   <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of travelers by different means.</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $38$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 61$&lt;br&gt;No. of travellers using the vehicle least $= 23$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$61 - 23 = 38$  is the answer.&lt;br&gt;#उत्तर : $38$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 23$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$61 - 23 = 38$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$38$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$40$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$39$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$37$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 3300$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 7400$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$3300 + 7400 = 10700$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3300$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7400$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3300 + 7400 = 10700$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10700$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10698$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10699$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10701$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 1600$&lt;br&gt;No. of travellers using the Bus  $= 3300$&lt;br&gt;No. of travellers using the Bicycle  $= 7400$&lt;br&gt;No. of travellers using the Scooter  $= 8100$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$1600 + 3300 + 7400 + 8100 = 20400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 1600$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 3300$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7400$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 8100$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$1600 + 3300 + 7400 + 8100 = 20400$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$20400$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$20398$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$20401$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$20402$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $92$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 98$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$98 - 6 = 92$  is the answer.&lt;br&gt;#उत्तर : $92$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$98 - 6 = 92$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$92$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$94$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$90$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$91$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$4$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$3$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $62$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 95$&lt;br&gt;No. of travellers using the vehicle least $= 33$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$95 - 33 = 62$  is the answer.&lt;br&gt;#उत्तर : $62$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 95$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 33$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$95 - 33 = 62$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$62$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$61$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$63$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$64$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$128$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$130$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$127$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$129$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Bus, Scooter, Bicycle&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bus$, $Scooter$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bus, Scooter, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bus$, $Scooter$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Bus, Scooter, Bicycle&lt;br&gt;#मोटरसायकल, बस, दुचाकी, सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle</t>
+  </si>
+  <si>
+    <t>$700$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$702$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$698$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$699$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 230$&lt;br&gt;No. of travellers using the Bus  $= 460$&lt;br&gt;No. of travellers using the Bicycle  $= 550$&lt;br&gt;No. of travellers using the Truck  $= 150$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$230 + 460 + 550 + 150 = 1390$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 230$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 460$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 550$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 150$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$230 + 460 + 550 + 150 = 1390$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1390$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1391$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1389$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1392$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 230$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 460$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$230 + 460 = 690$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 230$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 460$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$230 + 460 = 690$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$690$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$689$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$692$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$688$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>$1240$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1239$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1242$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1238$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
   </si>
   <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Truck, Scooter, Bus&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Scooter$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Scooter, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Scooter$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Truck, Scooter, Bus</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+    <t>$136$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$135$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$137$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$138$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 86$&lt;br&gt;No. of travellers using the Car  $= 83$&lt;br&gt;No. of travellers using the Scooter  $= 66$&lt;br&gt;No. of travellers using the Bus  $= 50$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$86 + 83 + 66 + 50 = 285$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 86$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 66$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 50$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$86 + 83 + 66 + 50 = 285$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$285$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$284$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$283$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$287$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 66$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 83$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$66 + 83 = 149$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 66$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$66 + 83 = 149$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$149$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$150$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$147$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$151$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $6$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9$&lt;br&gt;No. of travellers using the vehicle least $= 3$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9 - 3 = 6$  is the answer.&lt;br&gt;#उत्तर : $6$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9 - 3 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$7$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Truck, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Truck, Bus, Scooter&lt;br&gt;#सायकल, ट्रक, बस, दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 6$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 7$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$6 + 7 = 13$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$6 + 7 = 13$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$13$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$11$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$15$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Scooter, Motorcycle, Bicycle, Truck&lt;br&gt;From the given graph we can see that, $Scooter$, $Motorcycle$, $Bicycle$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Motorcycle, Bicycle, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Motorcycle$, $Bicycle$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter, Motorcycle, Bicycle, Truck&lt;br&gt;#दुचाकी, मोटरसायकल, सायकल, ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 7$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 9$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$7 + 9 = 16$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$7 + 9 = 16$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$16$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$18$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$17$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$14$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 3$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 4$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$3 + 4 = 7$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3 + 4 = 7$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>$8$ &lt;br&gt;</t>
@@ -149,274 +509,43 @@
     <t>$9$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>$7$ &lt;br&gt;</t>
-  </si>
-  <si>
     <t>$10$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>How much is the total of travellers for top 3 values?</t>
-  </si>
-  <si>
-    <t>$1250$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1251$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1249$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1252$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of travelers by different means.</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 210$&lt;br&gt;No. of travellers using the Bus  $= 220$&lt;br&gt;No. of travellers using the Truck  $= 390$&lt;br&gt;No. of travellers using the Scooter  $= 640$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$210 + 220 + 390 + 640 = 1460$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 210$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 220$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 390$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 640$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$210 + 220 + 390 + 640 = 1460$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1460$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1459$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1458$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1461$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 3$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 6$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$3 + 6 = 9$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3 + 6 = 9$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$11$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$4$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $7$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 8$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$8 - 1 = 7$  is the answer.&lt;br&gt;#उत्तर : $7$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$8 - 1 = 7$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 4$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 5$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$4 + 5 = 9$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$4 + 5 = 9$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 6$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$6 - 1 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$6 - 1 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$3$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 2$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 7$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$2 + 7 = 9$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$2 + 7 = 9$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$39$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$37$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$38$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$40$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>Ans: Truck, Motorcycle, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Truck$, $Motorcycle$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Truck, Motorcycle, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Truck$, $Motorcycle$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck, Motorcycle, Bus, Scooter</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 1$&lt;br&gt;No. of travellers using the Motorcycle  $= 10$&lt;br&gt;No. of travellers using the Bus  $= 18$&lt;br&gt;No. of travellers using the Scooter  $= 38$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$1 + 10 + 18 + 38 = 67$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 10$&lt;br&gt;Bus या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 18$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 38$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$1 + 10 + 18 + 38 = 67$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
+  </si>
+  <si>
+    <t>Ans: $67$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 73$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$73 - 6 = 67$  is the answer.&lt;br&gt;#उत्तर : $67$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 73$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$73 - 6 = 67$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>$67$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>$65$ &lt;br&gt;</t>
-  </si>
-  <si>
     <t>$66$ &lt;br&gt;</t>
   </si>
   <si>
+    <t>$69$ &lt;br&gt;</t>
+  </si>
+  <si>
     <t>$68$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>$990$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$988$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$991$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$989$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 240$&lt;br&gt;No. of travellers using the Car  $= 110$&lt;br&gt;No. of travellers using the Bicycle  $= 870$&lt;br&gt;No. of travellers using the Scooter  $= 880$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$240 + 110 + 870 + 880 = 2100$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 240$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 110$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 870$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 880$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$240 + 110 + 870 + 880 = 2100$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2100$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2098$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2102$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2099$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>Ans: $920$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 990$&lt;br&gt;No. of travellers using the vehicle least $= 70$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$990 - 70 = 920$  is the answer.&lt;br&gt;#उत्तर : $920$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 990$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 70$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$990 - 70 = 920$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$920$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$922$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$921$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$918$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 260$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 980$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$260 + 980 = 1240$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 260$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 980$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$260 + 980 = 1240$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1240$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1242$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1238$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1239$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Motorcycle, Bus, Scooter, Truck&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bus$, $Scooter$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bus, Scooter, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bus$, $Scooter$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle, Bus, Scooter, Truck</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>$79$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$77$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$81$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$80$ &lt;br&gt;</t>
   </si>
   <si>
     <t>****</t>
@@ -857,7 +986,7 @@
     <col min="3" max="3" width="12.4375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.66015625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="193.7734375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="63.5" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="67.39453125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="16.42578125" customWidth="true" bestFit="true"/>
@@ -1064,10 +1193,10 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1079,13 +1208,13 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K4" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="L4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="M4" t="s">
         <v>29</v>
@@ -1097,7 +1226,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1120,11 +1249,11 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" t="s">
         <v>41</v>
       </c>
-      <c r="F5" t="s">
-        <v>25</v>
-      </c>
       <c r="G5" t="s">
         <v>20</v>
       </c>
@@ -1135,13 +1264,13 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="K5" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="L5" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="M5" t="s">
         <v>29</v>
@@ -1153,7 +1282,7 @@
         <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1176,10 +1305,10 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1191,25 +1320,25 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="K6" t="s">
+        <v>49</v>
+      </c>
+      <c r="L6" t="s">
+        <v>50</v>
+      </c>
+      <c r="M6" t="s">
+        <v>29</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6" t="s">
         <v>45</v>
-      </c>
-      <c r="L6" t="s">
-        <v>46</v>
-      </c>
-      <c r="M6" t="s">
-        <v>29</v>
-      </c>
-      <c r="N6" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>31</v>
-      </c>
-      <c r="R6" t="s">
-        <v>20</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1232,10 +1361,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1247,28 +1376,28 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="K7" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="L7" t="s">
+        <v>55</v>
+      </c>
+      <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P7" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>31</v>
+      </c>
+      <c r="R7" t="s">
         <v>51</v>
-      </c>
-      <c r="M7" t="s">
-        <v>29</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P7" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>31</v>
-      </c>
-      <c r="R7" t="s">
-        <v>20</v>
       </c>
       <c r="T7" t="n">
         <v>110.0</v>
@@ -1291,10 +1420,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F8" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1306,13 +1435,13 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="K8" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="L8" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="M8" t="s">
         <v>29</v>
@@ -1324,7 +1453,7 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1347,10 +1476,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1362,13 +1491,13 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="K9" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="L9" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="M9" t="s">
         <v>29</v>
@@ -1380,7 +1509,7 @@
         <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1436,7 +1565,7 @@
         <v>31</v>
       </c>
       <c r="R10" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="T10" t="n">
         <v>110.0</v>
@@ -1515,10 +1644,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1530,13 +1659,13 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="K12" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="L12" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="M12" t="s">
         <v>29</v>
@@ -1545,7 +1674,7 @@
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="Q12" t="s">
         <v>31</v>
@@ -1574,10 +1703,10 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F13" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="G13" t="s">
         <v>20</v>
@@ -1589,13 +1718,13 @@
         <v>20</v>
       </c>
       <c r="J13" t="s">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="K13" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="L13" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="M13" t="s">
         <v>29</v>
@@ -1607,7 +1736,7 @@
         <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1630,40 +1759,40 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F14" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H14" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" t="s">
+        <v>35</v>
+      </c>
+      <c r="K14" t="s">
+        <v>36</v>
+      </c>
+      <c r="L14" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" t="s">
+        <v>29</v>
+      </c>
+      <c r="N14" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>31</v>
+      </c>
+      <c r="R14" t="s">
         <v>76</v>
-      </c>
-      <c r="G14" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" t="s">
-        <v>20</v>
-      </c>
-      <c r="J14" t="s">
-        <v>77</v>
-      </c>
-      <c r="K14" t="s">
-        <v>78</v>
-      </c>
-      <c r="L14" t="s">
-        <v>79</v>
-      </c>
-      <c r="M14" t="s">
-        <v>29</v>
-      </c>
-      <c r="N14" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>31</v>
-      </c>
-      <c r="R14" t="s">
-        <v>20</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1686,10 +1815,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1701,10 +1830,10 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="K15" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="L15" t="s">
         <v>44</v>
@@ -1719,7 +1848,7 @@
         <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>80</v>
+        <v>39</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1742,10 +1871,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>42</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1757,13 +1886,13 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="K16" t="s">
-        <v>43</v>
+        <v>82</v>
       </c>
       <c r="L16" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -1798,10 +1927,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F17" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1813,13 +1942,13 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="K17" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
       <c r="L17" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="M17" t="s">
         <v>29</v>
@@ -1828,13 +1957,13 @@
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="Q17" t="s">
         <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>20</v>
+        <v>84</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1857,10 +1986,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="F18" t="s">
-        <v>44</v>
+        <v>91</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1872,13 +2001,13 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="K18" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="L18" t="s">
-        <v>45</v>
+        <v>94</v>
       </c>
       <c r="M18" t="s">
         <v>29</v>
@@ -1890,7 +2019,7 @@
         <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -1913,10 +2042,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F19" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -1928,13 +2057,13 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K19" t="s">
-        <v>85</v>
+        <v>36</v>
       </c>
       <c r="L19" t="s">
-        <v>76</v>
+        <v>58</v>
       </c>
       <c r="M19" t="s">
         <v>29</v>
@@ -1946,7 +2075,7 @@
         <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -1969,10 +2098,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F20" t="s">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -1984,13 +2113,13 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="K20" t="s">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="L20" t="s">
-        <v>85</v>
+        <v>44</v>
       </c>
       <c r="M20" t="s">
         <v>29</v>
@@ -2002,7 +2131,7 @@
         <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2025,10 +2154,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="F21" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2040,13 +2169,13 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="K21" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="L21" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="M21" t="s">
         <v>29</v>
@@ -2058,7 +2187,7 @@
         <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2081,10 +2210,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>41</v>
+        <v>90</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>103</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2096,13 +2225,13 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
       <c r="K22" t="s">
-        <v>27</v>
+        <v>105</v>
       </c>
       <c r="L22" t="s">
-        <v>28</v>
+        <v>106</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -2111,13 +2240,13 @@
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="Q22" t="s">
         <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>91</v>
+        <v>20</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2140,10 +2269,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F23" t="s">
-        <v>44</v>
+        <v>109</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2155,13 +2284,13 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="K23" t="s">
-        <v>45</v>
+        <v>111</v>
       </c>
       <c r="L23" t="s">
-        <v>43</v>
+        <v>112</v>
       </c>
       <c r="M23" t="s">
         <v>29</v>
@@ -2173,7 +2302,7 @@
         <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2196,10 +2325,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="F24" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2211,13 +2340,13 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>61</v>
+        <v>115</v>
       </c>
       <c r="K24" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="L24" t="s">
-        <v>63</v>
+        <v>117</v>
       </c>
       <c r="M24" t="s">
         <v>29</v>
@@ -2229,7 +2358,7 @@
         <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>58</v>
+        <v>113</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2252,10 +2381,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>75</v>
+        <v>118</v>
       </c>
       <c r="F25" t="s">
-        <v>76</v>
+        <v>119</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2267,13 +2396,13 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="K25" t="s">
-        <v>79</v>
+        <v>121</v>
       </c>
       <c r="L25" t="s">
-        <v>78</v>
+        <v>122</v>
       </c>
       <c r="M25" t="s">
         <v>29</v>
@@ -2308,10 +2437,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="F26" t="s">
-        <v>87</v>
+        <v>58</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2323,13 +2452,13 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="K26" t="s">
-        <v>89</v>
+        <v>124</v>
       </c>
       <c r="L26" t="s">
-        <v>90</v>
+        <v>34</v>
       </c>
       <c r="M26" t="s">
         <v>29</v>
@@ -2341,7 +2470,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2364,10 +2493,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="F27" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2379,13 +2508,13 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>95</v>
+        <v>126</v>
       </c>
       <c r="K27" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
       <c r="L27" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="M27" t="s">
         <v>29</v>
@@ -2394,7 +2523,7 @@
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="Q27" t="s">
         <v>31</v>
@@ -2423,10 +2552,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F28" t="s">
-        <v>56</v>
+        <v>131</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2438,13 +2567,13 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>26</v>
+        <v>132</v>
       </c>
       <c r="K28" t="s">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="L28" t="s">
-        <v>57</v>
+        <v>134</v>
       </c>
       <c r="M28" t="s">
         <v>29</v>
@@ -2456,7 +2585,7 @@
         <v>31</v>
       </c>
       <c r="R28" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2482,7 +2611,7 @@
         <v>24</v>
       </c>
       <c r="F29" t="s">
-        <v>57</v>
+        <v>136</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2494,13 +2623,13 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>26</v>
+        <v>137</v>
       </c>
       <c r="K29" t="s">
-        <v>27</v>
+        <v>138</v>
       </c>
       <c r="L29" t="s">
-        <v>28</v>
+        <v>139</v>
       </c>
       <c r="M29" t="s">
         <v>29</v>
@@ -2512,7 +2641,7 @@
         <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>91</v>
+        <v>135</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2538,7 +2667,7 @@
         <v>33</v>
       </c>
       <c r="F30" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2553,10 +2682,10 @@
         <v>35</v>
       </c>
       <c r="K30" t="s">
-        <v>36</v>
+        <v>124</v>
       </c>
       <c r="L30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="M30" t="s">
         <v>29</v>
@@ -2568,7 +2697,7 @@
         <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2591,10 +2720,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="F31" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2606,13 +2735,13 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="K31" t="s">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="L31" t="s">
-        <v>105</v>
+        <v>34</v>
       </c>
       <c r="M31" t="s">
         <v>29</v>
@@ -2624,7 +2753,7 @@
         <v>31</v>
       </c>
       <c r="R31" t="s">
-        <v>101</v>
+        <v>140</v>
       </c>
       <c r="T31" t="n">
         <v>110.0</v>
@@ -2647,10 +2776,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="F32" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2662,13 +2791,13 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="K32" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="L32" t="s">
-        <v>63</v>
+        <v>142</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
@@ -2677,13 +2806,13 @@
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>106</v>
+        <v>143</v>
       </c>
       <c r="Q32" t="s">
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>58</v>
+        <v>141</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2706,10 +2835,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>39</v>
+        <v>98</v>
       </c>
       <c r="F33" t="s">
-        <v>57</v>
+        <v>145</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2721,13 +2850,13 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>26</v>
+        <v>100</v>
       </c>
       <c r="K33" t="s">
-        <v>27</v>
+        <v>101</v>
       </c>
       <c r="L33" t="s">
-        <v>28</v>
+        <v>102</v>
       </c>
       <c r="M33" t="s">
         <v>29</v>
@@ -2739,7 +2868,7 @@
         <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>107</v>
+        <v>144</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2762,10 +2891,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="F34" t="s">
-        <v>108</v>
+        <v>147</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2777,13 +2906,13 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>88</v>
+        <v>148</v>
       </c>
       <c r="K34" t="s">
-        <v>89</v>
+        <v>149</v>
       </c>
       <c r="L34" t="s">
-        <v>90</v>
+        <v>150</v>
       </c>
       <c r="M34" t="s">
         <v>29</v>
@@ -2795,7 +2924,7 @@
         <v>31</v>
       </c>
       <c r="R34" t="s">
-        <v>20</v>
+        <v>146</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2818,10 +2947,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="F35" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2833,13 +2962,13 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>25</v>
+        <v>151</v>
       </c>
       <c r="K35" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
       <c r="L35" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="M35" t="s">
         <v>29</v>
@@ -2851,7 +2980,7 @@
         <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>109</v>
+        <v>20</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2874,10 +3003,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="F36" t="s">
-        <v>57</v>
+        <v>96</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -2889,13 +3018,13 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K36" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="L36" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="M36" t="s">
         <v>29</v>
@@ -2907,7 +3036,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -2930,10 +3059,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>59</v>
+        <v>98</v>
       </c>
       <c r="F37" t="s">
-        <v>60</v>
+        <v>153</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -2945,13 +3074,13 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>61</v>
+        <v>100</v>
       </c>
       <c r="K37" t="s">
-        <v>62</v>
+        <v>101</v>
       </c>
       <c r="L37" t="s">
-        <v>63</v>
+        <v>102</v>
       </c>
       <c r="M37" t="s">
         <v>29</v>
@@ -2960,13 +3089,13 @@
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>110</v>
+        <v>154</v>
       </c>
       <c r="Q37" t="s">
         <v>31</v>
       </c>
       <c r="R37" t="s">
-        <v>58</v>
+        <v>152</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -2989,10 +3118,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F38" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3004,13 +3133,13 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>112</v>
+        <v>35</v>
       </c>
       <c r="K38" t="s">
-        <v>113</v>
+        <v>36</v>
       </c>
       <c r="L38" t="s">
-        <v>114</v>
+        <v>58</v>
       </c>
       <c r="M38" t="s">
         <v>29</v>
@@ -3022,7 +3151,7 @@
         <v>31</v>
       </c>
       <c r="R38" t="s">
-        <v>20</v>
+        <v>155</v>
       </c>
       <c r="T38" t="n">
         <v>110.0</v>
@@ -3045,10 +3174,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="F39" t="s">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3060,13 +3189,13 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
       <c r="K39" t="s">
-        <v>118</v>
+        <v>36</v>
       </c>
       <c r="L39" t="s">
-        <v>119</v>
+        <v>37</v>
       </c>
       <c r="M39" t="s">
         <v>29</v>
@@ -3078,7 +3207,7 @@
         <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>115</v>
+        <v>76</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3101,10 +3230,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F40" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3116,13 +3245,13 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K40" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="L40" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="M40" t="s">
         <v>29</v>
@@ -3134,7 +3263,7 @@
         <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3160,7 +3289,7 @@
         <v>24</v>
       </c>
       <c r="F41" t="s">
-        <v>26</v>
+        <v>157</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3172,13 +3301,13 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>25</v>
+        <v>158</v>
       </c>
       <c r="K41" t="s">
-        <v>40</v>
+        <v>159</v>
       </c>
       <c r="L41" t="s">
-        <v>57</v>
+        <v>160</v>
       </c>
       <c r="M41" t="s">
         <v>29</v>
@@ -3190,7 +3319,7 @@
         <v>31</v>
       </c>
       <c r="R41" t="s">
-        <v>109</v>
+        <v>156</v>
       </c>
       <c r="T41" t="n">
         <v>110.0</v>
@@ -3213,11 +3342,11 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
+        <v>40</v>
+      </c>
+      <c r="F42" t="s">
         <v>41</v>
       </c>
-      <c r="F42" t="s">
-        <v>27</v>
-      </c>
       <c r="G42" t="s">
         <v>20</v>
       </c>
@@ -3228,13 +3357,13 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="K42" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="L42" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="M42" t="s">
         <v>29</v>
@@ -3243,13 +3372,13 @@
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>120</v>
+        <v>161</v>
       </c>
       <c r="Q42" t="s">
         <v>31</v>
       </c>
       <c r="R42" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3272,28 +3401,28 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
+        <v>24</v>
+      </c>
+      <c r="F43" t="s">
+        <v>142</v>
+      </c>
+      <c r="G43" t="s">
+        <v>20</v>
+      </c>
+      <c r="H43" t="s">
+        <v>20</v>
+      </c>
+      <c r="I43" t="s">
+        <v>20</v>
+      </c>
+      <c r="J43" t="s">
+        <v>163</v>
+      </c>
+      <c r="K43" t="s">
         <v>81</v>
       </c>
-      <c r="F43" t="s">
-        <v>122</v>
-      </c>
-      <c r="G43" t="s">
-        <v>20</v>
-      </c>
-      <c r="H43" t="s">
-        <v>20</v>
-      </c>
-      <c r="I43" t="s">
-        <v>20</v>
-      </c>
-      <c r="J43" t="s">
-        <v>123</v>
-      </c>
-      <c r="K43" t="s">
-        <v>124</v>
-      </c>
       <c r="L43" t="s">
-        <v>125</v>
+        <v>164</v>
       </c>
       <c r="M43" t="s">
         <v>29</v>
@@ -3305,7 +3434,7 @@
         <v>31</v>
       </c>
       <c r="R43" t="s">
-        <v>121</v>
+        <v>162</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3328,10 +3457,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="F44" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3343,13 +3472,13 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>88</v>
+        <v>151</v>
       </c>
       <c r="K44" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="L44" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="M44" t="s">
         <v>29</v>
@@ -3384,10 +3513,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="F45" t="s">
-        <v>127</v>
+        <v>163</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3399,13 +3528,13 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="K45" t="s">
-        <v>129</v>
+        <v>82</v>
       </c>
       <c r="L45" t="s">
-        <v>130</v>
+        <v>165</v>
       </c>
       <c r="M45" t="s">
         <v>29</v>
@@ -3417,7 +3546,7 @@
         <v>31</v>
       </c>
       <c r="R45" t="s">
-        <v>126</v>
+        <v>20</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3440,10 +3569,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>33</v>
+        <v>59</v>
       </c>
       <c r="F46" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3455,13 +3584,13 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="K46" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="L46" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="M46" t="s">
         <v>29</v>
@@ -3473,7 +3602,7 @@
         <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>131</v>
+        <v>20</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3496,10 +3625,10 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F47" t="s">
-        <v>27</v>
+        <v>124</v>
       </c>
       <c r="G47" t="s">
         <v>20</v>
@@ -3511,13 +3640,13 @@
         <v>20</v>
       </c>
       <c r="J47" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="K47" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="L47" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="M47" t="s">
         <v>29</v>
@@ -3526,13 +3655,13 @@
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>133</v>
+        <v>168</v>
       </c>
       <c r="Q47" t="s">
         <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>53</v>
+        <v>167</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3555,10 +3684,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="F48" t="s">
-        <v>27</v>
+        <v>170</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3570,13 +3699,13 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>26</v>
+        <v>171</v>
       </c>
       <c r="K48" t="s">
-        <v>25</v>
+        <v>172</v>
       </c>
       <c r="L48" t="s">
-        <v>40</v>
+        <v>173</v>
       </c>
       <c r="M48" t="s">
         <v>29</v>
@@ -3588,7 +3717,7 @@
         <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>53</v>
+        <v>169</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3611,10 +3740,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="F49" t="s">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3626,13 +3755,13 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="K49" t="s">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="L49" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="M49" t="s">
         <v>29</v>
@@ -3644,7 +3773,7 @@
         <v>31</v>
       </c>
       <c r="R49" t="s">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3667,10 +3796,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="F50" t="s">
-        <v>60</v>
+        <v>174</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3682,13 +3811,13 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>61</v>
+        <v>175</v>
       </c>
       <c r="K50" t="s">
-        <v>62</v>
+        <v>176</v>
       </c>
       <c r="L50" t="s">
-        <v>63</v>
+        <v>177</v>
       </c>
       <c r="M50" t="s">
         <v>29</v>
@@ -3700,7 +3829,7 @@
         <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3723,10 +3852,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="F51" t="s">
-        <v>26</v>
+        <v>124</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3738,13 +3867,13 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="K51" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="L51" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="M51" t="s">
         <v>29</v>
@@ -3756,7 +3885,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>134</v>
+        <v>167</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3767,7 +3896,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>135</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
marathi array ans to wrong ans
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="159">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,22 +83,22 @@
     <t>09030201</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 36$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 51$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$36 + 51 = 87$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 36$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 51$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$36 + 51 = 87$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 370$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 470$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$370 + 470 = 840$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 470$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$370 + 470 = 840$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
   </si>
   <si>
-    <t>$87$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$89$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$85$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$88$ &lt;br&gt;</t>
+    <t>$840$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$842$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$838$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$839$ &lt;br&gt;</t>
   </si>
   <si>
     <t>60</t>
@@ -110,25 +110,106 @@
     <t>2022.chinmay.chaudhari@ves.ac.in</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1300$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1299$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1302$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1301$ &lt;br&gt;</t>
   </si>
   <si>
     <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
   </si>
   <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
     <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
   </si>
   <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>$1670$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1668$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1671$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1672$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$4$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$3$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
   </si>
   <si>
     <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
@@ -149,403 +230,262 @@
     <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Ans: $38$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 61$&lt;br&gt;No. of travellers using the vehicle least $= 23$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$61 - 23 = 38$  is the answer.&lt;br&gt;#उत्तर : $38$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 23$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$61 - 23 = 38$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $4$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 5$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$5 - 1 = 4$  is the answer.&lt;br&gt;#उत्तर : $4$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$5 - 1 = 4$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
   </si>
   <si>
-    <t>$38$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$40$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$39$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$37$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 3300$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 7400$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$3300 + 7400 = 10700$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3300$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7400$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3300 + 7400 = 10700$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$10700$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$10698$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$10699$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$10701$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+    <t>$5$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$7$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>$8700$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8701$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8702$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8698$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Car, Scooter, Motorcycle&lt;br&gt;From the given graph we can see that, $Bicycle$, $Car$, $Scooter$, $Motorcycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Car, Scooter, Motorcycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Car$, $Scooter$, $Motorcycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Car, Scooter, Motorcycle&lt;br&gt;#सायकल, कार, दुचाकी, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle&lt;br&gt;#कार, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter&lt;br&gt;#कार, बस, ट्रक, दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle&lt;br&gt;#सायकल, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bicycle $= 98$&lt;br&gt;No. of travellers using the Motorcycle  $= 25$&lt;br&gt;No. of travellers using the Scooter  $= 17$&lt;br&gt;No. of travellers using the Car  $= 24$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$98 + 25 + 17 + 24 = 164$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bicycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 25$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 17$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 24$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$98 + 25 + 17 + 24 = 164$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$164$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$163$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$165$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$166$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Motorcycle, Scooter, Car&lt;br&gt;From the given graph we can see that, $Bicycle$, $Motorcycle$, $Scooter$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Motorcycle, Scooter, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Motorcycle$, $Scooter$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Motorcycle, Scooter, Car&lt;br&gt;#सायकल, मोटरसायकल, दुचाकी, कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $81$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 98$&lt;br&gt;No. of travellers using the vehicle least $= 17$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$98 - 17 = 81$  is the answer.&lt;br&gt;#उत्तर : $81$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 17$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$98 - 17 = 81$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$81$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$79$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$82$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$80$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$147$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$148$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$146$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$145$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$19700$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$19702$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$19699$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$19701$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Truck, Scooter, Motorcycle, Bus&lt;br&gt;From the given graph we can see that, $Truck$, $Scooter$, $Motorcycle$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Truck, Scooter, Motorcycle, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Truck$, $Scooter$, $Motorcycle$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck, Scooter, Motorcycle, Bus&lt;br&gt;#ट्रक, दुचाकी, मोटरसायकल, बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Truck, Bicycle, Car&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Truck$, $Bicycle$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Truck, Bicycle, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Truck$, $Bicycle$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Truck, Bicycle, Car&lt;br&gt;#मोटरसायकल, ट्रक, सायकल, कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 40$&lt;br&gt;No. of travellers using the Truck  $= 10$&lt;br&gt;No. of travellers using the Bicycle  $= 46$&lt;br&gt;No. of travellers using the Car  $= 50$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$40 + 10 + 46 + 50 = 146$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 40$&lt;br&gt;Truck या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 10$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 46$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 50$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$40 + 10 + 46 + 50 = 146$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$136$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$135$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$134$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$137$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$11$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$13$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 5$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 6$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$5 + 6 = 11$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$5 + 6 = 11$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$9$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 4$&lt;br&gt;No. of travellers using the Bicycle  $= 5$&lt;br&gt;No. of travellers using the Scooter  $= 6$&lt;br&gt;No. of travellers using the Truck  $= 8$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$4 + 5 + 6 + 8 = 23$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$4 + 5 + 6 + 8 = 23$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$23$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$24$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$25$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$22$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
+  </si>
+  <si>
+    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 6$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$6 - 1 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$6 - 1 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Scooter, Truck, Motorcycle&lt;br&gt;From the given graph we can see that, $Bicycle$, $Scooter$, $Truck$, $Motorcycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Scooter, Truck, Motorcycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Scooter$, $Truck$, $Motorcycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Scooter, Truck, Motorcycle&lt;br&gt;#सायकल, दुचाकी, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2010$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2012$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2008$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2011$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
+  </si>
+  <si>
+    <t>Ans: Car, Scooter, Truck, Bicycle&lt;br&gt;From the given graph we can see that, $Car$, $Scooter$, $Truck$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Scooter, Truck, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Scooter$, $Truck$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Scooter, Truck, Bicycle&lt;br&gt;#कार, दुचाकी, ट्रक, सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 150$&lt;br&gt;No. of travellers using the Scooter  $= 540$&lt;br&gt;No. of travellers using the Truck  $= 570$&lt;br&gt;No. of travellers using the Bicycle  $= 900$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$150 + 540 + 570 + 900 = 2160$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 150$&lt;br&gt;Scooter या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 540$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 570$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 900$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$150 + 540 + 570 + 900 = 2160$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2160$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2159$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2161$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2158$ &lt;br&gt;</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 1600$&lt;br&gt;No. of travellers using the Bus  $= 3300$&lt;br&gt;No. of travellers using the Bicycle  $= 7400$&lt;br&gt;No. of travellers using the Scooter  $= 8100$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$1600 + 3300 + 7400 + 8100 = 20400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 1600$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 3300$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7400$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 8100$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$1600 + 3300 + 7400 + 8100 = 20400$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$20400$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$20398$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$20401$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$20402$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $92$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 98$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$98 - 6 = 92$  is the answer.&lt;br&gt;#उत्तर : $92$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$98 - 6 = 92$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$92$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$94$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$90$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$91$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$4$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$3$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $62$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 95$&lt;br&gt;No. of travellers using the vehicle least $= 33$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$95 - 33 = 62$  is the answer.&lt;br&gt;#उत्तर : $62$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 95$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 33$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$95 - 33 = 62$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$62$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$61$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$63$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$64$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$128$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$130$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$127$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$129$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Motorcycle, Bus, Scooter, Bicycle&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Bus$, $Scooter$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Bus, Scooter, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Bus$, $Scooter$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle, Bus, Scooter, Bicycle&lt;br&gt;#मोटरसायकल, बस, दुचाकी, सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle</t>
-  </si>
-  <si>
-    <t>$700$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$702$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$698$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$699$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 230$&lt;br&gt;No. of travellers using the Bus  $= 460$&lt;br&gt;No. of travellers using the Bicycle  $= 550$&lt;br&gt;No. of travellers using the Truck  $= 150$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$230 + 460 + 550 + 150 = 1390$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 230$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 460$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 550$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 150$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$230 + 460 + 550 + 150 = 1390$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1390$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1391$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1389$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1392$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 230$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 460$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$230 + 460 = 690$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 230$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 460$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$230 + 460 = 690$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$690$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$689$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$692$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$688$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?</t>
-  </si>
-  <si>
-    <t>$1240$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1239$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1242$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1238$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$136$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$135$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$137$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$138$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 86$&lt;br&gt;No. of travellers using the Car  $= 83$&lt;br&gt;No. of travellers using the Scooter  $= 66$&lt;br&gt;No. of travellers using the Bus  $= 50$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$86 + 83 + 66 + 50 = 285$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 86$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 66$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 50$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$86 + 83 + 66 + 50 = 285$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$285$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$284$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$283$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$287$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 66$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 83$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$66 + 83 = 149$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 66$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$66 + 83 = 149$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$149$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$150$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$147$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$151$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $6$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9$&lt;br&gt;No. of travellers using the vehicle least $= 3$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9 - 3 = 6$  is the answer.&lt;br&gt;#उत्तर : $6$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9 - 3 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$7$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Truck, Bus, Scooter&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Bus$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Bus, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Bus$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Truck, Bus, Scooter&lt;br&gt;#सायकल, ट्रक, बस, दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 6$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 7$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$6 + 7 = 13$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$6 + 7 = 13$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$13$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$11$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$12$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$15$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Scooter, Motorcycle, Bicycle, Truck&lt;br&gt;From the given graph we can see that, $Scooter$, $Motorcycle$, $Bicycle$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Scooter, Motorcycle, Bicycle, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Scooter$, $Motorcycle$, $Bicycle$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter, Motorcycle, Bicycle, Truck&lt;br&gt;#दुचाकी, मोटरसायकल, सायकल, ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 7$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 9$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$7 + 9 = 16$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$7 + 9 = 16$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$16$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$18$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$17$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$14$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 3$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 4$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$3 + 4 = 7$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3 + 4 = 7$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$8$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$9$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$10$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
-  </si>
-  <si>
-    <t>Ans: $67$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 73$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$73 - 6 = 67$  is the answer.&lt;br&gt;#उत्तर : $67$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 73$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$73 - 6 = 67$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$67$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$66$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$69$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$68$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$79$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$77$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$81$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$80$ &lt;br&gt;</t>
   </si>
   <si>
     <t>****</t>
@@ -1196,7 +1136,7 @@
         <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1208,13 +1148,13 @@
         <v>20</v>
       </c>
       <c r="J4" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="K4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="L4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="M4" t="s">
         <v>29</v>
@@ -1226,7 +1166,7 @@
         <v>31</v>
       </c>
       <c r="R4" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1249,10 +1189,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1264,13 +1204,13 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="K5" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="L5" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="M5" t="s">
         <v>29</v>
@@ -1282,7 +1222,7 @@
         <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1305,28 +1245,28 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+      <c r="I6" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" t="s">
+        <v>36</v>
+      </c>
+      <c r="K6" t="s">
         <v>46</v>
       </c>
-      <c r="F6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" t="s">
-        <v>48</v>
-      </c>
-      <c r="K6" t="s">
-        <v>49</v>
-      </c>
       <c r="L6" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="M6" t="s">
         <v>29</v>
@@ -1338,7 +1278,7 @@
         <v>31</v>
       </c>
       <c r="R6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1361,10 +1301,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1376,13 +1316,13 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="K7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="L7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="M7" t="s">
         <v>29</v>
@@ -1391,13 +1331,13 @@
         <v>4.0</v>
       </c>
       <c r="P7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="Q7" t="s">
         <v>31</v>
       </c>
       <c r="R7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="T7" t="n">
         <v>110.0</v>
@@ -1420,10 +1360,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1435,13 +1375,13 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="K8" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="L8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="M8" t="s">
         <v>29</v>
@@ -1453,7 +1393,7 @@
         <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1476,10 +1416,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>56</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1491,13 +1431,13 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="K9" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="L9" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="M9" t="s">
         <v>29</v>
@@ -1509,7 +1449,7 @@
         <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1532,10 +1472,10 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1547,13 +1487,13 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="K10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="M10" t="s">
         <v>29</v>
@@ -1588,40 +1528,40 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" t="s">
+        <v>69</v>
+      </c>
+      <c r="K11" t="s">
+        <v>70</v>
+      </c>
+      <c r="L11" t="s">
+        <v>71</v>
+      </c>
+      <c r="M11" t="s">
+        <v>29</v>
+      </c>
+      <c r="N11" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>31</v>
+      </c>
+      <c r="R11" t="s">
         <v>66</v>
-      </c>
-      <c r="G11" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" t="s">
-        <v>67</v>
-      </c>
-      <c r="K11" t="s">
-        <v>68</v>
-      </c>
-      <c r="L11" t="s">
-        <v>69</v>
-      </c>
-      <c r="M11" t="s">
-        <v>29</v>
-      </c>
-      <c r="N11" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>31</v>
-      </c>
-      <c r="R11" t="s">
-        <v>64</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1644,43 +1584,43 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" t="s">
+        <v>20</v>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" t="s">
+        <v>35</v>
+      </c>
+      <c r="K12" t="s">
+        <v>36</v>
+      </c>
+      <c r="L12" t="s">
         <v>46</v>
       </c>
-      <c r="F12" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>20</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="M12" t="s">
+        <v>29</v>
+      </c>
+      <c r="N12" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P12" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>31</v>
+      </c>
+      <c r="R12" t="s">
         <v>72</v>
-      </c>
-      <c r="K12" t="s">
-        <v>73</v>
-      </c>
-      <c r="L12" t="s">
-        <v>74</v>
-      </c>
-      <c r="M12" t="s">
-        <v>29</v>
-      </c>
-      <c r="N12" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P12" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>31</v>
-      </c>
-      <c r="R12" t="s">
-        <v>70</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1703,10 +1643,10 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="F13" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="G13" t="s">
         <v>20</v>
@@ -1724,7 +1664,7 @@
         <v>36</v>
       </c>
       <c r="L13" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="M13" t="s">
         <v>29</v>
@@ -1736,7 +1676,7 @@
         <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1759,7 +1699,7 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
         <v>34</v>
@@ -1792,7 +1732,7 @@
         <v>31</v>
       </c>
       <c r="R14" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1815,10 +1755,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>40</v>
+        <v>77</v>
       </c>
       <c r="F15" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1830,13 +1770,13 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="K15" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="L15" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="M15" t="s">
         <v>29</v>
@@ -1848,7 +1788,7 @@
         <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1871,28 +1811,28 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" t="s">
         <v>79</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J16" t="s">
+        <v>58</v>
+      </c>
+      <c r="K16" t="s">
         <v>80</v>
       </c>
-      <c r="G16" t="s">
-        <v>20</v>
-      </c>
-      <c r="H16" t="s">
-        <v>20</v>
-      </c>
-      <c r="I16" t="s">
-        <v>20</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="L16" t="s">
         <v>81</v>
-      </c>
-      <c r="K16" t="s">
-        <v>82</v>
-      </c>
-      <c r="L16" t="s">
-        <v>83</v>
       </c>
       <c r="M16" t="s">
         <v>29</v>
@@ -1927,10 +1867,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="F17" t="s">
-        <v>85</v>
+        <v>57</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1942,13 +1882,13 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="K17" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="L17" t="s">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="M17" t="s">
         <v>29</v>
@@ -1957,13 +1897,13 @@
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="Q17" t="s">
         <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1986,10 +1926,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -2001,13 +1941,13 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="K18" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="L18" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="M18" t="s">
         <v>29</v>
@@ -2019,7 +1959,7 @@
         <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -2042,10 +1982,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="F19" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -2057,13 +1997,13 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="K19" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="L19" t="s">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="M19" t="s">
         <v>29</v>
@@ -2075,7 +2015,7 @@
         <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2098,10 +2038,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="F20" t="s">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2113,13 +2053,13 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="K20" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="L20" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="M20" t="s">
         <v>29</v>
@@ -2131,7 +2071,7 @@
         <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>39</v>
+        <v>87</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2154,10 +2094,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>98</v>
+        <v>33</v>
       </c>
       <c r="F21" t="s">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2169,13 +2109,13 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>100</v>
+        <v>35</v>
       </c>
       <c r="K21" t="s">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="L21" t="s">
-        <v>102</v>
+        <v>46</v>
       </c>
       <c r="M21" t="s">
         <v>29</v>
@@ -2187,7 +2127,7 @@
         <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2210,10 +2150,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F22" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2225,13 +2165,13 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="K22" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="L22" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="M22" t="s">
         <v>29</v>
@@ -2240,13 +2180,13 @@
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="Q22" t="s">
         <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2269,10 +2209,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="F23" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2284,13 +2224,13 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>110</v>
+        <v>90</v>
       </c>
       <c r="K23" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="L23" t="s">
-        <v>112</v>
+        <v>92</v>
       </c>
       <c r="M23" t="s">
         <v>29</v>
@@ -2302,7 +2242,7 @@
         <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2325,10 +2265,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F24" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2340,13 +2280,13 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="K24" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="L24" t="s">
-        <v>117</v>
+        <v>106</v>
       </c>
       <c r="M24" t="s">
         <v>29</v>
@@ -2358,7 +2298,7 @@
         <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2381,10 +2321,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>118</v>
+        <v>51</v>
       </c>
       <c r="F25" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2396,13 +2336,13 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="K25" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="L25" t="s">
-        <v>122</v>
+        <v>110</v>
       </c>
       <c r="M25" t="s">
         <v>29</v>
@@ -2437,29 +2377,29 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
+        <v>56</v>
+      </c>
+      <c r="F26" t="s">
+        <v>57</v>
+      </c>
+      <c r="G26" t="s">
+        <v>20</v>
+      </c>
+      <c r="H26" t="s">
+        <v>20</v>
+      </c>
+      <c r="I26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J26" t="s">
+        <v>60</v>
+      </c>
+      <c r="K26" t="s">
+        <v>59</v>
+      </c>
+      <c r="L26" t="s">
         <v>78</v>
       </c>
-      <c r="F26" t="s">
-        <v>58</v>
-      </c>
-      <c r="G26" t="s">
-        <v>20</v>
-      </c>
-      <c r="H26" t="s">
-        <v>20</v>
-      </c>
-      <c r="I26" t="s">
-        <v>20</v>
-      </c>
-      <c r="J26" t="s">
-        <v>35</v>
-      </c>
-      <c r="K26" t="s">
-        <v>124</v>
-      </c>
-      <c r="L26" t="s">
-        <v>34</v>
-      </c>
       <c r="M26" t="s">
         <v>29</v>
       </c>
@@ -2470,7 +2410,7 @@
         <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>123</v>
+        <v>20</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2493,10 +2433,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="F27" t="s">
-        <v>125</v>
+        <v>36</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2508,13 +2448,13 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>126</v>
+        <v>35</v>
       </c>
       <c r="K27" t="s">
-        <v>127</v>
+        <v>48</v>
       </c>
       <c r="L27" t="s">
-        <v>128</v>
+        <v>49</v>
       </c>
       <c r="M27" t="s">
         <v>29</v>
@@ -2523,13 +2463,13 @@
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="Q27" t="s">
         <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2552,10 +2492,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="F28" t="s">
-        <v>131</v>
+        <v>37</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2567,13 +2507,13 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>132</v>
+        <v>35</v>
       </c>
       <c r="K28" t="s">
-        <v>133</v>
+        <v>48</v>
       </c>
       <c r="L28" t="s">
-        <v>134</v>
+        <v>49</v>
       </c>
       <c r="M28" t="s">
         <v>29</v>
@@ -2585,7 +2525,7 @@
         <v>31</v>
       </c>
       <c r="R28" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2608,10 +2548,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="F29" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2623,13 +2563,13 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>137</v>
+        <v>115</v>
       </c>
       <c r="K29" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
       <c r="L29" t="s">
-        <v>139</v>
+        <v>117</v>
       </c>
       <c r="M29" t="s">
         <v>29</v>
@@ -2641,7 +2581,7 @@
         <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>135</v>
+        <v>20</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2664,10 +2604,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="F30" t="s">
-        <v>58</v>
+        <v>119</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2679,13 +2619,13 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="K30" t="s">
-        <v>124</v>
+        <v>91</v>
       </c>
       <c r="L30" t="s">
-        <v>34</v>
+        <v>92</v>
       </c>
       <c r="M30" t="s">
         <v>29</v>
@@ -2697,7 +2637,7 @@
         <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2720,10 +2660,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F31" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2738,10 +2678,10 @@
         <v>35</v>
       </c>
       <c r="K31" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="L31" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="M31" t="s">
         <v>29</v>
@@ -2753,7 +2693,7 @@
         <v>31</v>
       </c>
       <c r="R31" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
       <c r="T31" t="n">
         <v>110.0</v>
@@ -2776,10 +2716,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="F32" t="s">
-        <v>82</v>
+        <v>121</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2791,13 +2731,13 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="K32" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="L32" t="s">
-        <v>142</v>
+        <v>92</v>
       </c>
       <c r="M32" t="s">
         <v>29</v>
@@ -2806,13 +2746,13 @@
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>143</v>
+        <v>122</v>
       </c>
       <c r="Q32" t="s">
         <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>141</v>
+        <v>120</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2835,10 +2775,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
       <c r="F33" t="s">
-        <v>145</v>
+        <v>68</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2850,13 +2790,13 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="K33" t="s">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="L33" t="s">
-        <v>102</v>
+        <v>71</v>
       </c>
       <c r="M33" t="s">
         <v>29</v>
@@ -2868,7 +2808,7 @@
         <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>144</v>
+        <v>66</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2891,10 +2831,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="F34" t="s">
-        <v>147</v>
+        <v>37</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2906,13 +2846,13 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
       <c r="K34" t="s">
-        <v>149</v>
+        <v>48</v>
       </c>
       <c r="L34" t="s">
-        <v>150</v>
+        <v>49</v>
       </c>
       <c r="M34" t="s">
         <v>29</v>
@@ -2924,7 +2864,7 @@
         <v>31</v>
       </c>
       <c r="R34" t="s">
-        <v>146</v>
+        <v>113</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2947,10 +2887,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="F35" t="s">
-        <v>80</v>
+        <v>109</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2962,13 +2902,13 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>151</v>
+        <v>107</v>
       </c>
       <c r="K35" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="L35" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="M35" t="s">
         <v>29</v>
@@ -2980,7 +2920,7 @@
         <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -3003,10 +2943,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="F36" t="s">
-        <v>96</v>
+        <v>124</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -3018,13 +2958,13 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>35</v>
+        <v>125</v>
       </c>
       <c r="K36" t="s">
-        <v>36</v>
+        <v>126</v>
       </c>
       <c r="L36" t="s">
-        <v>58</v>
+        <v>127</v>
       </c>
       <c r="M36" t="s">
         <v>29</v>
@@ -3036,7 +2976,7 @@
         <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -3059,10 +2999,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>98</v>
+        <v>38</v>
       </c>
       <c r="F37" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3074,13 +3014,13 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="K37" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="L37" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
       <c r="M37" t="s">
         <v>29</v>
@@ -3089,13 +3029,13 @@
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>154</v>
+        <v>131</v>
       </c>
       <c r="Q37" t="s">
         <v>31</v>
       </c>
       <c r="R37" t="s">
-        <v>152</v>
+        <v>20</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3118,10 +3058,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="F38" t="s">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3139,7 +3079,7 @@
         <v>36</v>
       </c>
       <c r="L38" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="M38" t="s">
         <v>29</v>
@@ -3151,7 +3091,7 @@
         <v>31</v>
       </c>
       <c r="R38" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="T38" t="n">
         <v>110.0</v>
@@ -3174,10 +3114,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="F39" t="s">
-        <v>34</v>
+        <v>129</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3189,13 +3129,13 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>35</v>
+        <v>130</v>
       </c>
       <c r="K39" t="s">
-        <v>36</v>
+        <v>128</v>
       </c>
       <c r="L39" t="s">
-        <v>37</v>
+        <v>134</v>
       </c>
       <c r="M39" t="s">
         <v>29</v>
@@ -3207,7 +3147,7 @@
         <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>76</v>
+        <v>133</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3230,10 +3170,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="F40" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3251,7 +3191,7 @@
         <v>36</v>
       </c>
       <c r="L40" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="M40" t="s">
         <v>29</v>
@@ -3263,7 +3203,7 @@
         <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3286,10 +3226,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="F41" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3301,13 +3241,13 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="K41" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="L41" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="M41" t="s">
         <v>29</v>
@@ -3319,7 +3259,7 @@
         <v>31</v>
       </c>
       <c r="R41" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="T41" t="n">
         <v>110.0</v>
@@ -3342,10 +3282,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="F42" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3357,13 +3297,13 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="K42" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="L42" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="M42" t="s">
         <v>29</v>
@@ -3372,13 +3312,13 @@
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>161</v>
+        <v>140</v>
       </c>
       <c r="Q42" t="s">
         <v>31</v>
       </c>
       <c r="R42" t="s">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3401,10 +3341,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F43" t="s">
-        <v>142</v>
+        <v>78</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3416,13 +3356,13 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>163</v>
+        <v>57</v>
       </c>
       <c r="K43" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L43" t="s">
-        <v>164</v>
+        <v>58</v>
       </c>
       <c r="M43" t="s">
         <v>29</v>
@@ -3434,7 +3374,7 @@
         <v>31</v>
       </c>
       <c r="R43" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3457,10 +3397,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F44" t="s">
-        <v>80</v>
+        <v>143</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3472,13 +3412,13 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>151</v>
+        <v>90</v>
       </c>
       <c r="K44" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="L44" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="M44" t="s">
         <v>29</v>
@@ -3490,7 +3430,7 @@
         <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3513,10 +3453,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="F45" t="s">
-        <v>163</v>
+        <v>48</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3528,13 +3468,13 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>142</v>
+        <v>35</v>
       </c>
       <c r="K45" t="s">
-        <v>82</v>
+        <v>36</v>
       </c>
       <c r="L45" t="s">
-        <v>165</v>
+        <v>46</v>
       </c>
       <c r="M45" t="s">
         <v>29</v>
@@ -3546,7 +3486,7 @@
         <v>31</v>
       </c>
       <c r="R45" t="s">
-        <v>20</v>
+        <v>144</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3569,10 +3509,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="F46" t="s">
-        <v>166</v>
+        <v>48</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3584,13 +3524,13 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="K46" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="L46" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="M46" t="s">
         <v>29</v>
@@ -3602,7 +3542,7 @@
         <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>20</v>
+        <v>144</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3625,10 +3565,10 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F47" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="G47" t="s">
         <v>20</v>
@@ -3640,13 +3580,13 @@
         <v>20</v>
       </c>
       <c r="J47" t="s">
-        <v>35</v>
+        <v>146</v>
       </c>
       <c r="K47" t="s">
-        <v>36</v>
+        <v>147</v>
       </c>
       <c r="L47" t="s">
-        <v>37</v>
+        <v>148</v>
       </c>
       <c r="M47" t="s">
         <v>29</v>
@@ -3655,13 +3595,13 @@
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>168</v>
+        <v>149</v>
       </c>
       <c r="Q47" t="s">
         <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>167</v>
+        <v>20</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3684,29 +3624,29 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
+        <v>75</v>
+      </c>
+      <c r="F48" t="s">
+        <v>49</v>
+      </c>
+      <c r="G48" t="s">
+        <v>20</v>
+      </c>
+      <c r="H48" t="s">
+        <v>20</v>
+      </c>
+      <c r="I48" t="s">
+        <v>20</v>
+      </c>
+      <c r="J48" t="s">
+        <v>35</v>
+      </c>
+      <c r="K48" t="s">
+        <v>36</v>
+      </c>
+      <c r="L48" t="s">
         <v>46</v>
       </c>
-      <c r="F48" t="s">
-        <v>170</v>
-      </c>
-      <c r="G48" t="s">
-        <v>20</v>
-      </c>
-      <c r="H48" t="s">
-        <v>20</v>
-      </c>
-      <c r="I48" t="s">
-        <v>20</v>
-      </c>
-      <c r="J48" t="s">
-        <v>171</v>
-      </c>
-      <c r="K48" t="s">
-        <v>172</v>
-      </c>
-      <c r="L48" t="s">
-        <v>173</v>
-      </c>
       <c r="M48" t="s">
         <v>29</v>
       </c>
@@ -3717,7 +3657,7 @@
         <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>169</v>
+        <v>132</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3740,10 +3680,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="F49" t="s">
-        <v>41</v>
+        <v>151</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3755,13 +3695,13 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="K49" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="L49" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="M49" t="s">
         <v>29</v>
@@ -3773,7 +3713,7 @@
         <v>31</v>
       </c>
       <c r="R49" t="s">
-        <v>39</v>
+        <v>150</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3796,10 +3736,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F50" t="s">
-        <v>174</v>
+        <v>153</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3811,13 +3751,13 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>175</v>
+        <v>154</v>
       </c>
       <c r="K50" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="L50" t="s">
-        <v>177</v>
+        <v>156</v>
       </c>
       <c r="M50" t="s">
         <v>29</v>
@@ -3829,7 +3769,7 @@
         <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>20</v>
+        <v>152</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3852,10 +3792,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="F51" t="s">
-        <v>124</v>
+        <v>35</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3867,10 +3807,10 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K51" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="L51" t="s">
         <v>37</v>
@@ -3885,7 +3825,7 @@
         <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3896,7 +3836,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added solution for top 3
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="196">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,409 +83,520 @@
     <t>09030201</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 370$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 470$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$370 + 470 = 840$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 470$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$370 + 470 = 840$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12900$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12902$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12901$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12898$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$4$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$3$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $6700$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9800$&lt;br&gt;No. of travellers using the vehicle least $= 3100$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9800 - 3100 = 6700$  is the answer.&lt;br&gt;#उत्तर : $6700$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9800$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3100$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9800 - 3100 = 6700$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6700$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6699$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6701$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$6698$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Car, Bicycle, Scooter, Motorcycle&lt;br&gt;From the given graph we can see that, $Car$, $Bicycle$, $Scooter$, $Motorcycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Bicycle, Scooter, Motorcycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Bicycle$, $Scooter$, $Motorcycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bicycle, Scooter, Motorcycle&lt;br&gt;#कार, सायकल, दुचाकी, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle&lt;br&gt;#कार, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter&lt;br&gt;#कार, बस, ट्रक, दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle&lt;br&gt;#सायकल, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 92$&lt;br&gt;No. of travellers using the Bicycle  $= 63$&lt;br&gt;No. of travellers using the Scooter  $= 99$&lt;br&gt;No. of travellers using the Truck  $= 41$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$92 + 63 + 99 + 41 = 295$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 92$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 63$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 99$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 41$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$92 + 63 + 99 + 41 = 295$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$295$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$296$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$294$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$293$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$140$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$138$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$141$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$139$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 5$&lt;br&gt;No. of travellers using the vehicle least $= 0$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$5 - 0 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 0$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$5 - 0 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$7$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of travelers by different means.</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 210$&lt;br&gt;No. of travellers using the Bicycle  $= 370$&lt;br&gt;No. of travellers using the Motorcycle  $= 200$&lt;br&gt;No. of travellers using the Car  $= 250$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$210 + 370 + 200 + 250 = 1030$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 210$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 200$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 250$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$210 + 370 + 200 + 250 = 1030$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1030$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1031$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1029$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1028$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 370$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 250$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 210$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$370 + 250 + 210 = 830$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 250$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 210$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$370 + 250 + 210 = 830$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>$830$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$829$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$828$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$831$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $170$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 370$&lt;br&gt;No. of travellers using the vehicle least $= 200$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$370 - 200 = 170$  is the answer.&lt;br&gt;#उत्तर : $170$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 200$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$370 - 200 = 170$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$170$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$169$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$168$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$172$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 130$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 940$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$130 + 940 = 1070$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 130$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 940$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$130 + 940 = 1070$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
   </si>
   <si>
-    <t>$840$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$842$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$838$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$839$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+    <t>$1070$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1068$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1071$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1072$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1300$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1299$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1302$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1301$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>Ans: Bus, Bicycle, Car, Scooter&lt;br&gt;From the given graph we can see that, $Bus$, $Bicycle$, $Car$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bus, Bicycle, Car, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bus$, $Bicycle$, $Car$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus, Bicycle, Car, Scooter&lt;br&gt;#बस, सायकल, कार, दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 9300$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 8300$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 4000$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$9300 + 8300 + 4000 = 21600$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8300$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4000$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$9300 + 8300 + 4000 = 21600$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$21600$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$21602$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$21601$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$21599$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 3800$&lt;br&gt;No. of travellers using the Bicycle  $= 4000$&lt;br&gt;No. of travellers using the Car  $= 8300$&lt;br&gt;No. of travellers using the Scooter  $= 9300$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$3800 + 4000 + 8300 + 9300 = 25400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 4000$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 8300$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$3800 + 4000 + 8300 + 9300 = 25400$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$25400$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$25401$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$25398$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$25399$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $5500$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9300$&lt;br&gt;No. of travellers using the vehicle least $= 3800$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9300 - 3800 = 5500$  is the answer.&lt;br&gt;#उत्तर : $5500$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9300 - 3800 = 5500$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5500$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5498$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5502$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$5501$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Bus, Car, Motorcycle, Truck&lt;br&gt;From the given graph we can see that, $Bus$, $Car$, $Motorcycle$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bus, Car, Motorcycle, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bus$, $Car$, $Motorcycle$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus, Car, Motorcycle, Truck&lt;br&gt;#बस, कार, मोटरसायकल, ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
   </si>
   <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?</t>
-  </si>
-  <si>
-    <t>$1670$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1668$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1671$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1672$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$4$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$3$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of travelers by different means.</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $4$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 5$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$5 - 1 = 4$  is the answer.&lt;br&gt;#उत्तर : $4$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$5 - 1 = 4$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5$ &lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 98$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 69$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 61$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$98 + 69 + 61 = 228$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 69$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$98 + 69 + 61 = 228$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$228$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$230$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$229$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$226$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $44$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 98$&lt;br&gt;No. of travellers using the vehicle least $= 54$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$98 - 54 = 44$  is the answer.&lt;br&gt;#उत्तर : $44$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 54$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$98 - 54 = 44$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$44$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$45$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$43$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$46$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 1$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 2$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$1 + 2 = 3$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$1 + 2 = 3$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 3$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 2$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 1$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$3 + 2 + 1 = 6$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3 + 2 + 1 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>$8$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>$7$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$10$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>$8700$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$8701$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$8702$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$8698$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Car, Scooter, Motorcycle&lt;br&gt;From the given graph we can see that, $Bicycle$, $Car$, $Scooter$, $Motorcycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Car, Scooter, Motorcycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Car$, $Scooter$, $Motorcycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Car, Scooter, Motorcycle&lt;br&gt;#सायकल, कार, दुचाकी, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle&lt;br&gt;#कार, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter&lt;br&gt;#कार, बस, ट्रक, दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle&lt;br&gt;#सायकल, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bicycle $= 98$&lt;br&gt;No. of travellers using the Motorcycle  $= 25$&lt;br&gt;No. of travellers using the Scooter  $= 17$&lt;br&gt;No. of travellers using the Car  $= 24$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$98 + 25 + 17 + 24 = 164$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bicycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 25$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 17$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 24$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$98 + 25 + 17 + 24 = 164$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$164$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$163$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$165$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$166$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Motorcycle, Scooter, Car&lt;br&gt;From the given graph we can see that, $Bicycle$, $Motorcycle$, $Scooter$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Motorcycle, Scooter, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Motorcycle$, $Scooter$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Motorcycle, Scooter, Car&lt;br&gt;#सायकल, मोटरसायकल, दुचाकी, कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $81$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 98$&lt;br&gt;No. of travellers using the vehicle least $= 17$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$98 - 17 = 81$  is the answer.&lt;br&gt;#उत्तर : $81$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 17$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$98 - 17 = 81$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$81$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$79$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$82$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$80$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$147$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$148$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$146$ &lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 0$&lt;br&gt;No. of travellers using the Car  $= 1$&lt;br&gt;No. of travellers using the Motorcycle  $= 2$&lt;br&gt;No. of travellers using the Scooter  $= 3$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$0 + 1 + 2 + 3 = 6$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 0$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$0 + 1 + 2 + 3 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
+  </si>
+  <si>
+    <t>$117$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$119$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$115$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$118$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $69$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 93$&lt;br&gt;No. of travellers using the vehicle least $= 24$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$93 - 24 = 69$  is the answer.&lt;br&gt;#उत्तर : $69$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 93$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 24$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$93 - 24 = 69$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$69$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$70$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$68$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$71$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 51$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 92$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$51 + 92 = 143$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 51$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 92$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$51 + 92 = 143$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$143$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$142$ &lt;br&gt;</t>
   </si>
   <si>
     <t>$145$ &lt;br&gt;</t>
   </si>
   <si>
+    <t>$144$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 93$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 92$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 51$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$93 + 92 + 51 = 236$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 93$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 92$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 51$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$93 + 92 + 51 = 236$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$236$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$238$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$237$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$235$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Scooter, Truck, Bus&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Scooter$, $Truck$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Scooter, Truck, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Scooter$, $Truck$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Scooter, Truck, Bus&lt;br&gt;#मोटरसायकल, दुचाकी, ट्रक, बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 810$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 790$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 440$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$810 + 790 + 440 = 2040$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 810$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 790$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 440$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$810 + 790 + 440 = 2040$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2040$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2042$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2039$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$2038$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 440$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 790$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$440 + 790 = 1230$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 440$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 790$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$440 + 790 = 1230$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1230$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1229$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1228$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1231$ &lt;br&gt;</t>
+  </si>
+  <si>
     <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
   </si>
   <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$19700$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$19702$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$19699$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$19701$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Truck, Scooter, Motorcycle, Bus&lt;br&gt;From the given graph we can see that, $Truck$, $Scooter$, $Motorcycle$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Truck, Scooter, Motorcycle, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Truck$, $Scooter$, $Motorcycle$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck, Scooter, Motorcycle, Bus&lt;br&gt;#ट्रक, दुचाकी, मोटरसायकल, बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Motorcycle, Truck, Bicycle, Car&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Truck$, $Bicycle$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Truck, Bicycle, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Truck$, $Bicycle$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle, Truck, Bicycle, Car&lt;br&gt;#मोटरसायकल, ट्रक, सायकल, कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 40$&lt;br&gt;No. of travellers using the Truck  $= 10$&lt;br&gt;No. of travellers using the Bicycle  $= 46$&lt;br&gt;No. of travellers using the Car  $= 50$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$40 + 10 + 46 + 50 = 146$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 40$&lt;br&gt;Truck या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 10$&lt;br&gt;Bicycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 46$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 50$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$40 + 10 + 46 + 50 = 146$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$136$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$135$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$134$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$137$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$12$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$11$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$13$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 5$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 6$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$5 + 6 = 11$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$5 + 6 = 11$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$9$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Motorcycle $= 4$&lt;br&gt;No. of travellers using the Bicycle  $= 5$&lt;br&gt;No. of travellers using the Scooter  $= 6$&lt;br&gt;No. of travellers using the Truck  $= 8$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$4 + 5 + 6 + 8 = 23$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Motorcycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$4 + 5 + 6 + 8 = 23$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$23$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$24$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$25$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$22$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 6$&lt;br&gt;No. of travellers using the vehicle least $= 1$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$6 - 1 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$6 - 1 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Bicycle, Scooter, Truck, Motorcycle&lt;br&gt;From the given graph we can see that, $Bicycle$, $Scooter$, $Truck$, $Motorcycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Scooter, Truck, Motorcycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Scooter$, $Truck$, $Motorcycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Scooter, Truck, Motorcycle&lt;br&gt;#सायकल, दुचाकी, ट्रक, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2010$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2012$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2008$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2011$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
-  </si>
-  <si>
-    <t>Ans: Car, Scooter, Truck, Bicycle&lt;br&gt;From the given graph we can see that, $Car$, $Scooter$, $Truck$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Scooter, Truck, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Scooter$, $Truck$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Scooter, Truck, Bicycle&lt;br&gt;#कार, दुचाकी, ट्रक, सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 150$&lt;br&gt;No. of travellers using the Scooter  $= 540$&lt;br&gt;No. of travellers using the Truck  $= 570$&lt;br&gt;No. of travellers using the Bicycle  $= 900$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$150 + 540 + 570 + 900 = 2160$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 150$&lt;br&gt;Scooter या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 540$&lt;br&gt;Truck या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 570$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 900$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$150 + 540 + 570 + 900 = 2160$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2160$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2159$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2161$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2158$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+    <t>$1060$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1058$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1059$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1062$ &lt;br&gt;</t>
   </si>
   <si>
     <t>****</t>
@@ -926,7 +1037,7 @@
     <col min="3" max="3" width="12.4375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.66015625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="193.7734375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="67.39453125" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="65.68359375" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="16.42578125" customWidth="true" bestFit="true"/>
@@ -1018,43 +1129,43 @@
         <v>22</v>
       </c>
       <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
         <v>24</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
         <v>25</v>
       </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>26</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" t="s">
-        <v>28</v>
-      </c>
       <c r="M2" t="s">
+        <v>28</v>
+      </c>
+      <c r="N2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P2" t="s">
-        <v>30</v>
-      </c>
       <c r="Q2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="T2" t="n">
         <v>110.0</v>
@@ -1077,40 +1188,40 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
         <v>33</v>
       </c>
-      <c r="F3" t="s">
+      <c r="K3" t="s">
         <v>34</v>
       </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>35</v>
       </c>
-      <c r="K3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" t="s">
-        <v>37</v>
-      </c>
       <c r="M3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N3" t="n">
         <v>4.0</v>
       </c>
       <c r="Q3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R3" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="T3" t="n">
         <v>110.0</v>
@@ -1133,40 +1244,40 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" t="s">
         <v>38</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
         <v>39</v>
       </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>40</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>41</v>
       </c>
-      <c r="L4" t="s">
-        <v>42</v>
-      </c>
       <c r="M4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N4" t="n">
         <v>4.0</v>
       </c>
       <c r="Q4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R4" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1192,7 +1303,7 @@
         <v>43</v>
       </c>
       <c r="F5" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1204,25 +1315,25 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="K5" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="L5" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="M5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N5" t="n">
         <v>4.0</v>
       </c>
       <c r="Q5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R5" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1245,10 +1356,10 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1260,25 +1371,25 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="L6" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="M6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N6" t="n">
         <v>4.0</v>
       </c>
       <c r="Q6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1301,10 +1412,10 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="G7" t="s">
         <v>20</v>
@@ -1316,28 +1427,28 @@
         <v>20</v>
       </c>
       <c r="J7" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="K7" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="L7" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="M7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N7" t="n">
         <v>4.0</v>
       </c>
       <c r="P7" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R7" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="T7" t="n">
         <v>110.0</v>
@@ -1360,10 +1471,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1375,25 +1486,25 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="K8" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="L8" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="M8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N8" t="n">
         <v>4.0</v>
       </c>
       <c r="Q8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R8" t="s">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1416,10 +1527,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1431,25 +1542,25 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="L9" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="M9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N9" t="n">
         <v>4.0</v>
       </c>
       <c r="Q9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R9" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1472,10 +1583,10 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>61</v>
+        <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1487,22 +1598,22 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="K10" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="L10" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="M10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N10" t="n">
         <v>4.0</v>
       </c>
       <c r="Q10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R10" t="s">
         <v>20</v>
@@ -1528,40 +1639,40 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" t="s">
+        <v>45</v>
+      </c>
+      <c r="K11" t="s">
+        <v>46</v>
+      </c>
+      <c r="L11" t="s">
         <v>68</v>
       </c>
-      <c r="G11" t="s">
-        <v>20</v>
-      </c>
-      <c r="H11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" t="s">
-        <v>69</v>
-      </c>
-      <c r="K11" t="s">
-        <v>70</v>
-      </c>
-      <c r="L11" t="s">
-        <v>71</v>
-      </c>
       <c r="M11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N11" t="n">
         <v>4.0</v>
       </c>
       <c r="Q11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R11" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1584,10 +1695,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="F12" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1599,28 +1710,28 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="K12" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="L12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N12" t="n">
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="Q12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R12" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1643,10 +1754,10 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F13" t="s">
-        <v>48</v>
+        <v>81</v>
       </c>
       <c r="G13" t="s">
         <v>20</v>
@@ -1661,22 +1772,22 @@
         <v>35</v>
       </c>
       <c r="K13" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="L13" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="M13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N13" t="n">
         <v>4.0</v>
       </c>
       <c r="Q13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R13" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1699,10 +1810,10 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>69</v>
       </c>
       <c r="G14" t="s">
         <v>20</v>
@@ -1714,25 +1825,25 @@
         <v>20</v>
       </c>
       <c r="J14" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="K14" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="L14" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="M14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N14" t="n">
         <v>4.0</v>
       </c>
       <c r="Q14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R14" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1755,10 +1866,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>57</v>
+        <v>86</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1770,25 +1881,25 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="K15" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="L15" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="M15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N15" t="n">
         <v>4.0</v>
       </c>
       <c r="Q15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R15" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1811,10 +1922,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="F16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1826,22 +1937,22 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="K16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L16" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="M16" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N16" t="n">
         <v>4.0</v>
       </c>
       <c r="Q16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R16" t="s">
         <v>20</v>
@@ -1867,10 +1978,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="F17" t="s">
-        <v>57</v>
+        <v>91</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1882,28 +1993,28 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="K17" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
       <c r="L17" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
       <c r="M17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N17" t="n">
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="Q17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R17" t="s">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -1926,10 +2037,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>97</v>
       </c>
       <c r="F18" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -1941,25 +2052,25 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="K18" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="L18" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="M18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N18" t="n">
         <v>4.0</v>
       </c>
       <c r="Q18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R18" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -1982,10 +2093,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="F19" t="s">
-        <v>83</v>
+        <v>45</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -1997,25 +2108,25 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>84</v>
+        <v>46</v>
       </c>
       <c r="K19" t="s">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="L19" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="M19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N19" t="n">
         <v>4.0</v>
       </c>
       <c r="Q19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R19" t="s">
-        <v>20</v>
+        <v>102</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2038,10 +2149,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>88</v>
+        <v>43</v>
       </c>
       <c r="F20" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2053,25 +2164,25 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="K20" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="L20" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="M20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N20" t="n">
         <v>4.0</v>
       </c>
       <c r="Q20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R20" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2094,10 +2205,10 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F21" t="s">
-        <v>48</v>
+        <v>104</v>
       </c>
       <c r="G21" t="s">
         <v>20</v>
@@ -2109,25 +2220,25 @@
         <v>20</v>
       </c>
       <c r="J21" t="s">
-        <v>35</v>
+        <v>105</v>
       </c>
       <c r="K21" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="L21" t="s">
-        <v>46</v>
+        <v>107</v>
       </c>
       <c r="M21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N21" t="n">
         <v>4.0</v>
       </c>
       <c r="Q21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R21" t="s">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2150,10 +2261,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="F22" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2165,28 +2276,28 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="K22" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="L22" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="M22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N22" t="n">
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="Q22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R22" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2209,40 +2320,40 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
+        <v>85</v>
+      </c>
+      <c r="F23" t="s">
+        <v>86</v>
+      </c>
+      <c r="G23" t="s">
+        <v>20</v>
+      </c>
+      <c r="H23" t="s">
+        <v>20</v>
+      </c>
+      <c r="I23" t="s">
+        <v>20</v>
+      </c>
+      <c r="J23" t="s">
+        <v>87</v>
+      </c>
+      <c r="K23" t="s">
         <v>88</v>
       </c>
-      <c r="F23" t="s">
-        <v>101</v>
-      </c>
-      <c r="G23" t="s">
-        <v>20</v>
-      </c>
-      <c r="H23" t="s">
-        <v>20</v>
-      </c>
-      <c r="I23" t="s">
-        <v>20</v>
-      </c>
-      <c r="J23" t="s">
-        <v>90</v>
-      </c>
-      <c r="K23" t="s">
-        <v>91</v>
-      </c>
       <c r="L23" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="M23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N23" t="n">
         <v>4.0</v>
       </c>
       <c r="Q23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R23" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2265,10 +2376,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
       <c r="F24" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2280,25 +2391,25 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="K24" t="s">
-        <v>105</v>
+        <v>57</v>
       </c>
       <c r="L24" t="s">
-        <v>106</v>
+        <v>58</v>
       </c>
       <c r="M24" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N24" t="n">
         <v>4.0</v>
       </c>
       <c r="Q24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R24" t="s">
-        <v>102</v>
+        <v>20</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2321,10 +2432,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="F25" t="s">
-        <v>107</v>
+        <v>45</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2336,25 +2447,25 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="K25" t="s">
-        <v>109</v>
+        <v>47</v>
       </c>
       <c r="L25" t="s">
-        <v>110</v>
+        <v>68</v>
       </c>
       <c r="M25" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N25" t="n">
         <v>4.0</v>
       </c>
       <c r="Q25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R25" t="s">
-        <v>20</v>
+        <v>116</v>
       </c>
       <c r="T25" t="n">
         <v>110.0</v>
@@ -2377,10 +2488,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F26" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2392,25 +2503,25 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="K26" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="L26" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="M26" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N26" t="n">
         <v>4.0</v>
       </c>
       <c r="Q26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R26" t="s">
-        <v>20</v>
+        <v>116</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2433,43 +2544,43 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
+        <v>78</v>
+      </c>
+      <c r="F27" t="s">
+        <v>76</v>
+      </c>
+      <c r="G27" t="s">
+        <v>20</v>
+      </c>
+      <c r="H27" t="s">
+        <v>20</v>
+      </c>
+      <c r="I27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J27" t="s">
         <v>45</v>
       </c>
-      <c r="F27" t="s">
-        <v>36</v>
-      </c>
-      <c r="G27" t="s">
-        <v>20</v>
-      </c>
-      <c r="H27" t="s">
-        <v>20</v>
-      </c>
-      <c r="I27" t="s">
-        <v>20</v>
-      </c>
-      <c r="J27" t="s">
-        <v>35</v>
-      </c>
       <c r="K27" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="L27" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="M27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N27" t="n">
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="Q27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R27" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2492,10 +2603,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="F28" t="s">
-        <v>37</v>
+        <v>120</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2507,25 +2618,25 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="K28" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="L28" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="M28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N28" t="n">
         <v>4.0</v>
       </c>
       <c r="Q28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R28" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2548,10 +2659,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>51</v>
+        <v>97</v>
       </c>
       <c r="F29" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2563,25 +2674,25 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="K29" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="L29" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="M29" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N29" t="n">
         <v>4.0</v>
       </c>
       <c r="Q29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R29" t="s">
-        <v>20</v>
+        <v>121</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2604,10 +2715,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="F30" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2619,25 +2730,25 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="K30" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="L30" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="M30" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N30" t="n">
         <v>4.0</v>
       </c>
       <c r="Q30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R30" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2660,10 +2771,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F31" t="s">
-        <v>37</v>
+        <v>132</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2675,25 +2786,25 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>35</v>
+        <v>133</v>
       </c>
       <c r="K31" t="s">
-        <v>48</v>
+        <v>134</v>
       </c>
       <c r="L31" t="s">
-        <v>49</v>
+        <v>135</v>
       </c>
       <c r="M31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N31" t="n">
         <v>4.0</v>
       </c>
       <c r="Q31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R31" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="T31" t="n">
         <v>110.0</v>
@@ -2716,10 +2827,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>88</v>
+        <v>49</v>
       </c>
       <c r="F32" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2731,28 +2842,28 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="K32" t="s">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="L32" t="s">
-        <v>92</v>
+        <v>53</v>
       </c>
       <c r="M32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N32" t="n">
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="Q32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R32" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2778,7 +2889,7 @@
         <v>67</v>
       </c>
       <c r="F33" t="s">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2790,25 +2901,25 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
+        <v>45</v>
+      </c>
+      <c r="K33" t="s">
+        <v>44</v>
+      </c>
+      <c r="L33" t="s">
         <v>69</v>
       </c>
-      <c r="K33" t="s">
-        <v>70</v>
-      </c>
-      <c r="L33" t="s">
-        <v>71</v>
-      </c>
       <c r="M33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N33" t="n">
         <v>4.0</v>
       </c>
       <c r="Q33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R33" t="s">
-        <v>66</v>
+        <v>139</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2831,10 +2942,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="F34" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2846,25 +2957,25 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>35</v>
+        <v>81</v>
       </c>
       <c r="K34" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="L34" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="M34" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N34" t="n">
         <v>4.0</v>
       </c>
       <c r="Q34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R34" t="s">
-        <v>113</v>
+        <v>20</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2887,10 +2998,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F35" t="s">
-        <v>109</v>
+        <v>141</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -2902,25 +3013,25 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>107</v>
+        <v>142</v>
       </c>
       <c r="K35" t="s">
-        <v>110</v>
+        <v>143</v>
       </c>
       <c r="L35" t="s">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="M35" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N35" t="n">
         <v>4.0</v>
       </c>
       <c r="Q35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R35" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -2943,10 +3054,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="F36" t="s">
-        <v>124</v>
+        <v>146</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -2958,25 +3069,25 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="K36" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="L36" t="s">
-        <v>127</v>
+        <v>149</v>
       </c>
       <c r="M36" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N36" t="n">
         <v>4.0</v>
       </c>
       <c r="Q36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R36" t="s">
-        <v>20</v>
+        <v>145</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -2999,10 +3110,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="F37" t="s">
-        <v>128</v>
+        <v>76</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3014,28 +3125,28 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
-        <v>129</v>
+        <v>45</v>
       </c>
       <c r="K37" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="L37" t="s">
-        <v>130</v>
+        <v>68</v>
       </c>
       <c r="M37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N37" t="n">
         <v>4.0</v>
       </c>
       <c r="P37" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="Q37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R37" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3058,10 +3169,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>45</v>
+        <v>109</v>
       </c>
       <c r="F38" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3073,25 +3184,25 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K38" t="s">
-        <v>36</v>
+        <v>152</v>
       </c>
       <c r="L38" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="M38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N38" t="n">
         <v>4.0</v>
       </c>
       <c r="Q38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R38" t="s">
-        <v>132</v>
+        <v>151</v>
       </c>
       <c r="T38" t="n">
         <v>110.0</v>
@@ -3114,10 +3225,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>24</v>
+        <v>97</v>
       </c>
       <c r="F39" t="s">
-        <v>129</v>
+        <v>33</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3129,25 +3240,25 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>130</v>
+        <v>81</v>
       </c>
       <c r="K39" t="s">
-        <v>128</v>
+        <v>82</v>
       </c>
       <c r="L39" t="s">
-        <v>134</v>
+        <v>154</v>
       </c>
       <c r="M39" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N39" t="n">
         <v>4.0</v>
       </c>
       <c r="Q39" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R39" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3170,11 +3281,11 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
+        <v>61</v>
+      </c>
+      <c r="F40" t="s">
         <v>33</v>
       </c>
-      <c r="F40" t="s">
-        <v>48</v>
-      </c>
       <c r="G40" t="s">
         <v>20</v>
       </c>
@@ -3185,25 +3296,25 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>35</v>
+        <v>154</v>
       </c>
       <c r="K40" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="L40" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="M40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N40" t="n">
         <v>4.0</v>
       </c>
       <c r="Q40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R40" t="s">
-        <v>72</v>
+        <v>155</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3226,10 +3337,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>94</v>
+        <v>31</v>
       </c>
       <c r="F41" t="s">
-        <v>136</v>
+        <v>35</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3241,25 +3352,25 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="K41" t="s">
-        <v>138</v>
+        <v>34</v>
       </c>
       <c r="L41" t="s">
-        <v>139</v>
+        <v>32</v>
       </c>
       <c r="M41" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N41" t="n">
         <v>4.0</v>
       </c>
       <c r="Q41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R41" t="s">
-        <v>135</v>
+        <v>20</v>
       </c>
       <c r="T41" t="n">
         <v>110.0</v>
@@ -3285,7 +3396,7 @@
         <v>67</v>
       </c>
       <c r="F42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3297,28 +3408,28 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="K42" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="L42" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="M42" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N42" t="n">
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="Q42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R42" t="s">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3341,10 +3452,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>77</v>
+        <v>23</v>
       </c>
       <c r="F43" t="s">
-        <v>78</v>
+        <v>158</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3356,25 +3467,25 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>57</v>
+        <v>159</v>
       </c>
       <c r="K43" t="s">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="L43" t="s">
-        <v>58</v>
+        <v>161</v>
       </c>
       <c r="M43" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N43" t="n">
         <v>4.0</v>
       </c>
       <c r="Q43" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R43" t="s">
-        <v>141</v>
+        <v>20</v>
       </c>
       <c r="T43" t="n">
         <v>110.0</v>
@@ -3397,10 +3508,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>88</v>
+        <v>37</v>
       </c>
       <c r="F44" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3412,25 +3523,25 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>90</v>
+        <v>164</v>
       </c>
       <c r="K44" t="s">
-        <v>91</v>
+        <v>165</v>
       </c>
       <c r="L44" t="s">
-        <v>92</v>
+        <v>166</v>
       </c>
       <c r="M44" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N44" t="n">
         <v>4.0</v>
       </c>
       <c r="Q44" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R44" t="s">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3453,10 +3564,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>75</v>
+        <v>109</v>
       </c>
       <c r="F45" t="s">
-        <v>48</v>
+        <v>168</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3468,25 +3579,25 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>35</v>
+        <v>169</v>
       </c>
       <c r="K45" t="s">
-        <v>36</v>
+        <v>170</v>
       </c>
       <c r="L45" t="s">
-        <v>46</v>
+        <v>171</v>
       </c>
       <c r="M45" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N45" t="n">
         <v>4.0</v>
       </c>
       <c r="Q45" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R45" t="s">
-        <v>144</v>
+        <v>167</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3509,10 +3620,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>45</v>
+        <v>97</v>
       </c>
       <c r="F46" t="s">
-        <v>48</v>
+        <v>173</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3524,25 +3635,25 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>35</v>
+        <v>174</v>
       </c>
       <c r="K46" t="s">
-        <v>36</v>
+        <v>175</v>
       </c>
       <c r="L46" t="s">
-        <v>46</v>
+        <v>176</v>
       </c>
       <c r="M46" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N46" t="n">
         <v>4.0</v>
       </c>
       <c r="Q46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R46" t="s">
-        <v>144</v>
+        <v>172</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3565,43 +3676,43 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
+        <v>49</v>
+      </c>
+      <c r="F47" t="s">
+        <v>178</v>
+      </c>
+      <c r="G47" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" t="s">
+        <v>20</v>
+      </c>
+      <c r="I47" t="s">
+        <v>20</v>
+      </c>
+      <c r="J47" t="s">
         <v>51</v>
       </c>
-      <c r="F47" t="s">
-        <v>145</v>
-      </c>
-      <c r="G47" t="s">
-        <v>20</v>
-      </c>
-      <c r="H47" t="s">
-        <v>20</v>
-      </c>
-      <c r="I47" t="s">
-        <v>20</v>
-      </c>
-      <c r="J47" t="s">
-        <v>146</v>
-      </c>
       <c r="K47" t="s">
-        <v>147</v>
+        <v>52</v>
       </c>
       <c r="L47" t="s">
-        <v>148</v>
+        <v>53</v>
       </c>
       <c r="M47" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N47" t="n">
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="Q47" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R47" t="s">
-        <v>20</v>
+        <v>177</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3624,10 +3735,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="F48" t="s">
-        <v>49</v>
+        <v>181</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3639,25 +3750,25 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>35</v>
+        <v>182</v>
       </c>
       <c r="K48" t="s">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="L48" t="s">
-        <v>46</v>
+        <v>184</v>
       </c>
       <c r="M48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N48" t="n">
         <v>4.0</v>
       </c>
       <c r="Q48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R48" t="s">
-        <v>132</v>
+        <v>180</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3680,10 +3791,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="F49" t="s">
-        <v>151</v>
+        <v>186</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3695,25 +3806,25 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>90</v>
+        <v>187</v>
       </c>
       <c r="K49" t="s">
-        <v>91</v>
+        <v>188</v>
       </c>
       <c r="L49" t="s">
-        <v>92</v>
+        <v>189</v>
       </c>
       <c r="M49" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N49" t="n">
         <v>4.0</v>
       </c>
       <c r="Q49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R49" t="s">
-        <v>150</v>
+        <v>185</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3736,10 +3847,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="F50" t="s">
-        <v>153</v>
+        <v>46</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3751,25 +3862,25 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>154</v>
+        <v>45</v>
       </c>
       <c r="K50" t="s">
-        <v>155</v>
+        <v>44</v>
       </c>
       <c r="L50" t="s">
-        <v>156</v>
+        <v>69</v>
       </c>
       <c r="M50" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N50" t="n">
         <v>4.0</v>
       </c>
       <c r="Q50" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R50" t="s">
-        <v>152</v>
+        <v>190</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3792,10 +3903,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="F51" t="s">
-        <v>35</v>
+        <v>191</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3807,25 +3918,25 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>36</v>
+        <v>192</v>
       </c>
       <c r="K51" t="s">
-        <v>46</v>
+        <v>193</v>
       </c>
       <c r="L51" t="s">
-        <v>37</v>
+        <v>194</v>
       </c>
       <c r="M51" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N51" t="n">
         <v>4.0</v>
       </c>
       <c r="Q51" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="R51" t="s">
-        <v>157</v>
+        <v>20</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3836,7 +3947,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>158</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
least and most sum solution added
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="154">
   <si>
     <t>Sr. No</t>
   </si>
@@ -83,28 +83,160 @@
     <t>09030201</t>
   </si>
   <si>
+    <t>Ans: Truck, Bus, Car, Bicycle&lt;br&gt;From the given graph we can see that, $Truck$, $Bus$, $Car$, $Bicycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Truck, Bus, Car, Bicycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Truck$, $Bus$, $Car$, $Bicycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck, Bus, Car, Bicycle&lt;br&gt;#ट्रक, बस, कार, सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Motorcycle&lt;br&gt;#कार, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car, Bus, Truck, Scooter&lt;br&gt;#कार, बस, ट्रक, दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Bus, Truck, Motorcycle&lt;br&gt;#सायकल, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
+  </si>
+  <si>
+    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 9$&lt;br&gt;No. of travellers using the Bus  $= 9$&lt;br&gt;No. of travellers using the Car  $= 7$&lt;br&gt;No. of travellers using the Bicycle  $= 2$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$9 + 9 + 7 + 2 = 27$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;Bus या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 7$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$9 + 9 + 7 + 2 = 27$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$27$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$28$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$26$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$29$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $154$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 94$&lt;br&gt;No. of travellers using the vehicle least $= 60$&lt;br&gt;By taking the sum of these two numbers we get  &lt;br&gt;$94 + 60 = 154$  is the answer.&lt;br&gt;#उत्तर : $154$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 94$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 60$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी बेरीज घेऊन आपल्याला &lt;br&gt;$94 + 60 = 154$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
     <t>How many are the total travellers travelling by the vehicles used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे वाहन आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्यातील प्रवाशांची एकूण संख्या किती आहे?&lt;br&gt;</t>
   </si>
   <si>
-    <t>$12900$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$12902$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$12901$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$12898$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_1.png</t>
-  </si>
-  <si>
-    <t>2022.chinmay.chaudhari@ves.ac.in</t>
+    <t>$154$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$152$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$155$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$153$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 61$&lt;br&gt;No. of travellers using the Scooter  $= 89$&lt;br&gt;No. of travellers using the Motorcycle  $= 94$&lt;br&gt;No. of travellers using the Bicycle  $= 60$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$61 + 89 + 94 + 60 = 304$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;Scooter या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 89$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 94$&lt;br&gt;Bicycle या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 60$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$61 + 89 + 94 + 60 = 304$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$304$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$305$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$302$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$306$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of travelers by different means.</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
+  </si>
+  <si>
+    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
   </si>
   <si>
     <t>How many different vehicles do travellers use?&lt;br&gt;#प्रवाशांनी किती विविध वाहने वापरतात?&lt;br&gt;</t>
@@ -113,490 +245,232 @@
     <t>$4$ &lt;br&gt;</t>
   </si>
   <si>
+    <t>$2$ &lt;br&gt;</t>
+  </si>
+  <si>
     <t>$6$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>$2$ &lt;br&gt;</t>
+    <t>$5$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9$&lt;br&gt;No. of travellers using the vehicle least $= 4$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9 - 4 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9 - 4 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$7$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $12$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9$&lt;br&gt;No. of travellers using the vehicle least $= 3$&lt;br&gt;By taking the sum of these two numbers we get  &lt;br&gt;$9 + 3 = 12$  is the answer.&lt;br&gt;#उत्तर : $12$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी बेरीज घेऊन आपल्याला &lt;br&gt;$9 + 3 = 12$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$12$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$14$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$11$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 1$ vehicles.&lt;br&gt;#$1$ एकक $= 1$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 9$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 6$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 5$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$9 + 6 + 5 = 20$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$9 + 6 + 5 = 20$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>How much is the total of travellers for top 3 values?</t>
+  </si>
+  <si>
+    <t>$20$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$22$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$21$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$18$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bicycle $= 3800$&lt;br&gt;No. of travellers using the Truck  $= 200$&lt;br&gt;No. of travellers using the Bus  $= 6100$&lt;br&gt;No. of travellers using the Car  $= 800$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$3800 + 200 + 6100 + 800 = 10900$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bicycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;Truck या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 200$&lt;br&gt;Bus या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 6100$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 800$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$3800 + 200 + 6100 + 800 = 10900$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10900$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10899$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10898$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10902$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 6100$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 3800$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 800$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$6100 + 3800 + 800 = 10700$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6100$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 800$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$6100 + 3800 + 800 = 10700$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10700$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10699$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10698$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$10702$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Bicycle, Truck, Bus, Car&lt;br&gt;From the given graph we can see that, $Bicycle$, $Truck$, $Bus$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bicycle, Truck, Bus, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bicycle$, $Truck$, $Bus$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Bicycle, Truck, Bus, Car&lt;br&gt;#सायकल, ट्रक, बस, कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$1$ unit $= 1000$ vehicles.&lt;br&gt;#$1$ एकक $= 1000$ वाहने &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: Motorcycle, Truck, Bicycle, Car&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Truck$, $Bicycle$, $Car$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Truck, Bicycle, Car&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Truck$, $Bicycle$, $Car$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Motorcycle, Truck, Bicycle, Car&lt;br&gt;#मोटरसायकल, ट्रक, सायकल, कार&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
+  </si>
+  <si>
+    <t>Ans: $10700$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9500$&lt;br&gt;No. of travellers using the vehicle least $= 1200$&lt;br&gt;By taking the sum of these two numbers we get  &lt;br&gt;$9500 + 1200 = 10700$  is the answer.&lt;br&gt;#उत्तर : $10700$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9500$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1200$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी बेरीज घेऊन आपल्याला &lt;br&gt;$9500 + 1200 = 10700$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $8300$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9500$&lt;br&gt;No. of travellers using the vehicle least $= 1200$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9500 - 1200 = 8300$  is the answer.&lt;br&gt;#उत्तर : $8300$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9500$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1200$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9500 - 1200 = 8300$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8300$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8298$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8302$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8301$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
+  </si>
+  <si>
+    <t>Ans: $8$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 8$&lt;br&gt;No. of travellers using the vehicle least $= 0$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$8 - 0 = 8$  is the answer.&lt;br&gt;#उत्तर : $8$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 0$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$8 - 0 = 8$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$8$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$9$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 83$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 79$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 74$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$83 + 79 + 74 = 236$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 79$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 74$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$83 + 79 + 74 = 236$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$236$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$237$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$238$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$234$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
   </si>
   <si>
     <t>$3$ &lt;br&gt;</t>
   </si>
   <si>
-    <t>Ans: $6700$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9800$&lt;br&gt;No. of travellers using the vehicle least $= 3100$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9800 - 3100 = 6700$  is the answer.&lt;br&gt;#उत्तर : $6700$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9800$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3100$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9800 - 3100 = 6700$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the difference in the number of travellers between the vehicle used most and least?&lt;br&gt;#प्रवासासाठी सगळ्यात जास्त वापरले जाणारे आणि सगळ्यात कमी वापरले जाणारे वाहन, यांच्या प्रवाशातील फरकाची संख्या किती आहे?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6700$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6699$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6701$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$6698$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most?&lt;br&gt;#कोणता वाहन सर्वाधिक वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle&lt;br&gt;#मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car&lt;br&gt;#कार&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus&lt;br&gt;#बस&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Car, Bicycle, Scooter, Motorcycle&lt;br&gt;From the given graph we can see that, $Car$, $Bicycle$, $Scooter$, $Motorcycle$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Car, Bicycle, Scooter, Motorcycle&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Car$, $Bicycle$, $Scooter$, $Motorcycle$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which are the different vehicles used by travellers?&lt;br&gt;#प्रवासासाठी वापरलेली वेगवेगळी वाहने कोणती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bicycle, Scooter, Motorcycle&lt;br&gt;#कार, सायकल, दुचाकी, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Motorcycle&lt;br&gt;#कार, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Car, Bus, Truck, Scooter&lt;br&gt;#कार, बस, ट्रक, दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle, Bus, Truck, Motorcycle&lt;br&gt;#सायकल, बस, ट्रक, मोटरसायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scale used in this graph is?&lt;br&gt;#या स्तंभालेखासाठी वापरलेले प्रमाण . . . .  आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 10$ vehicles.&lt;br&gt;#$1$ एकक $= 10$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 25$ vehicles.&lt;br&gt;#$1$ एकक $= 25$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 250$ vehicles.&lt;br&gt;#$1$ एकक $= 250$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 150$ vehicles.&lt;br&gt;#$1$ एकक $= 150$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_2.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Car $= 92$&lt;br&gt;No. of travellers using the Bicycle  $= 63$&lt;br&gt;No. of travellers using the Scooter  $= 99$&lt;br&gt;No. of travellers using the Truck  $= 41$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$92 + 63 + 99 + 41 = 295$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Car या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 92$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 63$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 99$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 41$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$92 + 63 + 99 + 41 = 295$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How many are the total travellers?&lt;br&gt;#एकूण प्रवासी किती आहेत?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$295$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$296$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$294$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$293$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Truck$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= ट्रक$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least for travelling?&lt;br&gt;#प्रवासासाठी सर्वात कमी वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Truck&lt;br&gt;#ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bicycle&lt;br&gt;#सायकल&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$140$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$138$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$141$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$139$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used most for travelling?&lt;br&gt;#प्रवासासाठी सर्वात जास्त वापर कोणत्या वाहनाचा होतो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Scooter&lt;br&gt;#दुचाकी &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Motorcycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= मोटरसायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Which vehicle is used least?&lt;br&gt;#कोणता वाहन सर्वाधिक कमी वापरला जातो?&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_3.png</t>
-  </si>
-  <si>
-    <t>Ans: $5$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 5$&lt;br&gt;No. of travellers using the vehicle least $= 0$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$5 - 0 = 5$  is the answer.&lt;br&gt;#उत्तर : $5$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 5$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 0$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$5 - 0 = 5$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$7$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>As mentioned in the problem statement, the bar graph shows the number of travellers, travelling by different vehicles.&lt;br&gt;#प्रश्नात दिल्यानुसार वेगवेगळ्या वाहनातून प्रवास करणाऱ्या प्रवाशांची संख्या दाखविण्यासाठी हे स्तंभालेख आहे.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph is for?&lt;br&gt;#हा स्तंभालेख . . . . . साठी आहे. &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of travelers by different means.</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of students by different means.&lt;br&gt;#हा स्तंभालेख विविध स्थानिकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of teachers by different means.&lt;br&gt;#हा स्तंभालेख विविध शिक्षकांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>This bar graph represents the number of principal by different means.&lt;br&gt;#हा स्तंभालेख विविध प्रमुखांची संख्या दर्शवितोय.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 210$&lt;br&gt;No. of travellers using the Bicycle  $= 370$&lt;br&gt;No. of travellers using the Motorcycle  $= 200$&lt;br&gt;No. of travellers using the Car  $= 250$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$210 + 370 + 200 + 250 = 1030$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 210$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 200$&lt;br&gt;Car या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 250$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$210 + 370 + 200 + 250 = 1030$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1030$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1031$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1029$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1028$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_4.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 370$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 250$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 210$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$370 + 250 + 210 = 830$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 250$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 210$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$370 + 250 + 210 = 830$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>How much is the total of travellers for top 3 values?</t>
-  </si>
-  <si>
-    <t>$830$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$829$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$828$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$831$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $170$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 370$&lt;br&gt;No. of travellers using the vehicle least $= 200$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$370 - 200 = 170$  is the answer.&lt;br&gt;#उत्तर : $170$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 370$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 200$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$370 - 200 = 170$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$170$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$169$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$168$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$172$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 130$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 940$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$130 + 940 = 1070$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 130$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 940$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$130 + 940 = 1070$  हे उत्तर मिळते.&lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 74$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 79$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$74 + 79 = 153$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 74$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 79$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$74 + 79 = 153$  हे उत्तर मिळते.&lt;br&gt;</t>
   </si>
   <si>
     <t>How many are the total of travellers travelling by the second and third most used vehicle?&lt;br&gt;#दोन क्रमांकाचे सर्वात जास्त वापरले जाणारे  वाहन आणि तीन क्रमांकाचे सर्वात जास्त वापरले जाणारे वाहन यांची मिळून एकूण प्रवाशांची एकूण संख्या किती?&lt;br&gt;</t>
   </si>
   <si>
-    <t>$1070$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1068$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1071$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1072$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_5.png</t>
-  </si>
-  <si>
-    <t>$1$ unit $= 100$ vehicles.&lt;br&gt;#$1$ एकक $= 100$ वाहने &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Car$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= कार$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Scooter$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= दुचाकी$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_6.png</t>
-  </si>
-  <si>
-    <t>Ans: Bus, Bicycle, Car, Scooter&lt;br&gt;From the given graph we can see that, $Bus$, $Bicycle$, $Car$, $Scooter$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bus, Bicycle, Car, Scooter&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bus$, $Bicycle$, $Car$, $Scooter$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus, Bicycle, Car, Scooter&lt;br&gt;#बस, सायकल, कार, दुचाकी&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 9300$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 8300$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 4000$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$9300 + 8300 + 4000 = 21600$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 8300$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 4000$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$9300 + 8300 + 4000 = 21600$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$21600$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$21602$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$21601$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$21599$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 3800$&lt;br&gt;No. of travellers using the Bicycle  $= 4000$&lt;br&gt;No. of travellers using the Car  $= 8300$&lt;br&gt;No. of travellers using the Scooter  $= 9300$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$3800 + 4000 + 8300 + 9300 = 25400$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;Bicycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 4000$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 8300$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$3800 + 4000 + 8300 + 9300 = 25400$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$25400$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$25401$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$25398$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$25399$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $5500$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 9300$&lt;br&gt;No. of travellers using the vehicle least $= 3800$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$9300 - 3800 = 5500$  is the answer.&lt;br&gt;#उत्तर : $5500$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 9300$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3800$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$9300 - 3800 = 5500$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5500$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5498$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5502$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$5501$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Bus, Car, Motorcycle, Truck&lt;br&gt;From the given graph we can see that, $Bus$, $Car$, $Motorcycle$, $Truck$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Bus, Car, Motorcycle, Truck&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Bus$, $Car$, $Motorcycle$, $Truck$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Bus, Car, Motorcycle, Truck&lt;br&gt;#बस, कार, मोटरसायकल, ट्रक&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_7.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 98$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 69$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 61$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$98 + 69 + 61 = 228$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 69$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 61$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$98 + 69 + 61 = 228$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$228$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$230$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$229$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$226$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $44$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 98$&lt;br&gt;No. of travellers using the vehicle least $= 54$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$98 - 54 = 44$  is the answer.&lt;br&gt;#उत्तर : $44$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 98$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 54$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$98 - 54 = 44$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$44$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$45$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$43$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$46$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_8.png</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 1$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 2$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$1 + 2 = 3$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$1 + 2 = 3$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 3$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 2$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 1$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$3 + 2 + 1 = 6$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$3 + 2 + 1 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$8$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bus $= 0$&lt;br&gt;No. of travellers using the Car  $= 1$&lt;br&gt;No. of travellers using the Motorcycle  $= 2$&lt;br&gt;No. of travellers using the Scooter  $= 3$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$0 + 1 + 2 + 3 = 6$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bus या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 0$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 1$&lt;br&gt;Motorcycle या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2$&lt;br&gt;Scooter या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 3$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$0 + 1 + 2 + 3 = 6$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the least used vehicle is $= Bicycle$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात कमी वापरलेल्या वाहनासाठी प्रवाशांची संख्या $= सायकल$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_9.png</t>
-  </si>
-  <si>
-    <t>$117$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$119$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$115$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$118$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: $69$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 93$&lt;br&gt;No. of travellers using the vehicle least $= 24$&lt;br&gt;By taking the difference of these two numbers we get  &lt;br&gt;$93 - 24 = 69$  is the answer.&lt;br&gt;#उत्तर : $69$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 93$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 24$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी फरक  घेऊन आपल्याला &lt;br&gt;$93 - 24 = 69$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$69$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$70$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$68$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$71$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 51$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 92$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$51 + 92 = 143$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 51$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 92$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$51 + 92 = 143$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$143$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$142$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$145$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$144$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 93$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 92$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 51$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$93 + 92 + 51 = 236$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 93$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 92$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 51$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$93 + 92 + 51 = 236$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$236$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$238$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$237$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$235$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Ans: Motorcycle, Scooter, Truck, Bus&lt;br&gt;From the given graph we can see that, $Motorcycle$, $Scooter$, $Truck$, $Bus$ these are the different vehicles used is the answer.&lt;br&gt;#उत्तर : Motorcycle, Scooter, Truck, Bus&lt;br&gt;दिलेल्या स्तंभालेखानुसार $Motorcycle$, $Scooter$, $Truck$, $Bus$ अशी वाहने वापरली जातात हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>Motorcycle, Scooter, Truck, Bus&lt;br&gt;#मोटरसायकल, दुचाकी, ट्रक, बस&lt;br&gt;</t>
+    <t>$151$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Bicycle $= 6$&lt;br&gt;No. of travellers using the Motorcycle  $= 74$&lt;br&gt;No. of travellers using the Car  $= 79$&lt;br&gt;No. of travellers using the Truck  $= 83$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$6 + 74 + 79 + 83 = 242$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Bicycle या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;Motorcycle या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 74$&lt;br&gt;Car या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 79$&lt;br&gt;Truck या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$6 + 74 + 79 + 83 = 242$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$242$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$240$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$243$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$241$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>Ans: $89$ &lt;br&gt;From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most $= 83$&lt;br&gt;No. of travellers using the vehicle least $= 6$&lt;br&gt;By taking the sum of these two numbers we get  &lt;br&gt;$83 + 6 = 89$  is the answer.&lt;br&gt;#उत्तर : $89$&lt;br&gt;दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 83$&lt;br&gt;सगळ्यात कमी वापरलेल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 6$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची वेगवेगळी बेरीज घेऊन आपल्याला &lt;br&gt;$83 + 6 = 89$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$89$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$87$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$88$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$91$ &lt;br&gt;</t>
   </si>
   <si>
     <t>/Users/chinmay/Documents/ganit/ganitt/img/chart_10.png</t>
   </si>
   <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers travelling by most used vehicle is $= 810$  &lt;br&gt;No. of travellers travelling by second most used vehicle is $= 790$  &lt;br&gt;No. of travellers travelling by third most used vehicle is $= 440$  &lt;br&gt;By taking the addition of these three numbers we get  &lt;br&gt;$810 + 790 + 440 = 2040$  is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 810$&lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 790$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 440$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$810 + 790 + 440 = 2040$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2040$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2042$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2039$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$2038$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the second most used vehicle is $= 440$ &lt;br&gt;No. of travellers using the third most used vehicle is $= 790$ &lt;br&gt;By taking the addition of these two numbers we get  &lt;br&gt;$440 + 790 = 1230$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;दोन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 440$&lt;br&gt;तीन क्रमांकाचे सर्वात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= 790$&lt;br&gt;या दोन्ही प्रवाशांच्या संख्यांची बेरीज  घेऊन आपल्याला &lt;br&gt;$440 + 790 = 1230$  हे उत्तर मिळते.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1230$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1229$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1228$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1231$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the vehicle most is $= Bus$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;सगळ्यात जास्त वापरल्या जाणाऱ्या वाहनासाठी प्रवाशांची संख्या $= बस$ आहे, हे उत्तर.&lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1060$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1058$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1059$ &lt;br&gt;</t>
-  </si>
-  <si>
-    <t>$1062$ &lt;br&gt;</t>
+    <t>From the given graph we can see that&lt;br&gt;No. of travellers using the Truck $= 4100$&lt;br&gt;No. of travellers using the Car  $= 5100$&lt;br&gt;No. of travellers using the Scooter  $= 2900$&lt;br&gt;No. of travellers using the Bus  $= 1000$&lt;br&gt;By taking the total of these numbers we get  &lt;br&gt;$4100 + 5100 + 2900 + 1000 = 13100$ is the answer.&lt;br&gt;#दिलेल्या स्तंभालेखानुसार &lt;br&gt;Truck या पहिल्या वाहनासाठी प्रवाशांची संख्या $= 4100$&lt;br&gt;Car या दुसऱ्या वाहनासाठी प्रवाशांची संख्या $= 5100$&lt;br&gt;Scooter या तिसऱ्या वाहनासाठी प्रवाशांची संख्या $= 2900$&lt;br&gt;Bus या . . . . . . वाहनासाठी प्रवाशांची संख्या $= 1000$&lt;br&gt;या सर्व  प्रवासी संख्येची बेरीज  घेऊन आपल्याला &lt;br&gt;$4100 + 5100 + 2900 + 1000 = 13100$  हे उत्तर मिळते.&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$13100$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$13099$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$13101$ &lt;br&gt;</t>
+  </si>
+  <si>
+    <t>$13102$ &lt;br&gt;</t>
   </si>
   <si>
     <t>****</t>
@@ -1037,7 +911,7 @@
     <col min="3" max="3" width="12.4375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="13.66015625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="193.7734375" customWidth="true" bestFit="true"/>
-    <col min="6" max="6" width="65.68359375" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="63.5" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="16.42578125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="16.42578125" customWidth="true" bestFit="true"/>
@@ -1129,43 +1003,43 @@
         <v>22</v>
       </c>
       <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P2" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>31</v>
+      </c>
+      <c r="R2" t="s">
         <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
-      </c>
-      <c r="M2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>30</v>
-      </c>
-      <c r="R2" t="s">
-        <v>20</v>
       </c>
       <c r="T2" t="n">
         <v>110.0</v>
@@ -1188,40 +1062,40 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>31</v>
+      </c>
+      <c r="R3" t="s">
         <v>32</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" t="s">
-        <v>34</v>
-      </c>
-      <c r="L3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M3" t="s">
-        <v>28</v>
-      </c>
-      <c r="N3" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>30</v>
-      </c>
-      <c r="R3" t="s">
-        <v>20</v>
       </c>
       <c r="T3" t="n">
         <v>110.0</v>
@@ -1244,40 +1118,40 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L4" t="s">
+        <v>43</v>
+      </c>
+      <c r="M4" t="s">
+        <v>29</v>
+      </c>
+      <c r="N4" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>31</v>
+      </c>
+      <c r="R4" t="s">
         <v>38</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" t="s">
-        <v>39</v>
-      </c>
-      <c r="K4" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>30</v>
-      </c>
-      <c r="R4" t="s">
-        <v>36</v>
       </c>
       <c r="T4" t="n">
         <v>110.0</v>
@@ -1300,10 +1174,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1315,25 +1189,25 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K5" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="L5" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N5" t="n">
         <v>4.0</v>
       </c>
       <c r="Q5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R5" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="T5" t="n">
         <v>110.0</v>
@@ -1356,10 +1230,10 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1371,25 +1245,25 @@
         <v>20</v>
       </c>
       <c r="J6" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="K6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="L6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N6" t="n">
         <v>4.0</v>
       </c>
       <c r="Q6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="T6" t="n">
         <v>110.0</v>
@@ -1412,43 +1286,43 @@
         <v>22</v>
       </c>
       <c r="E7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" t="s">
+        <v>53</v>
+      </c>
+      <c r="L7" t="s">
         <v>54</v>
       </c>
-      <c r="F7" t="s">
+      <c r="M7" t="s">
+        <v>29</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P7" t="s">
         <v>55</v>
       </c>
-      <c r="G7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" t="s">
-        <v>56</v>
-      </c>
-      <c r="K7" t="s">
-        <v>57</v>
-      </c>
-      <c r="L7" t="s">
-        <v>58</v>
-      </c>
-      <c r="M7" t="s">
-        <v>28</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P7" t="s">
-        <v>59</v>
-      </c>
       <c r="Q7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R7" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="T7" t="n">
         <v>110.0</v>
@@ -1471,10 +1345,10 @@
         <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
@@ -1486,25 +1360,25 @@
         <v>20</v>
       </c>
       <c r="J8" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="K8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="L8" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="M8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N8" t="n">
         <v>4.0</v>
       </c>
       <c r="Q8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="T8" t="n">
         <v>110.0</v>
@@ -1527,10 +1401,10 @@
         <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
@@ -1542,25 +1416,25 @@
         <v>20</v>
       </c>
       <c r="J9" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="L9" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="M9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N9" t="n">
         <v>4.0</v>
       </c>
       <c r="Q9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="T9" t="n">
         <v>110.0</v>
@@ -1583,10 +1457,10 @@
         <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>37</v>
       </c>
       <c r="G10" t="s">
         <v>20</v>
@@ -1598,25 +1472,25 @@
         <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="K10" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
       <c r="L10" t="s">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="M10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N10" t="n">
         <v>4.0</v>
       </c>
       <c r="Q10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R10" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="T10" t="n">
         <v>110.0</v>
@@ -1639,10 +1513,10 @@
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
         <v>20</v>
@@ -1654,25 +1528,25 @@
         <v>20</v>
       </c>
       <c r="J11" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="K11" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="L11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N11" t="n">
         <v>4.0</v>
       </c>
       <c r="Q11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R11" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="T11" t="n">
         <v>110.0</v>
@@ -1695,10 +1569,10 @@
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="G12" t="s">
         <v>20</v>
@@ -1710,28 +1584,28 @@
         <v>20</v>
       </c>
       <c r="J12" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="L12" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="M12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N12" t="n">
         <v>4.0</v>
       </c>
       <c r="P12" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="Q12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R12" t="s">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="T12" t="n">
         <v>110.0</v>
@@ -1754,10 +1628,10 @@
         <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="G13" t="s">
         <v>20</v>
@@ -1769,25 +1643,25 @@
         <v>20</v>
       </c>
       <c r="J13" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="K13" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="L13" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="M13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N13" t="n">
         <v>4.0</v>
       </c>
       <c r="Q13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R13" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="T13" t="n">
         <v>110.0</v>
@@ -1810,10 +1684,10 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="F14" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G14" t="s">
         <v>20</v>
@@ -1825,25 +1699,25 @@
         <v>20</v>
       </c>
       <c r="J14" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="K14" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="L14" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="M14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N14" t="n">
         <v>4.0</v>
       </c>
       <c r="Q14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R14" t="s">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="T14" t="n">
         <v>110.0</v>
@@ -1866,10 +1740,10 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="F15" t="s">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="G15" t="s">
         <v>20</v>
@@ -1881,25 +1755,25 @@
         <v>20</v>
       </c>
       <c r="J15" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="K15" t="s">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="L15" t="s">
-        <v>89</v>
+        <v>48</v>
       </c>
       <c r="M15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N15" t="n">
         <v>4.0</v>
       </c>
       <c r="Q15" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R15" t="s">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="T15" t="n">
         <v>110.0</v>
@@ -1922,10 +1796,10 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G16" t="s">
         <v>20</v>
@@ -1937,22 +1811,22 @@
         <v>20</v>
       </c>
       <c r="J16" t="s">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="K16" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="L16" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="M16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N16" t="n">
         <v>4.0</v>
       </c>
       <c r="Q16" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R16" t="s">
         <v>20</v>
@@ -1978,10 +1852,10 @@
         <v>22</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G17" t="s">
         <v>20</v>
@@ -1993,28 +1867,28 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="K17" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="L17" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="M17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N17" t="n">
         <v>4.0</v>
       </c>
       <c r="P17" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="Q17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R17" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="T17" t="n">
         <v>110.0</v>
@@ -2037,10 +1911,10 @@
         <v>22</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="F18" t="s">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="G18" t="s">
         <v>20</v>
@@ -2052,25 +1926,25 @@
         <v>20</v>
       </c>
       <c r="J18" t="s">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="K18" t="s">
-        <v>100</v>
+        <v>66</v>
       </c>
       <c r="L18" t="s">
-        <v>101</v>
+        <v>67</v>
       </c>
       <c r="M18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N18" t="n">
         <v>4.0</v>
       </c>
       <c r="Q18" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R18" t="s">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="T18" t="n">
         <v>110.0</v>
@@ -2093,10 +1967,10 @@
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="F19" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G19" t="s">
         <v>20</v>
@@ -2108,25 +1982,25 @@
         <v>20</v>
       </c>
       <c r="J19" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="K19" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="L19" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="M19" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N19" t="n">
         <v>4.0</v>
       </c>
       <c r="Q19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R19" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="T19" t="n">
         <v>110.0</v>
@@ -2149,10 +2023,10 @@
         <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F20" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G20" t="s">
         <v>20</v>
@@ -2164,25 +2038,25 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="K20" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="L20" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="M20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N20" t="n">
         <v>4.0</v>
       </c>
       <c r="Q20" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R20" t="s">
-        <v>102</v>
+        <v>32</v>
       </c>
       <c r="T20" t="n">
         <v>110.0</v>
@@ -2205,40 +2079,40 @@
         <v>22</v>
       </c>
       <c r="E21" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" t="s">
+        <v>20</v>
+      </c>
+      <c r="H21" t="s">
+        <v>20</v>
+      </c>
+      <c r="I21" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" t="s">
+        <v>35</v>
+      </c>
+      <c r="K21" t="s">
+        <v>36</v>
+      </c>
+      <c r="L21" t="s">
         <v>37</v>
       </c>
-      <c r="F21" t="s">
-        <v>104</v>
-      </c>
-      <c r="G21" t="s">
-        <v>20</v>
-      </c>
-      <c r="H21" t="s">
-        <v>20</v>
-      </c>
-      <c r="I21" t="s">
-        <v>20</v>
-      </c>
-      <c r="J21" t="s">
-        <v>105</v>
-      </c>
-      <c r="K21" t="s">
-        <v>106</v>
-      </c>
-      <c r="L21" t="s">
-        <v>107</v>
-      </c>
       <c r="M21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N21" t="n">
         <v>4.0</v>
       </c>
       <c r="Q21" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R21" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="T21" t="n">
         <v>110.0</v>
@@ -2261,10 +2135,10 @@
         <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>109</v>
+        <v>50</v>
       </c>
       <c r="F22" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="G22" t="s">
         <v>20</v>
@@ -2276,28 +2150,28 @@
         <v>20</v>
       </c>
       <c r="J22" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="K22" t="s">
-        <v>112</v>
+        <v>88</v>
       </c>
       <c r="L22" t="s">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="M22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N22" t="n">
         <v>4.0</v>
       </c>
       <c r="P22" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="Q22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R22" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="T22" t="n">
         <v>110.0</v>
@@ -2320,10 +2194,10 @@
         <v>22</v>
       </c>
       <c r="E23" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="F23" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="G23" t="s">
         <v>20</v>
@@ -2335,25 +2209,25 @@
         <v>20</v>
       </c>
       <c r="J23" t="s">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="K23" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="L23" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="M23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N23" t="n">
         <v>4.0</v>
       </c>
       <c r="Q23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R23" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="T23" t="n">
         <v>110.0</v>
@@ -2376,10 +2250,10 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="F24" t="s">
-        <v>115</v>
+        <v>47</v>
       </c>
       <c r="G24" t="s">
         <v>20</v>
@@ -2391,25 +2265,25 @@
         <v>20</v>
       </c>
       <c r="J24" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="K24" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="L24" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="M24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N24" t="n">
         <v>4.0</v>
       </c>
       <c r="Q24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R24" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="T24" t="n">
         <v>110.0</v>
@@ -2432,10 +2306,10 @@
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="F25" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="G25" t="s">
         <v>20</v>
@@ -2447,25 +2321,25 @@
         <v>20</v>
       </c>
       <c r="J25" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="K25" t="s">
-        <v>47</v>
+        <v>97</v>
       </c>
       <c r="L25" t="s">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="M25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N25" t="n">
         <v>4.0</v>
       </c>
       <c r="Q25" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R25" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="T25" t="n">
         <v>110.0</v>
@@ -2488,10 +2362,10 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="F26" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G26" t="s">
         <v>20</v>
@@ -2503,25 +2377,25 @@
         <v>20</v>
       </c>
       <c r="J26" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="K26" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="L26" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="M26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N26" t="n">
         <v>4.0</v>
       </c>
       <c r="Q26" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R26" t="s">
-        <v>116</v>
+        <v>84</v>
       </c>
       <c r="T26" t="n">
         <v>110.0</v>
@@ -2544,10 +2418,10 @@
         <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>78</v>
+        <v>39</v>
       </c>
       <c r="F27" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="G27" t="s">
         <v>20</v>
@@ -2559,28 +2433,28 @@
         <v>20</v>
       </c>
       <c r="J27" t="s">
-        <v>45</v>
+        <v>101</v>
       </c>
       <c r="K27" t="s">
-        <v>46</v>
+        <v>102</v>
       </c>
       <c r="L27" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="M27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N27" t="n">
         <v>4.0</v>
       </c>
       <c r="P27" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="Q27" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R27" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="T27" t="n">
         <v>110.0</v>
@@ -2603,10 +2477,10 @@
         <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="F28" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="G28" t="s">
         <v>20</v>
@@ -2618,25 +2492,25 @@
         <v>20</v>
       </c>
       <c r="J28" t="s">
-        <v>51</v>
+        <v>107</v>
       </c>
       <c r="K28" t="s">
-        <v>52</v>
+        <v>108</v>
       </c>
       <c r="L28" t="s">
-        <v>53</v>
+        <v>109</v>
       </c>
       <c r="M28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N28" t="n">
         <v>4.0</v>
       </c>
       <c r="Q28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R28" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="T28" t="n">
         <v>110.0</v>
@@ -2659,10 +2533,10 @@
         <v>22</v>
       </c>
       <c r="E29" t="s">
-        <v>97</v>
+        <v>44</v>
       </c>
       <c r="F29" t="s">
-        <v>122</v>
+        <v>35</v>
       </c>
       <c r="G29" t="s">
         <v>20</v>
@@ -2674,25 +2548,25 @@
         <v>20</v>
       </c>
       <c r="J29" t="s">
-        <v>123</v>
+        <v>47</v>
       </c>
       <c r="K29" t="s">
-        <v>124</v>
+        <v>48</v>
       </c>
       <c r="L29" t="s">
-        <v>125</v>
+        <v>34</v>
       </c>
       <c r="M29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N29" t="n">
         <v>4.0</v>
       </c>
       <c r="Q29" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R29" t="s">
-        <v>121</v>
+        <v>110</v>
       </c>
       <c r="T29" t="n">
         <v>110.0</v>
@@ -2715,10 +2589,10 @@
         <v>22</v>
       </c>
       <c r="E30" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="F30" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="G30" t="s">
         <v>20</v>
@@ -2730,25 +2604,25 @@
         <v>20</v>
       </c>
       <c r="J30" t="s">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="K30" t="s">
-        <v>129</v>
+        <v>27</v>
       </c>
       <c r="L30" t="s">
-        <v>130</v>
+        <v>28</v>
       </c>
       <c r="M30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N30" t="n">
         <v>4.0</v>
       </c>
       <c r="Q30" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R30" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="T30" t="n">
         <v>110.0</v>
@@ -2771,10 +2645,10 @@
         <v>22</v>
       </c>
       <c r="E31" t="s">
-        <v>37</v>
+        <v>69</v>
       </c>
       <c r="F31" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="G31" t="s">
         <v>20</v>
@@ -2786,25 +2660,25 @@
         <v>20</v>
       </c>
       <c r="J31" t="s">
-        <v>133</v>
+        <v>71</v>
       </c>
       <c r="K31" t="s">
-        <v>134</v>
+        <v>72</v>
       </c>
       <c r="L31" t="s">
-        <v>135</v>
+        <v>73</v>
       </c>
       <c r="M31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N31" t="n">
         <v>4.0</v>
       </c>
       <c r="Q31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R31" t="s">
-        <v>131</v>
+        <v>20</v>
       </c>
       <c r="T31" t="n">
         <v>110.0</v>
@@ -2827,10 +2701,10 @@
         <v>22</v>
       </c>
       <c r="E32" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="F32" t="s">
-        <v>137</v>
+        <v>115</v>
       </c>
       <c r="G32" t="s">
         <v>20</v>
@@ -2842,28 +2716,28 @@
         <v>20</v>
       </c>
       <c r="J32" t="s">
-        <v>51</v>
+        <v>26</v>
       </c>
       <c r="K32" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="L32" t="s">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="M32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N32" t="n">
         <v>4.0</v>
       </c>
       <c r="P32" t="s">
-        <v>138</v>
+        <v>116</v>
       </c>
       <c r="Q32" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R32" t="s">
-        <v>136</v>
+        <v>114</v>
       </c>
       <c r="T32" t="n">
         <v>110.0</v>
@@ -2886,10 +2760,10 @@
         <v>22</v>
       </c>
       <c r="E33" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F33" t="s">
-        <v>46</v>
+        <v>113</v>
       </c>
       <c r="G33" t="s">
         <v>20</v>
@@ -2901,25 +2775,25 @@
         <v>20</v>
       </c>
       <c r="J33" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="K33" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="L33" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="M33" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N33" t="n">
         <v>4.0</v>
       </c>
       <c r="Q33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R33" t="s">
-        <v>139</v>
+        <v>20</v>
       </c>
       <c r="T33" t="n">
         <v>110.0</v>
@@ -2942,10 +2816,10 @@
         <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="F34" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="G34" t="s">
         <v>20</v>
@@ -2957,25 +2831,25 @@
         <v>20</v>
       </c>
       <c r="J34" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="K34" t="s">
-        <v>34</v>
+        <v>109</v>
       </c>
       <c r="L34" t="s">
-        <v>33</v>
+        <v>107</v>
       </c>
       <c r="M34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N34" t="n">
         <v>4.0</v>
       </c>
       <c r="Q34" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R34" t="s">
-        <v>20</v>
+        <v>117</v>
       </c>
       <c r="T34" t="n">
         <v>110.0</v>
@@ -2998,10 +2872,10 @@
         <v>22</v>
       </c>
       <c r="E35" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="F35" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="G35" t="s">
         <v>20</v>
@@ -3013,25 +2887,25 @@
         <v>20</v>
       </c>
       <c r="J35" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="K35" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="L35" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="M35" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N35" t="n">
         <v>4.0</v>
       </c>
       <c r="Q35" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R35" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="T35" t="n">
         <v>110.0</v>
@@ -3054,10 +2928,10 @@
         <v>22</v>
       </c>
       <c r="E36" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="F36" t="s">
-        <v>146</v>
+        <v>64</v>
       </c>
       <c r="G36" t="s">
         <v>20</v>
@@ -3069,25 +2943,25 @@
         <v>20</v>
       </c>
       <c r="J36" t="s">
-        <v>147</v>
+        <v>65</v>
       </c>
       <c r="K36" t="s">
-        <v>148</v>
+        <v>66</v>
       </c>
       <c r="L36" t="s">
-        <v>149</v>
+        <v>67</v>
       </c>
       <c r="M36" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N36" t="n">
         <v>4.0</v>
       </c>
       <c r="Q36" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R36" t="s">
-        <v>145</v>
+        <v>62</v>
       </c>
       <c r="T36" t="n">
         <v>110.0</v>
@@ -3110,10 +2984,10 @@
         <v>22</v>
       </c>
       <c r="E37" t="s">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="F37" t="s">
-        <v>76</v>
+        <v>37</v>
       </c>
       <c r="G37" t="s">
         <v>20</v>
@@ -3125,28 +2999,28 @@
         <v>20</v>
       </c>
       <c r="J37" t="s">
+        <v>35</v>
+      </c>
+      <c r="K37" t="s">
+        <v>47</v>
+      </c>
+      <c r="L37" t="s">
+        <v>48</v>
+      </c>
+      <c r="M37" t="s">
+        <v>29</v>
+      </c>
+      <c r="N37" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="P37" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>31</v>
+      </c>
+      <c r="R37" t="s">
         <v>45</v>
-      </c>
-      <c r="K37" t="s">
-        <v>46</v>
-      </c>
-      <c r="L37" t="s">
-        <v>68</v>
-      </c>
-      <c r="M37" t="s">
-        <v>28</v>
-      </c>
-      <c r="N37" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="P37" t="s">
-        <v>150</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>30</v>
-      </c>
-      <c r="R37" t="s">
-        <v>117</v>
       </c>
       <c r="T37" t="n">
         <v>110.0</v>
@@ -3169,10 +3043,10 @@
         <v>22</v>
       </c>
       <c r="E38" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="F38" t="s">
-        <v>35</v>
+        <v>125</v>
       </c>
       <c r="G38" t="s">
         <v>20</v>
@@ -3184,25 +3058,25 @@
         <v>20</v>
       </c>
       <c r="J38" t="s">
-        <v>32</v>
+        <v>89</v>
       </c>
       <c r="K38" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="L38" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="M38" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N38" t="n">
         <v>4.0</v>
       </c>
       <c r="Q38" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R38" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
       <c r="T38" t="n">
         <v>110.0</v>
@@ -3225,10 +3099,10 @@
         <v>22</v>
       </c>
       <c r="E39" t="s">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="F39" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G39" t="s">
         <v>20</v>
@@ -3240,25 +3114,25 @@
         <v>20</v>
       </c>
       <c r="J39" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="K39" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="L39" t="s">
-        <v>154</v>
+        <v>48</v>
       </c>
       <c r="M39" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N39" t="n">
         <v>4.0</v>
       </c>
       <c r="Q39" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R39" t="s">
-        <v>153</v>
+        <v>45</v>
       </c>
       <c r="T39" t="n">
         <v>110.0</v>
@@ -3281,10 +3155,10 @@
         <v>22</v>
       </c>
       <c r="E40" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F40" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="G40" t="s">
         <v>20</v>
@@ -3296,25 +3170,25 @@
         <v>20</v>
       </c>
       <c r="J40" t="s">
-        <v>154</v>
+        <v>65</v>
       </c>
       <c r="K40" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="L40" t="s">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="M40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N40" t="n">
         <v>4.0</v>
       </c>
       <c r="Q40" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R40" t="s">
-        <v>155</v>
+        <v>62</v>
       </c>
       <c r="T40" t="n">
         <v>110.0</v>
@@ -3337,10 +3211,10 @@
         <v>22</v>
       </c>
       <c r="E41" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="F41" t="s">
-        <v>35</v>
+        <v>91</v>
       </c>
       <c r="G41" t="s">
         <v>20</v>
@@ -3352,22 +3226,22 @@
         <v>20</v>
       </c>
       <c r="J41" t="s">
-        <v>152</v>
+        <v>71</v>
       </c>
       <c r="K41" t="s">
-        <v>34</v>
+        <v>72</v>
       </c>
       <c r="L41" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="M41" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N41" t="n">
         <v>4.0</v>
       </c>
       <c r="Q41" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R41" t="s">
         <v>20</v>
@@ -3393,10 +3267,10 @@
         <v>22</v>
       </c>
       <c r="E42" t="s">
-        <v>67</v>
+        <v>94</v>
       </c>
       <c r="F42" t="s">
-        <v>69</v>
+        <v>128</v>
       </c>
       <c r="G42" t="s">
         <v>20</v>
@@ -3408,28 +3282,28 @@
         <v>20</v>
       </c>
       <c r="J42" t="s">
-        <v>45</v>
+        <v>129</v>
       </c>
       <c r="K42" t="s">
-        <v>46</v>
+        <v>130</v>
       </c>
       <c r="L42" t="s">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="M42" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N42" t="n">
         <v>4.0</v>
       </c>
       <c r="P42" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="Q42" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R42" t="s">
-        <v>156</v>
+        <v>127</v>
       </c>
       <c r="T42" t="n">
         <v>110.0</v>
@@ -3452,10 +3326,10 @@
         <v>22</v>
       </c>
       <c r="E43" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="F43" t="s">
-        <v>158</v>
+        <v>76</v>
       </c>
       <c r="G43" t="s">
         <v>20</v>
@@ -3467,22 +3341,22 @@
         <v>20</v>
       </c>
       <c r="J43" t="s">
-        <v>159</v>
+        <v>78</v>
       </c>
       <c r="K43" t="s">
-        <v>160</v>
+        <v>133</v>
       </c>
       <c r="L43" t="s">
-        <v>161</v>
+        <v>79</v>
       </c>
       <c r="M43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N43" t="n">
         <v>4.0</v>
       </c>
       <c r="Q43" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R43" t="s">
         <v>20</v>
@@ -3508,10 +3382,10 @@
         <v>22</v>
       </c>
       <c r="E44" t="s">
-        <v>37</v>
+        <v>135</v>
       </c>
       <c r="F44" t="s">
-        <v>163</v>
+        <v>54</v>
       </c>
       <c r="G44" t="s">
         <v>20</v>
@@ -3523,25 +3397,25 @@
         <v>20</v>
       </c>
       <c r="J44" t="s">
-        <v>164</v>
+        <v>136</v>
       </c>
       <c r="K44" t="s">
-        <v>165</v>
+        <v>53</v>
       </c>
       <c r="L44" t="s">
-        <v>166</v>
+        <v>52</v>
       </c>
       <c r="M44" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N44" t="n">
         <v>4.0</v>
       </c>
       <c r="Q44" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R44" t="s">
-        <v>162</v>
+        <v>134</v>
       </c>
       <c r="T44" t="n">
         <v>110.0</v>
@@ -3564,10 +3438,10 @@
         <v>22</v>
       </c>
       <c r="E45" t="s">
-        <v>109</v>
+        <v>39</v>
       </c>
       <c r="F45" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
       <c r="G45" t="s">
         <v>20</v>
@@ -3579,25 +3453,25 @@
         <v>20</v>
       </c>
       <c r="J45" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
       <c r="K45" t="s">
-        <v>170</v>
+        <v>140</v>
       </c>
       <c r="L45" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
       <c r="M45" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N45" t="n">
         <v>4.0</v>
       </c>
       <c r="Q45" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R45" t="s">
-        <v>167</v>
+        <v>137</v>
       </c>
       <c r="T45" t="n">
         <v>110.0</v>
@@ -3620,10 +3494,10 @@
         <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>97</v>
+        <v>50</v>
       </c>
       <c r="F46" t="s">
-        <v>173</v>
+        <v>143</v>
       </c>
       <c r="G46" t="s">
         <v>20</v>
@@ -3635,25 +3509,25 @@
         <v>20</v>
       </c>
       <c r="J46" t="s">
-        <v>174</v>
+        <v>144</v>
       </c>
       <c r="K46" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
       <c r="L46" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="M46" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N46" t="n">
         <v>4.0</v>
       </c>
       <c r="Q46" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R46" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="T46" t="n">
         <v>110.0</v>
@@ -3676,10 +3550,10 @@
         <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="F47" t="s">
-        <v>178</v>
+        <v>64</v>
       </c>
       <c r="G47" t="s">
         <v>20</v>
@@ -3691,28 +3565,28 @@
         <v>20</v>
       </c>
       <c r="J47" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="K47" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="L47" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="M47" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N47" t="n">
         <v>4.0</v>
       </c>
       <c r="P47" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="Q47" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R47" t="s">
-        <v>177</v>
+        <v>62</v>
       </c>
       <c r="T47" t="n">
         <v>110.0</v>
@@ -3735,10 +3609,10 @@
         <v>22</v>
       </c>
       <c r="E48" t="s">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="F48" t="s">
-        <v>181</v>
+        <v>113</v>
       </c>
       <c r="G48" t="s">
         <v>20</v>
@@ -3750,25 +3624,25 @@
         <v>20</v>
       </c>
       <c r="J48" t="s">
-        <v>182</v>
+        <v>71</v>
       </c>
       <c r="K48" t="s">
-        <v>183</v>
+        <v>72</v>
       </c>
       <c r="L48" t="s">
-        <v>184</v>
+        <v>73</v>
       </c>
       <c r="M48" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N48" t="n">
         <v>4.0</v>
       </c>
       <c r="Q48" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R48" t="s">
-        <v>180</v>
+        <v>20</v>
       </c>
       <c r="T48" t="n">
         <v>110.0</v>
@@ -3791,10 +3665,10 @@
         <v>22</v>
       </c>
       <c r="E49" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="F49" t="s">
-        <v>186</v>
+        <v>47</v>
       </c>
       <c r="G49" t="s">
         <v>20</v>
@@ -3806,25 +3680,25 @@
         <v>20</v>
       </c>
       <c r="J49" t="s">
-        <v>187</v>
+        <v>35</v>
       </c>
       <c r="K49" t="s">
-        <v>188</v>
+        <v>36</v>
       </c>
       <c r="L49" t="s">
-        <v>189</v>
+        <v>37</v>
       </c>
       <c r="M49" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N49" t="n">
         <v>4.0</v>
       </c>
       <c r="Q49" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R49" t="s">
-        <v>185</v>
+        <v>84</v>
       </c>
       <c r="T49" t="n">
         <v>110.0</v>
@@ -3847,10 +3721,10 @@
         <v>22</v>
       </c>
       <c r="E50" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="F50" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="G50" t="s">
         <v>20</v>
@@ -3862,25 +3736,25 @@
         <v>20</v>
       </c>
       <c r="J50" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="K50" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L50" t="s">
-        <v>69</v>
+        <v>34</v>
       </c>
       <c r="M50" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N50" t="n">
         <v>4.0</v>
       </c>
       <c r="Q50" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R50" t="s">
-        <v>190</v>
+        <v>110</v>
       </c>
       <c r="T50" t="n">
         <v>110.0</v>
@@ -3903,10 +3777,10 @@
         <v>22</v>
       </c>
       <c r="E51" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="F51" t="s">
-        <v>191</v>
+        <v>149</v>
       </c>
       <c r="G51" t="s">
         <v>20</v>
@@ -3918,25 +3792,25 @@
         <v>20</v>
       </c>
       <c r="J51" t="s">
-        <v>192</v>
+        <v>150</v>
       </c>
       <c r="K51" t="s">
-        <v>193</v>
+        <v>151</v>
       </c>
       <c r="L51" t="s">
-        <v>194</v>
+        <v>152</v>
       </c>
       <c r="M51" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N51" t="n">
         <v>4.0</v>
       </c>
       <c r="Q51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R51" t="s">
-        <v>20</v>
+        <v>148</v>
       </c>
       <c r="T51" t="n">
         <v>110.0</v>
@@ -3947,7 +3821,7 @@
     </row>
     <row r="1002">
       <c r="A1002" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>